<commit_message>
V. 118 "Menudas Piezas"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB1D494-7649-41CC-ACC8-E35F622E27C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B90450-11A2-4BC6-AADA-E4D61F32F3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19320" yWindow="6015" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="220">
   <si>
     <t>Película</t>
   </si>
@@ -1233,6 +1233,9 @@
   </si>
   <si>
     <t>Blue Beetle</t>
+  </si>
+  <si>
+    <t>Menudas Piezas</t>
   </si>
 </sst>
 </file>
@@ -1336,13 +1339,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1354,45 +1357,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1433,6 +1397,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1559,48 +1562,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M68" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M68" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M68" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M68">
     <sortCondition descending="1" ref="C2:C68"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I138" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I138" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I138">
-    <sortCondition descending="1" ref="C2:C138"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I139" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I139" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I139">
+    <sortCondition descending="1" ref="C2:C139"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2087,7 +2090,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2123,7 +2126,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2190,7 +2193,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2228,7 +2231,7 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -2262,7 +2265,7 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -4310,7 +4313,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K138"/>
+  <dimension ref="B2:K139"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4348,7 +4351,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4378,7 +4381,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4406,7 +4409,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -6407,18 +6410,18 @@
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B79" s="2" t="s">
-        <v>41</v>
+      <c r="B79" s="9" t="s">
+        <v>219</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D79" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E79" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F79" s="1">
         <v>8</v>
@@ -6427,106 +6430,106 @@
         <v>7</v>
       </c>
       <c r="H79" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I79" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D80" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E80" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G80" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H80" s="3">
         <v>6.3</v>
       </c>
       <c r="I80" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D81" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E81" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F81" s="1">
         <v>7</v>
       </c>
       <c r="G81" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H81" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I81" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D82" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E82" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" s="1">
         <v>7</v>
       </c>
       <c r="G82" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H82" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I82" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D83" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E83" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F83" s="1">
         <v>7</v>
@@ -6535,76 +6538,76 @@
         <v>6</v>
       </c>
       <c r="H83" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I83" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D84" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" s="1">
         <v>7</v>
       </c>
       <c r="G84" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H84" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I84" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D85" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E85" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F85" s="1">
         <v>7</v>
       </c>
       <c r="G85" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H85" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I85" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D86" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E86" s="1">
         <v>6</v>
@@ -6616,25 +6619,25 @@
         <v>7</v>
       </c>
       <c r="H86" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I86" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D87" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E87" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" s="1">
         <v>7</v>
@@ -6643,79 +6646,79 @@
         <v>7</v>
       </c>
       <c r="H87" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I87" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D88" s="1">
         <v>7</v>
       </c>
       <c r="E88" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F88" s="1">
         <v>7</v>
       </c>
       <c r="G88" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H88" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I88" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
         <v>6.35</v>
       </c>
       <c r="D89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E89" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G89" s="1">
         <v>6</v>
       </c>
       <c r="H89" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I89" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D90" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F90" s="1">
         <v>6</v>
@@ -6724,42 +6727,42 @@
         <v>6</v>
       </c>
       <c r="H90" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I90" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E91" s="1">
         <v>6</v>
       </c>
       <c r="F91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H91" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I91" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
@@ -6769,163 +6772,163 @@
         <v>6</v>
       </c>
       <c r="E92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H92" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I92" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F93" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G93" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I93" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D94" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" s="1">
         <v>8</v>
       </c>
       <c r="G94" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H94" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I94" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D95" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F95" s="1">
         <v>8</v>
       </c>
       <c r="G95" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I95" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D96" s="1">
         <v>7</v>
       </c>
       <c r="E96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G96" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H96" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I96" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>214</v>
+        <v>158</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D97" s="1">
         <v>7</v>
       </c>
       <c r="E97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F97" s="1">
         <v>7</v>
       </c>
       <c r="G97" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H97" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I97" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D98" s="1">
         <v>7</v>
@@ -6937,49 +6940,49 @@
         <v>7</v>
       </c>
       <c r="G98" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H98" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I98" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.05</v>
       </c>
       <c r="D99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E99" s="1">
         <v>6</v>
       </c>
       <c r="F99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I99" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D100" s="1">
         <v>6</v>
@@ -6988,133 +6991,133 @@
         <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G100" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H100" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I100" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D101" s="1">
         <v>6</v>
       </c>
       <c r="E101" s="1">
+        <v>6</v>
+      </c>
+      <c r="F101" s="1">
+        <v>8</v>
+      </c>
+      <c r="G101" s="1">
         <v>5</v>
       </c>
-      <c r="F101" s="1">
-        <v>6</v>
-      </c>
-      <c r="G101" s="1">
-        <v>6</v>
-      </c>
       <c r="H101" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I101" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E102" s="1">
         <v>5</v>
       </c>
       <c r="F102" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I102" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D103" s="1">
         <v>7</v>
       </c>
       <c r="E103" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F103" s="1">
         <v>5</v>
       </c>
       <c r="G103" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H103" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I103" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D104" s="1">
         <v>7</v>
       </c>
       <c r="E104" s="1">
+        <v>6</v>
+      </c>
+      <c r="F104" s="1">
         <v>5</v>
       </c>
-      <c r="F104" s="1">
-        <v>4</v>
-      </c>
       <c r="G104" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H104" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I104" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D105" s="1">
         <v>7</v>
@@ -7126,37 +7129,37 @@
         <v>4</v>
       </c>
       <c r="G105" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I105" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D106" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E106" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F106" s="1">
+        <v>4</v>
+      </c>
+      <c r="G106" s="1">
         <v>5</v>
       </c>
-      <c r="G106" s="1">
-        <v>6</v>
-      </c>
       <c r="H106" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I106" s="3">
         <v>6.4</v>
@@ -7164,50 +7167,50 @@
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D107" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E107" s="1">
+        <v>3</v>
+      </c>
+      <c r="F107" s="1">
         <v>5</v>
       </c>
-      <c r="F107" s="1">
-        <v>6</v>
-      </c>
       <c r="G107" s="1">
         <v>6</v>
       </c>
       <c r="H107" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I107" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D108" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E108" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F108" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G108" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H108" s="3">
         <v>5.8</v>
@@ -7218,260 +7221,260 @@
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D109" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E109" s="1">
         <v>6</v>
       </c>
       <c r="F109" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G109" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H109" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I109" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E110" s="1">
         <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I110" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D111" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E111" s="1">
+        <v>6</v>
+      </c>
+      <c r="F111" s="1">
         <v>5</v>
       </c>
-      <c r="F111" s="1">
-        <v>6</v>
-      </c>
       <c r="G111" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H111" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I111" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D112" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F112" s="1">
         <v>6</v>
       </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H112" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I112" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D113" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I113" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D114" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E114" s="1">
         <v>5</v>
       </c>
       <c r="F114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H114" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I114" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E115" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F115" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G115" s="1">
         <v>6</v>
       </c>
       <c r="H115" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I115" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.05</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E116" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F116" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G116" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I116" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D117" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E117" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F117" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G117" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H117" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I117" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E118" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F118" s="1">
         <v>5</v>
@@ -7480,397 +7483,397 @@
         <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I118" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D119" s="1">
+        <v>6</v>
+      </c>
+      <c r="E119" s="1">
+        <v>3</v>
+      </c>
+      <c r="F119" s="1">
         <v>5</v>
       </c>
-      <c r="E119" s="1">
-        <v>5</v>
-      </c>
-      <c r="F119" s="1">
-        <v>3</v>
-      </c>
       <c r="G119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I119" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D120" s="1">
         <v>5</v>
       </c>
       <c r="E120" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F120" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G120" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H120" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I120" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I120" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D121" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E121" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F121" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G121" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H121" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I121" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D122" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E122" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F122" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G122" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H122" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I122" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D123" s="1">
         <v>5</v>
       </c>
       <c r="E123" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F123" s="1">
         <v>5</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H123" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I123" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D124" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E124" s="1">
         <v>4</v>
       </c>
       <c r="F124" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G124" s="1">
         <v>5</v>
       </c>
       <c r="H124" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I124" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D125" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E125" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F125" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G125" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H125" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I125" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D126" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E126" s="1">
+        <v>0</v>
+      </c>
+      <c r="F126" s="1">
         <v>2</v>
       </c>
-      <c r="F126" s="1">
-        <v>4</v>
-      </c>
       <c r="G126" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H126" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I126" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D127" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E127" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F127" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G127" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H127" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I127" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D128" s="1">
+        <v>5</v>
+      </c>
+      <c r="E128" s="1">
         <v>3</v>
       </c>
-      <c r="E128" s="1">
-        <v>4</v>
-      </c>
       <c r="F128" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G128" s="1">
         <v>4</v>
       </c>
       <c r="H128" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I128" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D129" s="1">
+        <v>3</v>
+      </c>
+      <c r="E129" s="1">
         <v>4</v>
       </c>
-      <c r="E129" s="1">
-        <v>3</v>
-      </c>
       <c r="F129" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G129" s="1">
         <v>4</v>
       </c>
       <c r="H129" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I129" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D130" s="1">
         <v>4</v>
       </c>
       <c r="E130" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F130" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G130" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H130" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I130" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D131" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E131" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F131" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I131" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B132" s="9" t="s">
-        <v>218</v>
+      <c r="B132" s="2" t="s">
+        <v>68</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D132" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E132" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F132" s="1">
         <v>2</v>
       </c>
       <c r="G132" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H132" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I132" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D133" s="1">
         <v>3</v>
@@ -7879,150 +7882,177 @@
         <v>3</v>
       </c>
       <c r="F133" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G133" s="1">
         <v>4</v>
       </c>
       <c r="H133" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I133" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I133" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D134" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E134" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F134" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G134" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H134" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I134" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D135" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E135" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="1">
         <v>2</v>
       </c>
       <c r="G135" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H135" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I135" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D136" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E136" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F136" s="1">
         <v>2</v>
       </c>
       <c r="G136" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H136" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I136" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D137" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E137" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G137" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H137" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I137" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D138" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E138" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F138" s="1">
         <v>0</v>
       </c>
       <c r="G138" s="1">
+        <v>1</v>
+      </c>
+      <c r="H138" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I138" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="139" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B139" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C139" s="5">
+        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D139" s="1">
         <v>0</v>
       </c>
-      <c r="H138" s="3">
+      <c r="E139" s="1">
+        <v>0</v>
+      </c>
+      <c r="F139" s="1">
+        <v>0</v>
+      </c>
+      <c r="G139" s="1">
+        <v>0</v>
+      </c>
+      <c r="H139" s="3">
         <v>7.6</v>
       </c>
-      <c r="I138" s="3">
+      <c r="I139" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 119 "Torrente Presidente"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B90450-11A2-4BC6-AADA-E4D61F32F3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A04B974-483E-4858-B308-7B85F38012BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="6015" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="221">
   <si>
     <t>Película</t>
   </si>
@@ -1236,6 +1236,9 @@
   </si>
   <si>
     <t>Menudas Piezas</t>
+  </si>
+  <si>
+    <t>Torrente Presidente</t>
   </si>
 </sst>
 </file>
@@ -1588,10 +1591,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I139" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I139" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I139">
-    <sortCondition descending="1" ref="C2:C139"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I140" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I140" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I140">
+    <sortCondition descending="1" ref="C2:C140"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4313,7 +4316,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K139"/>
+  <dimension ref="B2:K140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5546,39 +5549,39 @@
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="2" t="s">
-        <v>175</v>
+      <c r="B47" s="9" t="s">
+        <v>220</v>
       </c>
       <c r="C47" s="5">
         <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
-        <v>7.3624999999999989</v>
+        <v>7.3624999999999998</v>
       </c>
       <c r="D47" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E47" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F47" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G47" s="1">
         <v>8</v>
       </c>
       <c r="H47" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I47" s="3">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>52</v>
+        <v>175</v>
       </c>
       <c r="C48" s="5">
         <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
-        <v>7.3500000000000005</v>
+        <v>7.3624999999999989</v>
       </c>
       <c r="D48" s="1">
         <v>8</v>
@@ -5587,25 +5590,25 @@
         <v>8</v>
       </c>
       <c r="F48" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G48" s="1">
         <v>8</v>
       </c>
       <c r="H48" s="3">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="I48" s="3">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>165</v>
+        <v>52</v>
       </c>
       <c r="C49" s="5">
         <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
-        <v>7.3249999999999993</v>
+        <v>7.3500000000000005</v>
       </c>
       <c r="D49" s="1">
         <v>8</v>
@@ -5617,82 +5620,82 @@
         <v>8</v>
       </c>
       <c r="G49" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H49" s="3">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="I49" s="3">
-        <v>6</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>111</v>
+        <v>165</v>
       </c>
       <c r="C50" s="5">
         <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
-        <v>7.3</v>
+        <v>7.3249999999999993</v>
       </c>
       <c r="D50" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E50" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F50" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G50" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H50" s="3">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="I50" s="3">
-        <v>5.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C51" s="5">
         <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
-        <v>7.2750000000000004</v>
+        <v>7.3</v>
       </c>
       <c r="D51" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E51" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G51" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H51" s="3">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="I51" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="C52" s="5">
         <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D52" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E52" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F52" s="1">
         <v>8</v>
@@ -5701,25 +5704,25 @@
         <v>8</v>
       </c>
       <c r="H52" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="I52" s="3">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="C53" s="5">
         <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
-        <v>7.2374999999999998</v>
+        <v>7.2750000000000004</v>
       </c>
       <c r="D53" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E53" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F53" s="1">
         <v>8</v>
@@ -5728,127 +5731,127 @@
         <v>8</v>
       </c>
       <c r="H53" s="3">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="I53" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="C54" s="5">
         <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
-        <v>7.2250000000000005</v>
+        <v>7.2374999999999998</v>
       </c>
       <c r="D54" s="1">
         <v>7</v>
       </c>
       <c r="E54" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F54" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G54" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H54" s="3">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="I54" s="3">
-        <v>7.6</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C55" s="5">
         <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
-        <v>7.2125000000000004</v>
+        <v>7.2250000000000005</v>
       </c>
       <c r="D55" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E55" s="1">
         <v>7</v>
       </c>
       <c r="F55" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G55" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H55" s="3">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="I55" s="3">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>146</v>
+        <v>65</v>
       </c>
       <c r="C56" s="5">
         <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
-        <v>7.2124999999999995</v>
+        <v>7.2125000000000004</v>
       </c>
       <c r="D56" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F56" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G56" s="1">
         <v>8</v>
       </c>
       <c r="H56" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I56" s="3">
         <v>6.3</v>
-      </c>
-      <c r="I56" s="3">
-        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="C57" s="5">
         <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
-        <v>7.1999999999999993</v>
+        <v>7.2124999999999995</v>
       </c>
       <c r="D57" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E57" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F57" s="1">
         <v>9</v>
       </c>
       <c r="G57" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H57" s="3">
         <v>6.3</v>
       </c>
       <c r="I57" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="C58" s="5">
         <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
-        <v>7.1499999999999995</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D58" s="1">
         <v>8</v>
@@ -5857,217 +5860,217 @@
         <v>7</v>
       </c>
       <c r="F58" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G58" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H58" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I58" s="3">
-        <v>6.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="C59" s="5">
         <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
-        <v>7.1375000000000011</v>
+        <v>7.1499999999999995</v>
       </c>
       <c r="D59" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E59" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F59" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G59" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H59" s="3">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="I59" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="C60" s="5">
         <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
-        <v>7.1250000000000009</v>
+        <v>7.1375000000000011</v>
       </c>
       <c r="D60" s="1">
         <v>7</v>
       </c>
       <c r="E60" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F60" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G60" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H60" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I60" s="3">
         <v>6.7</v>
-      </c>
-      <c r="I60" s="3">
-        <v>6.6</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C61" s="5">
         <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
-        <v>7.125</v>
+        <v>7.1250000000000009</v>
       </c>
       <c r="D61" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E61" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F61" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G61" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H61" s="3">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="I61" s="3">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>133</v>
+        <v>39</v>
       </c>
       <c r="C62" s="5">
         <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
-        <v>7.0875000000000004</v>
+        <v>7.125</v>
       </c>
       <c r="D62" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E62" s="1">
         <v>8</v>
       </c>
       <c r="F62" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G62" s="1">
         <v>7</v>
       </c>
       <c r="H62" s="3">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="I62" s="3">
-        <v>6.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="C63" s="5">
         <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
-        <v>7.0750000000000011</v>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D63" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E63" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F63" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G63" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H63" s="3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="I63" s="3">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C64" s="5">
         <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D64" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E64" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" s="1">
         <v>8</v>
       </c>
       <c r="G64" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H64" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I64" s="3">
         <v>6.2</v>
-      </c>
-      <c r="I64" s="3">
-        <v>5.2</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="C65" s="5">
         <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
-        <v>7.0750000000000002</v>
+        <v>7.0750000000000011</v>
       </c>
       <c r="D65" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E65" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F65" s="1">
         <v>8</v>
       </c>
       <c r="G65" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H65" s="3">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="I65" s="3">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="C66" s="5">
         <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D66" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
         <v>7</v>
@@ -6076,55 +6079,55 @@
         <v>8</v>
       </c>
       <c r="G66" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H66" s="3">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="I66" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="C67" s="5">
         <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
-        <v>7.0749999999999993</v>
+        <v>7.0750000000000002</v>
       </c>
       <c r="D67" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E67" s="1">
         <v>7</v>
       </c>
       <c r="F67" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G67" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H67" s="3">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="I67" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C68" s="5">
         <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
-        <v>7.05</v>
+        <v>7.0749999999999993</v>
       </c>
       <c r="D68" s="1">
         <v>8</v>
       </c>
       <c r="E68" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" s="1">
         <v>7</v>
@@ -6133,46 +6136,46 @@
         <v>8</v>
       </c>
       <c r="H68" s="3">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="I68" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>95</v>
+        <v>176</v>
       </c>
       <c r="C69" s="5">
         <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
-        <v>6.9375</v>
+        <v>7.05</v>
       </c>
       <c r="D69" s="1">
         <v>8</v>
       </c>
       <c r="E69" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F69" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G69" s="1">
         <v>8</v>
       </c>
       <c r="H69" s="3">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="I69" s="3">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>164</v>
+        <v>95</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
-        <v>6.9124999999999996</v>
+        <v>6.9375</v>
       </c>
       <c r="D70" s="1">
         <v>8</v>
@@ -6184,72 +6187,72 @@
         <v>8</v>
       </c>
       <c r="G70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H70" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="I70" s="3">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
-        <v>6.8999999999999995</v>
+        <v>6.9124999999999996</v>
       </c>
       <c r="D71" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E71" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F71" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G71" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H71" s="3">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="I71" s="3">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>88</v>
+        <v>157</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
-        <v>6.8624999999999989</v>
+        <v>6.8999999999999995</v>
       </c>
       <c r="D72" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E72" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G72" s="1">
         <v>8</v>
       </c>
       <c r="H72" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I72" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>184</v>
+        <v>88</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
@@ -6276,179 +6279,179 @@
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
-        <v>6.85</v>
+        <v>6.8624999999999989</v>
       </c>
       <c r="D74" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E74" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F74" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G74" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H74" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I74" s="3">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C75" s="5">
         <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
-        <v>6.7999999999999989</v>
+        <v>6.85</v>
       </c>
       <c r="D75" s="1">
         <v>8</v>
       </c>
       <c r="E75" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G75" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H75" s="3">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="I75" s="3">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="2" t="s">
-        <v>57</v>
+        <v>196</v>
       </c>
       <c r="C76" s="5">
         <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
-        <v>6.6999999999999993</v>
+        <v>6.7999999999999989</v>
       </c>
       <c r="D76" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E76" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F76" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G76" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H76" s="3">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="I76" s="3">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C77" s="5">
         <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
-        <v>6.6875</v>
+        <v>6.6999999999999993</v>
       </c>
       <c r="D77" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E77" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G77" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H77" s="3">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="I77" s="3">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
       <c r="C78" s="5">
         <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
-        <v>6.6375000000000002</v>
+        <v>6.6875</v>
       </c>
       <c r="D78" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E78" s="1">
         <v>7</v>
       </c>
       <c r="F78" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G78" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H78" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I78" s="3">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B79" s="9" t="s">
-        <v>219</v>
+      <c r="B79" s="2" t="s">
+        <v>211</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
-        <v>6.6374999999999993</v>
+        <v>6.6375000000000002</v>
       </c>
       <c r="D79" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E79" s="1">
         <v>7</v>
       </c>
       <c r="F79" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G79" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H79" s="3">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="I79" s="3">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D80" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E80" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F80" s="1">
         <v>8</v>
@@ -6457,106 +6460,106 @@
         <v>7</v>
       </c>
       <c r="H80" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I80" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D81" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E81" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G81" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H81" s="3">
         <v>6.3</v>
       </c>
       <c r="I81" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D82" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E82" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F82" s="1">
         <v>7</v>
       </c>
       <c r="G82" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H82" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I82" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D83" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E83" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" s="1">
         <v>7</v>
       </c>
       <c r="G83" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H83" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I83" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D84" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E84" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F84" s="1">
         <v>7</v>
@@ -6565,76 +6568,76 @@
         <v>6</v>
       </c>
       <c r="H84" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I84" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D85" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E85" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" s="1">
         <v>7</v>
       </c>
       <c r="G85" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H85" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I85" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D86" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E86" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F86" s="1">
         <v>7</v>
       </c>
       <c r="G86" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H86" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I86" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D87" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E87" s="1">
         <v>6</v>
@@ -6646,25 +6649,25 @@
         <v>7</v>
       </c>
       <c r="H87" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I87" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D88" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E88" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" s="1">
         <v>7</v>
@@ -6673,79 +6676,79 @@
         <v>7</v>
       </c>
       <c r="H88" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I88" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D89" s="1">
         <v>7</v>
       </c>
       <c r="E89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F89" s="1">
         <v>7</v>
       </c>
       <c r="G89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H89" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I89" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
         <v>6.35</v>
       </c>
       <c r="D90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E90" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G90" s="1">
         <v>6</v>
       </c>
       <c r="H90" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I90" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F91" s="1">
         <v>6</v>
@@ -6754,42 +6757,42 @@
         <v>6</v>
       </c>
       <c r="H91" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I91" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E92" s="1">
         <v>6</v>
       </c>
       <c r="F92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H92" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I92" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
@@ -6799,163 +6802,163 @@
         <v>6</v>
       </c>
       <c r="E93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H93" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I93" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F94" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G94" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H94" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I94" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D95" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" s="1">
         <v>8</v>
       </c>
       <c r="G95" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H95" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I95" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D96" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F96" s="1">
         <v>8</v>
       </c>
       <c r="G96" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H96" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I96" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D97" s="1">
         <v>7</v>
       </c>
       <c r="E97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G97" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H97" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I97" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>214</v>
+        <v>158</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D98" s="1">
         <v>7</v>
       </c>
       <c r="E98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F98" s="1">
         <v>7</v>
       </c>
       <c r="G98" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H98" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I98" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D99" s="1">
         <v>7</v>
@@ -6967,49 +6970,49 @@
         <v>7</v>
       </c>
       <c r="G99" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H99" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I99" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
         <v>6.05</v>
       </c>
       <c r="D100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E100" s="1">
         <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H100" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I100" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D101" s="1">
         <v>6</v>
@@ -7018,133 +7021,133 @@
         <v>6</v>
       </c>
       <c r="F101" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G101" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H101" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I101" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D102" s="1">
         <v>6</v>
       </c>
       <c r="E102" s="1">
+        <v>6</v>
+      </c>
+      <c r="F102" s="1">
+        <v>8</v>
+      </c>
+      <c r="G102" s="1">
         <v>5</v>
       </c>
-      <c r="F102" s="1">
-        <v>6</v>
-      </c>
-      <c r="G102" s="1">
-        <v>6</v>
-      </c>
       <c r="H102" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I102" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D103" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E103" s="1">
         <v>5</v>
       </c>
       <c r="F103" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G103" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H103" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I103" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D104" s="1">
         <v>7</v>
       </c>
       <c r="E104" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F104" s="1">
         <v>5</v>
       </c>
       <c r="G104" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H104" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I104" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D105" s="1">
         <v>7</v>
       </c>
       <c r="E105" s="1">
+        <v>6</v>
+      </c>
+      <c r="F105" s="1">
         <v>5</v>
       </c>
-      <c r="F105" s="1">
-        <v>4</v>
-      </c>
       <c r="G105" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H105" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I105" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
@@ -7156,37 +7159,37 @@
         <v>4</v>
       </c>
       <c r="G106" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H106" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I106" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D107" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E107" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F107" s="1">
+        <v>4</v>
+      </c>
+      <c r="G107" s="1">
         <v>5</v>
       </c>
-      <c r="G107" s="1">
-        <v>6</v>
-      </c>
       <c r="H107" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I107" s="3">
         <v>6.4</v>
@@ -7194,50 +7197,50 @@
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D108" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E108" s="1">
+        <v>3</v>
+      </c>
+      <c r="F108" s="1">
         <v>5</v>
       </c>
-      <c r="F108" s="1">
-        <v>6</v>
-      </c>
       <c r="G108" s="1">
         <v>6</v>
       </c>
       <c r="H108" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I108" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D109" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E109" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F109" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G109" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H109" s="3">
         <v>5.8</v>
@@ -7248,260 +7251,260 @@
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D110" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E110" s="1">
         <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G110" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H110" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I110" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E111" s="1">
         <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H111" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I111" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E112" s="1">
+        <v>6</v>
+      </c>
+      <c r="F112" s="1">
         <v>5</v>
       </c>
-      <c r="F112" s="1">
-        <v>6</v>
-      </c>
       <c r="G112" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H112" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I112" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D113" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F113" s="1">
         <v>6</v>
       </c>
       <c r="G113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H113" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I113" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D114" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I114" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D115" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E115" s="1">
         <v>5</v>
       </c>
       <c r="F115" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G115" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H115" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I115" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E116" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F116" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G116" s="1">
         <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I116" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.05</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E117" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F117" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G117" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I117" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D118" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E118" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F118" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G118" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H118" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I118" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D119" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E119" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F119" s="1">
         <v>5</v>
@@ -7510,397 +7513,397 @@
         <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I119" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D120" s="1">
+        <v>6</v>
+      </c>
+      <c r="E120" s="1">
+        <v>3</v>
+      </c>
+      <c r="F120" s="1">
         <v>5</v>
       </c>
-      <c r="E120" s="1">
-        <v>5</v>
-      </c>
-      <c r="F120" s="1">
-        <v>3</v>
-      </c>
       <c r="G120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I120" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D121" s="1">
         <v>5</v>
       </c>
       <c r="E121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F121" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G121" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H121" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I121" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I121" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D122" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E122" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F122" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G122" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H122" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I122" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D123" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E123" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F123" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G123" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H123" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I123" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D124" s="1">
         <v>5</v>
       </c>
       <c r="E124" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
         <v>5</v>
       </c>
       <c r="G124" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H124" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I124" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D125" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E125" s="1">
         <v>4</v>
       </c>
       <c r="F125" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G125" s="1">
         <v>5</v>
       </c>
       <c r="H125" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I125" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D126" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E126" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F126" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G126" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H126" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I126" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D127" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E127" s="1">
+        <v>0</v>
+      </c>
+      <c r="F127" s="1">
         <v>2</v>
       </c>
-      <c r="F127" s="1">
-        <v>4</v>
-      </c>
       <c r="G127" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H127" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I127" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D128" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E128" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F128" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G128" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H128" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I128" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D129" s="1">
+        <v>5</v>
+      </c>
+      <c r="E129" s="1">
         <v>3</v>
       </c>
-      <c r="E129" s="1">
-        <v>4</v>
-      </c>
       <c r="F129" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G129" s="1">
         <v>4</v>
       </c>
       <c r="H129" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I129" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D130" s="1">
+        <v>3</v>
+      </c>
+      <c r="E130" s="1">
         <v>4</v>
       </c>
-      <c r="E130" s="1">
-        <v>3</v>
-      </c>
       <c r="F130" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G130" s="1">
         <v>4</v>
       </c>
       <c r="H130" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I130" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D131" s="1">
         <v>4</v>
       </c>
       <c r="E131" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F131" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G131" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H131" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I131" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D132" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E132" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F132" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H132" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I132" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D133" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F133" s="1">
         <v>2</v>
       </c>
       <c r="G133" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H133" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I133" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D134" s="1">
         <v>3</v>
@@ -7909,150 +7912,177 @@
         <v>3</v>
       </c>
       <c r="F134" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G134" s="1">
         <v>4</v>
       </c>
       <c r="H134" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I134" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I134" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D135" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E135" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F135" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G135" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H135" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I135" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F136" s="1">
         <v>2</v>
       </c>
       <c r="G136" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H136" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I136" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D137" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E137" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F137" s="1">
         <v>2</v>
       </c>
       <c r="G137" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H137" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I137" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D138" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E138" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F138" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G138" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H138" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I138" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D139" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E139" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F139" s="1">
         <v>0</v>
       </c>
       <c r="G139" s="1">
+        <v>1</v>
+      </c>
+      <c r="H139" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I139" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="140" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B140" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C140" s="5">
+        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D140" s="1">
         <v>0</v>
       </c>
-      <c r="H139" s="3">
+      <c r="E140" s="1">
+        <v>0</v>
+      </c>
+      <c r="F140" s="1">
+        <v>0</v>
+      </c>
+      <c r="G140" s="1">
+        <v>0</v>
+      </c>
+      <c r="H140" s="3">
         <v>7.6</v>
       </c>
-      <c r="I139" s="3">
+      <c r="I140" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 120 "El falsificador"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A04B974-483E-4858-B308-7B85F38012BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15DB091B-D745-4F35-AE3F-CB94841FCF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="222">
   <si>
     <t>Película</t>
   </si>
@@ -1239,6 +1239,9 @@
   </si>
   <si>
     <t>Torrente Presidente</t>
+  </si>
+  <si>
+    <t>El falsificador</t>
   </si>
 </sst>
 </file>
@@ -1591,10 +1594,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I140" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I140" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I140">
-    <sortCondition descending="1" ref="C2:C140"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I141" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I141" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I141">
+    <sortCondition descending="1" ref="C2:C141"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4316,7 +4319,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K140"/>
+  <dimension ref="B2:K141"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5549,7 +5552,7 @@
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="2" t="s">
         <v>220</v>
       </c>
       <c r="C47" s="5">
@@ -6170,12 +6173,12 @@
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B70" s="2" t="s">
-        <v>95</v>
+      <c r="B70" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
-        <v>6.9375</v>
+        <v>7.0250000000000004</v>
       </c>
       <c r="D70" s="1">
         <v>8</v>
@@ -6187,22 +6190,22 @@
         <v>8</v>
       </c>
       <c r="G70" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H70" s="3">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="I70" s="3">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>164</v>
+        <v>95</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
-        <v>6.9124999999999996</v>
+        <v>6.9375</v>
       </c>
       <c r="D71" s="1">
         <v>8</v>
@@ -6214,72 +6217,72 @@
         <v>8</v>
       </c>
       <c r="G71" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H71" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="I71" s="3">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
-        <v>6.8999999999999995</v>
+        <v>6.9124999999999996</v>
       </c>
       <c r="D72" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E72" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F72" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G72" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H72" s="3">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="I72" s="3">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>88</v>
+        <v>157</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
-        <v>6.8624999999999989</v>
+        <v>6.8999999999999995</v>
       </c>
       <c r="D73" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E73" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F73" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G73" s="1">
         <v>8</v>
       </c>
       <c r="H73" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I73" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>184</v>
+        <v>88</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
@@ -6306,179 +6309,179 @@
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="C75" s="5">
         <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
-        <v>6.85</v>
+        <v>6.8624999999999989</v>
       </c>
       <c r="D75" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E75" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F75" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G75" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H75" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I75" s="3">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="2" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C76" s="5">
         <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
-        <v>6.7999999999999989</v>
+        <v>6.85</v>
       </c>
       <c r="D76" s="1">
         <v>8</v>
       </c>
       <c r="E76" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G76" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H76" s="3">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="I76" s="3">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
-        <v>57</v>
+        <v>196</v>
       </c>
       <c r="C77" s="5">
         <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
-        <v>6.6999999999999993</v>
+        <v>6.7999999999999989</v>
       </c>
       <c r="D77" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E77" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F77" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G77" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H77" s="3">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="I77" s="3">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C78" s="5">
         <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
-        <v>6.6875</v>
+        <v>6.6999999999999993</v>
       </c>
       <c r="D78" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E78" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G78" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H78" s="3">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="I78" s="3">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" s="2" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
-        <v>6.6375000000000002</v>
+        <v>6.6875</v>
       </c>
       <c r="D79" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E79" s="1">
         <v>7</v>
       </c>
       <c r="F79" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G79" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H79" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I79" s="3">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.6374999999999993</v>
+        <v>6.6375000000000002</v>
       </c>
       <c r="D80" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E80" s="1">
         <v>7</v>
       </c>
       <c r="F80" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G80" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H80" s="3">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="I80" s="3">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D81" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E81" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F81" s="1">
         <v>8</v>
@@ -6487,106 +6490,106 @@
         <v>7</v>
       </c>
       <c r="H81" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I81" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D82" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E82" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G82" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H82" s="3">
         <v>6.3</v>
       </c>
       <c r="I82" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D83" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E83" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F83" s="1">
         <v>7</v>
       </c>
       <c r="G83" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H83" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I83" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D84" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" s="1">
         <v>7</v>
       </c>
       <c r="G84" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H84" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I84" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D85" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E85" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F85" s="1">
         <v>7</v>
@@ -6595,76 +6598,76 @@
         <v>6</v>
       </c>
       <c r="H85" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I85" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D86" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E86" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" s="1">
         <v>7</v>
       </c>
       <c r="G86" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H86" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I86" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D87" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E87" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F87" s="1">
         <v>7</v>
       </c>
       <c r="G87" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H87" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I87" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D88" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E88" s="1">
         <v>6</v>
@@ -6676,25 +6679,25 @@
         <v>7</v>
       </c>
       <c r="H88" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I88" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D89" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E89" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" s="1">
         <v>7</v>
@@ -6703,79 +6706,79 @@
         <v>7</v>
       </c>
       <c r="H89" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I89" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D90" s="1">
         <v>7</v>
       </c>
       <c r="E90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F90" s="1">
         <v>7</v>
       </c>
       <c r="G90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H90" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I90" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
         <v>6.35</v>
       </c>
       <c r="D91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G91" s="1">
         <v>6</v>
       </c>
       <c r="H91" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I91" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F92" s="1">
         <v>6</v>
@@ -6784,42 +6787,42 @@
         <v>6</v>
       </c>
       <c r="H92" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I92" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E93" s="1">
         <v>6</v>
       </c>
       <c r="F93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I93" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
@@ -6829,163 +6832,163 @@
         <v>6</v>
       </c>
       <c r="E94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H94" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I94" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F95" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G95" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H95" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I95" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D96" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" s="1">
         <v>8</v>
       </c>
       <c r="G96" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H96" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I96" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D97" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F97" s="1">
         <v>8</v>
       </c>
       <c r="G97" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H97" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I97" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D98" s="1">
         <v>7</v>
       </c>
       <c r="E98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G98" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H98" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I98" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>214</v>
+        <v>158</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D99" s="1">
         <v>7</v>
       </c>
       <c r="E99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F99" s="1">
         <v>7</v>
       </c>
       <c r="G99" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I99" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D100" s="1">
         <v>7</v>
@@ -6997,49 +7000,49 @@
         <v>7</v>
       </c>
       <c r="G100" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H100" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I100" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
         <v>6.05</v>
       </c>
       <c r="D101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E101" s="1">
         <v>6</v>
       </c>
       <c r="F101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H101" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I101" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D102" s="1">
         <v>6</v>
@@ -7048,133 +7051,133 @@
         <v>6</v>
       </c>
       <c r="F102" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G102" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I102" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D103" s="1">
         <v>6</v>
       </c>
       <c r="E103" s="1">
+        <v>6</v>
+      </c>
+      <c r="F103" s="1">
+        <v>8</v>
+      </c>
+      <c r="G103" s="1">
         <v>5</v>
       </c>
-      <c r="F103" s="1">
-        <v>6</v>
-      </c>
-      <c r="G103" s="1">
-        <v>6</v>
-      </c>
       <c r="H103" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I103" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D104" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E104" s="1">
         <v>5</v>
       </c>
       <c r="F104" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G104" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H104" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I104" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D105" s="1">
         <v>7</v>
       </c>
       <c r="E105" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F105" s="1">
         <v>5</v>
       </c>
       <c r="G105" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H105" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I105" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
       </c>
       <c r="E106" s="1">
+        <v>6</v>
+      </c>
+      <c r="F106" s="1">
         <v>5</v>
       </c>
-      <c r="F106" s="1">
-        <v>4</v>
-      </c>
       <c r="G106" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H106" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I106" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D107" s="1">
         <v>7</v>
@@ -7186,37 +7189,37 @@
         <v>4</v>
       </c>
       <c r="G107" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H107" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I107" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D108" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E108" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F108" s="1">
+        <v>4</v>
+      </c>
+      <c r="G108" s="1">
         <v>5</v>
       </c>
-      <c r="G108" s="1">
-        <v>6</v>
-      </c>
       <c r="H108" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I108" s="3">
         <v>6.4</v>
@@ -7224,50 +7227,50 @@
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D109" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E109" s="1">
+        <v>3</v>
+      </c>
+      <c r="F109" s="1">
         <v>5</v>
       </c>
-      <c r="F109" s="1">
-        <v>6</v>
-      </c>
       <c r="G109" s="1">
         <v>6</v>
       </c>
       <c r="H109" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I109" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D110" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E110" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F110" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
         <v>5.8</v>
@@ -7278,260 +7281,260 @@
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D111" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E111" s="1">
         <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G111" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H111" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I111" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E112" s="1">
         <v>6</v>
       </c>
       <c r="F112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H112" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I112" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E113" s="1">
+        <v>6</v>
+      </c>
+      <c r="F113" s="1">
         <v>5</v>
       </c>
-      <c r="F113" s="1">
-        <v>6</v>
-      </c>
       <c r="G113" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H113" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I113" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D114" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F114" s="1">
         <v>6</v>
       </c>
       <c r="G114" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H114" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I114" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D115" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H115" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I115" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D116" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E116" s="1">
         <v>5</v>
       </c>
       <c r="F116" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G116" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H116" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I116" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D117" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E117" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F117" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
         <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I117" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.05</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E118" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F118" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G118" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I118" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D119" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E119" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F119" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G119" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H119" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I119" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E120" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F120" s="1">
         <v>5</v>
@@ -7540,397 +7543,397 @@
         <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I120" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D121" s="1">
+        <v>6</v>
+      </c>
+      <c r="E121" s="1">
+        <v>3</v>
+      </c>
+      <c r="F121" s="1">
         <v>5</v>
       </c>
-      <c r="E121" s="1">
-        <v>5</v>
-      </c>
-      <c r="F121" s="1">
-        <v>3</v>
-      </c>
       <c r="G121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I121" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D122" s="1">
         <v>5</v>
       </c>
       <c r="E122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F122" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G122" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H122" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I122" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I122" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D123" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E123" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F123" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G123" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H123" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I123" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D124" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E124" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F124" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G124" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H124" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I124" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D125" s="1">
         <v>5</v>
       </c>
       <c r="E125" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F125" s="1">
         <v>5</v>
       </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H125" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I125" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D126" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E126" s="1">
         <v>4</v>
       </c>
       <c r="F126" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G126" s="1">
         <v>5</v>
       </c>
       <c r="H126" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I126" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D127" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E127" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F127" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G127" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H127" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I127" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D128" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E128" s="1">
+        <v>0</v>
+      </c>
+      <c r="F128" s="1">
         <v>2</v>
       </c>
-      <c r="F128" s="1">
-        <v>4</v>
-      </c>
       <c r="G128" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H128" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I128" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D129" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E129" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F129" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G129" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H129" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I129" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D130" s="1">
+        <v>5</v>
+      </c>
+      <c r="E130" s="1">
         <v>3</v>
       </c>
-      <c r="E130" s="1">
-        <v>4</v>
-      </c>
       <c r="F130" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G130" s="1">
         <v>4</v>
       </c>
       <c r="H130" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I130" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D131" s="1">
+        <v>3</v>
+      </c>
+      <c r="E131" s="1">
         <v>4</v>
       </c>
-      <c r="E131" s="1">
-        <v>3</v>
-      </c>
       <c r="F131" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G131" s="1">
         <v>4</v>
       </c>
       <c r="H131" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I131" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D132" s="1">
         <v>4</v>
       </c>
       <c r="E132" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F132" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G132" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H132" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I132" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D133" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E133" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F133" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H133" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I133" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D134" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E134" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F134" s="1">
         <v>2</v>
       </c>
       <c r="G134" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H134" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I134" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D135" s="1">
         <v>3</v>
@@ -7939,150 +7942,177 @@
         <v>3</v>
       </c>
       <c r="F135" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G135" s="1">
         <v>4</v>
       </c>
       <c r="H135" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I135" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I135" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D136" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E136" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F136" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G136" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H136" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I136" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D137" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E137" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="1">
         <v>2</v>
       </c>
       <c r="G137" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H137" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I137" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D138" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E138" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F138" s="1">
         <v>2</v>
       </c>
       <c r="G138" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H138" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I138" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D139" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E139" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F139" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G139" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H139" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I139" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D140" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E140" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F140" s="1">
         <v>0</v>
       </c>
       <c r="G140" s="1">
+        <v>1</v>
+      </c>
+      <c r="H140" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I140" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="141" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B141" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C141" s="5">
+        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D141" s="1">
         <v>0</v>
       </c>
-      <c r="H140" s="3">
+      <c r="E141" s="1">
+        <v>0</v>
+      </c>
+      <c r="F141" s="1">
+        <v>0</v>
+      </c>
+      <c r="G141" s="1">
+        <v>0</v>
+      </c>
+      <c r="H141" s="3">
         <v>7.6</v>
       </c>
-      <c r="I140" s="3">
+      <c r="I141" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 121 "53 domingos"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15DB091B-D745-4F35-AE3F-CB94841FCF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F761F992-8443-4F19-9150-ED81B1472C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="223">
   <si>
     <t>Película</t>
   </si>
@@ -1242,6 +1242,9 @@
   </si>
   <si>
     <t>El falsificador</t>
+  </si>
+  <si>
+    <t>53 domingos</t>
   </si>
 </sst>
 </file>
@@ -1594,10 +1597,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I141" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I141" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I141">
-    <sortCondition descending="1" ref="C2:C141"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I142" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I142" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I142">
+    <sortCondition descending="1" ref="C2:C142"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4319,7 +4322,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K141"/>
+  <dimension ref="B2:K142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -6173,7 +6176,7 @@
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B70" s="9" t="s">
+      <c r="B70" s="2" t="s">
         <v>221</v>
       </c>
       <c r="C70" s="5">
@@ -6983,12 +6986,12 @@
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B100" s="2" t="s">
-        <v>214</v>
+      <c r="B100" s="9" t="s">
+        <v>222</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D100" s="1">
         <v>7</v>
@@ -6997,25 +7000,25 @@
         <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G100" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H100" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I100" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D101" s="1">
         <v>7</v>
@@ -7027,49 +7030,49 @@
         <v>7</v>
       </c>
       <c r="G101" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H101" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I101" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
         <v>6.05</v>
       </c>
       <c r="D102" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E102" s="1">
         <v>6</v>
       </c>
       <c r="F102" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G102" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H102" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I102" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D103" s="1">
         <v>6</v>
@@ -7078,133 +7081,133 @@
         <v>6</v>
       </c>
       <c r="F103" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G103" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H103" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I103" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D104" s="1">
         <v>6</v>
       </c>
       <c r="E104" s="1">
+        <v>6</v>
+      </c>
+      <c r="F104" s="1">
+        <v>8</v>
+      </c>
+      <c r="G104" s="1">
         <v>5</v>
       </c>
-      <c r="F104" s="1">
-        <v>6</v>
-      </c>
-      <c r="G104" s="1">
-        <v>6</v>
-      </c>
       <c r="H104" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I104" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E105" s="1">
         <v>5</v>
       </c>
       <c r="F105" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I105" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
       </c>
       <c r="E106" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F106" s="1">
         <v>5</v>
       </c>
       <c r="G106" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H106" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I106" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D107" s="1">
         <v>7</v>
       </c>
       <c r="E107" s="1">
+        <v>6</v>
+      </c>
+      <c r="F107" s="1">
         <v>5</v>
       </c>
-      <c r="F107" s="1">
-        <v>4</v>
-      </c>
       <c r="G107" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H107" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I107" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D108" s="1">
         <v>7</v>
@@ -7216,37 +7219,37 @@
         <v>4</v>
       </c>
       <c r="G108" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H108" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I108" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D109" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E109" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F109" s="1">
+        <v>4</v>
+      </c>
+      <c r="G109" s="1">
         <v>5</v>
       </c>
-      <c r="G109" s="1">
-        <v>6</v>
-      </c>
       <c r="H109" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I109" s="3">
         <v>6.4</v>
@@ -7254,50 +7257,50 @@
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D110" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E110" s="1">
+        <v>3</v>
+      </c>
+      <c r="F110" s="1">
         <v>5</v>
       </c>
-      <c r="F110" s="1">
-        <v>6</v>
-      </c>
       <c r="G110" s="1">
         <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I110" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D111" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E111" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F111" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H111" s="3">
         <v>5.8</v>
@@ -7308,260 +7311,260 @@
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D112" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E112" s="1">
         <v>6</v>
       </c>
       <c r="F112" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H112" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I112" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E113" s="1">
         <v>6</v>
       </c>
       <c r="F113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I113" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E114" s="1">
+        <v>6</v>
+      </c>
+      <c r="F114" s="1">
         <v>5</v>
       </c>
-      <c r="F114" s="1">
-        <v>6</v>
-      </c>
       <c r="G114" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H114" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I114" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D115" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E115" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F115" s="1">
         <v>6</v>
       </c>
       <c r="G115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H115" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I115" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D116" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I116" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D117" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E117" s="1">
         <v>5</v>
       </c>
       <c r="F117" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G117" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H117" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I117" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E118" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F118" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G118" s="1">
         <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I118" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.05</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E119" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F119" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G119" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I119" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D120" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E120" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F120" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G120" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H120" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I120" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D121" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E121" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F121" s="1">
         <v>5</v>
@@ -7570,397 +7573,397 @@
         <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I121" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D122" s="1">
+        <v>6</v>
+      </c>
+      <c r="E122" s="1">
+        <v>3</v>
+      </c>
+      <c r="F122" s="1">
         <v>5</v>
       </c>
-      <c r="E122" s="1">
-        <v>5</v>
-      </c>
-      <c r="F122" s="1">
-        <v>3</v>
-      </c>
       <c r="G122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H122" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I122" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D123" s="1">
         <v>5</v>
       </c>
       <c r="E123" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F123" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G123" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H123" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I123" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I123" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D124" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E124" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F124" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G124" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H124" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I124" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D125" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E125" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F125" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G125" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H125" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I125" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D126" s="1">
         <v>5</v>
       </c>
       <c r="E126" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
         <v>5</v>
       </c>
       <c r="G126" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H126" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I126" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D127" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E127" s="1">
         <v>4</v>
       </c>
       <c r="F127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G127" s="1">
         <v>5</v>
       </c>
       <c r="H127" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I127" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D128" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E128" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F128" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G128" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I128" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D129" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E129" s="1">
+        <v>0</v>
+      </c>
+      <c r="F129" s="1">
         <v>2</v>
       </c>
-      <c r="F129" s="1">
-        <v>4</v>
-      </c>
       <c r="G129" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H129" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I129" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D130" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E130" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F130" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G130" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H130" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I130" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D131" s="1">
+        <v>5</v>
+      </c>
+      <c r="E131" s="1">
         <v>3</v>
       </c>
-      <c r="E131" s="1">
-        <v>4</v>
-      </c>
       <c r="F131" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G131" s="1">
         <v>4</v>
       </c>
       <c r="H131" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I131" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D132" s="1">
+        <v>3</v>
+      </c>
+      <c r="E132" s="1">
         <v>4</v>
       </c>
-      <c r="E132" s="1">
-        <v>3</v>
-      </c>
       <c r="F132" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G132" s="1">
         <v>4</v>
       </c>
       <c r="H132" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I132" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D133" s="1">
         <v>4</v>
       </c>
       <c r="E133" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F133" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G133" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H133" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I133" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D134" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E134" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F134" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G134" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H134" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I134" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D135" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E135" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F135" s="1">
         <v>2</v>
       </c>
       <c r="G135" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H135" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I135" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D136" s="1">
         <v>3</v>
@@ -7969,150 +7972,177 @@
         <v>3</v>
       </c>
       <c r="F136" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G136" s="1">
         <v>4</v>
       </c>
       <c r="H136" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I136" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I136" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D137" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E137" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F137" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G137" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H137" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I137" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D138" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E138" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F138" s="1">
         <v>2</v>
       </c>
       <c r="G138" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H138" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I138" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D139" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E139" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F139" s="1">
         <v>2</v>
       </c>
       <c r="G139" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H139" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I139" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D140" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E140" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F140" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G140" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H140" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I140" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D141" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E141" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F141" s="1">
         <v>0</v>
       </c>
       <c r="G141" s="1">
+        <v>1</v>
+      </c>
+      <c r="H141" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I141" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="142" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B142" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C142" s="5">
+        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D142" s="1">
         <v>0</v>
       </c>
-      <c r="H141" s="3">
+      <c r="E142" s="1">
+        <v>0</v>
+      </c>
+      <c r="F142" s="1">
+        <v>0</v>
+      </c>
+      <c r="G142" s="1">
+        <v>0</v>
+      </c>
+      <c r="H142" s="3">
         <v>7.6</v>
       </c>
-      <c r="I141" s="3">
+      <c r="I142" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 122 "El cambiazo"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F761F992-8443-4F19-9150-ED81B1472C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9BC705-AB7E-4139-802D-96E6E3C2C9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="224">
   <si>
     <t>Película</t>
   </si>
@@ -1245,6 +1245,9 @@
   </si>
   <si>
     <t>53 domingos</t>
+  </si>
+  <si>
+    <t>El cambiazo</t>
   </si>
 </sst>
 </file>
@@ -1597,10 +1600,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I142" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I142" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I142">
-    <sortCondition descending="1" ref="C2:C142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I143" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I143" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I143">
+    <sortCondition descending="1" ref="C2:C143"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4322,7 +4325,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K142"/>
+  <dimension ref="B2:K143"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -6986,7 +6989,7 @@
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B100" s="9" t="s">
+      <c r="B100" s="2" t="s">
         <v>222</v>
       </c>
       <c r="C100" s="5">
@@ -7526,72 +7529,72 @@
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B120" s="2" t="s">
-        <v>21</v>
+      <c r="B120" s="9" t="s">
+        <v>223</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D120" s="1">
         <v>5</v>
       </c>
       <c r="E120" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F120" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G120" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H120" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I120" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D121" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E121" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F121" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G121" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H121" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I121" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D122" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E122" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F122" s="1">
         <v>5</v>
@@ -7600,397 +7603,397 @@
         <v>6</v>
       </c>
       <c r="H122" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I122" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D123" s="1">
+        <v>6</v>
+      </c>
+      <c r="E123" s="1">
+        <v>3</v>
+      </c>
+      <c r="F123" s="1">
         <v>5</v>
       </c>
-      <c r="E123" s="1">
-        <v>5</v>
-      </c>
-      <c r="F123" s="1">
-        <v>3</v>
-      </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I123" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D124" s="1">
         <v>5</v>
       </c>
       <c r="E124" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G124" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H124" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I124" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I124" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D125" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E125" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F125" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G125" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H125" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I125" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D126" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E126" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F126" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G126" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H126" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I126" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D127" s="1">
         <v>5</v>
       </c>
       <c r="E127" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F127" s="1">
         <v>5</v>
       </c>
       <c r="G127" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H127" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I127" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D128" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E128" s="1">
         <v>4</v>
       </c>
       <c r="F128" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G128" s="1">
         <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I128" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D129" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E129" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F129" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G129" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H129" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I129" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D130" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E130" s="1">
+        <v>0</v>
+      </c>
+      <c r="F130" s="1">
         <v>2</v>
       </c>
-      <c r="F130" s="1">
-        <v>4</v>
-      </c>
       <c r="G130" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H130" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I130" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D131" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E131" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F131" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G131" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H131" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I131" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D132" s="1">
+        <v>5</v>
+      </c>
+      <c r="E132" s="1">
         <v>3</v>
       </c>
-      <c r="E132" s="1">
-        <v>4</v>
-      </c>
       <c r="F132" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G132" s="1">
         <v>4</v>
       </c>
       <c r="H132" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I132" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D133" s="1">
+        <v>3</v>
+      </c>
+      <c r="E133" s="1">
         <v>4</v>
       </c>
-      <c r="E133" s="1">
-        <v>3</v>
-      </c>
       <c r="F133" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G133" s="1">
         <v>4</v>
       </c>
       <c r="H133" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I133" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D134" s="1">
         <v>4</v>
       </c>
       <c r="E134" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F134" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G134" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H134" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I134" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D135" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E135" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F135" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I135" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D136" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F136" s="1">
         <v>2</v>
       </c>
       <c r="G136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I136" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D137" s="1">
         <v>3</v>
@@ -7999,150 +8002,177 @@
         <v>3</v>
       </c>
       <c r="F137" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G137" s="1">
         <v>4</v>
       </c>
       <c r="H137" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I137" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I137" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D138" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E138" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F138" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G138" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H138" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I138" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D139" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E139" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F139" s="1">
         <v>2</v>
       </c>
       <c r="G139" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H139" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I139" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D140" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E140" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="1">
         <v>2</v>
       </c>
       <c r="G140" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H140" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I140" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D141" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E141" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F141" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G141" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H141" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I141" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D142" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E142" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F142" s="1">
         <v>0</v>
       </c>
       <c r="G142" s="1">
+        <v>1</v>
+      </c>
+      <c r="H142" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I142" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="143" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B143" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C143" s="5">
+        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D143" s="1">
         <v>0</v>
       </c>
-      <c r="H142" s="3">
+      <c r="E143" s="1">
+        <v>0</v>
+      </c>
+      <c r="F143" s="1">
+        <v>0</v>
+      </c>
+      <c r="G143" s="1">
+        <v>0</v>
+      </c>
+      <c r="H143" s="3">
         <v>7.6</v>
       </c>
-      <c r="I142" s="3">
+      <c r="I143" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 123 "Ready Player One"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9BC705-AB7E-4139-802D-96E6E3C2C9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1DF647-B0CF-42BE-85CD-20671CEC2597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="225">
   <si>
     <t>Película</t>
   </si>
@@ -1248,6 +1248,9 @@
   </si>
   <si>
     <t>El cambiazo</t>
+  </si>
+  <si>
+    <t>Ready Player One</t>
   </si>
 </sst>
 </file>
@@ -1600,10 +1603,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I143" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I143" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I143">
-    <sortCondition descending="1" ref="C2:C143"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I144" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I144" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I144">
+    <sortCondition descending="1" ref="C2:C144"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4325,7 +4328,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K143"/>
+  <dimension ref="B2:K144"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5666,72 +5669,72 @@
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B51" s="2" t="s">
-        <v>111</v>
+      <c r="B51" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="C51" s="5">
         <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
-        <v>7.3</v>
+        <v>7.3125</v>
       </c>
       <c r="D51" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E51" s="1">
         <v>7</v>
       </c>
       <c r="F51" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G51" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H51" s="3">
-        <v>6.5</v>
+        <v>7.4</v>
       </c>
       <c r="I51" s="3">
-        <v>5.4</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C52" s="5">
         <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
-        <v>7.2750000000000004</v>
+        <v>7.3</v>
       </c>
       <c r="D52" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E52" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G52" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H52" s="3">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="I52" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="C53" s="5">
         <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D53" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E53" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F53" s="1">
         <v>8</v>
@@ -5740,25 +5743,25 @@
         <v>8</v>
       </c>
       <c r="H53" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="I53" s="3">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="C54" s="5">
         <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
-        <v>7.2374999999999998</v>
+        <v>7.2750000000000004</v>
       </c>
       <c r="D54" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E54" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F54" s="1">
         <v>8</v>
@@ -5767,127 +5770,127 @@
         <v>8</v>
       </c>
       <c r="H54" s="3">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="I54" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="C55" s="5">
         <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
-        <v>7.2250000000000005</v>
+        <v>7.2374999999999998</v>
       </c>
       <c r="D55" s="1">
         <v>7</v>
       </c>
       <c r="E55" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F55" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G55" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H55" s="3">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="I55" s="3">
-        <v>7.6</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C56" s="5">
         <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
-        <v>7.2125000000000004</v>
+        <v>7.2250000000000005</v>
       </c>
       <c r="D56" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E56" s="1">
         <v>7</v>
       </c>
       <c r="F56" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G56" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H56" s="3">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="I56" s="3">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>146</v>
+        <v>65</v>
       </c>
       <c r="C57" s="5">
         <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
-        <v>7.2124999999999995</v>
+        <v>7.2125000000000004</v>
       </c>
       <c r="D57" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E57" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G57" s="1">
         <v>8</v>
       </c>
       <c r="H57" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I57" s="3">
         <v>6.3</v>
-      </c>
-      <c r="I57" s="3">
-        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="C58" s="5">
         <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
-        <v>7.1999999999999993</v>
+        <v>7.2124999999999995</v>
       </c>
       <c r="D58" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E58" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F58" s="1">
         <v>9</v>
       </c>
       <c r="G58" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H58" s="3">
         <v>6.3</v>
       </c>
       <c r="I58" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="C59" s="5">
         <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
-        <v>7.1499999999999995</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D59" s="1">
         <v>8</v>
@@ -5896,217 +5899,217 @@
         <v>7</v>
       </c>
       <c r="F59" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G59" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H59" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I59" s="3">
-        <v>6.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="C60" s="5">
         <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
-        <v>7.1375000000000011</v>
+        <v>7.1499999999999995</v>
       </c>
       <c r="D60" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E60" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G60" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H60" s="3">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="I60" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="C61" s="5">
         <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
-        <v>7.1250000000000009</v>
+        <v>7.1375000000000011</v>
       </c>
       <c r="D61" s="1">
         <v>7</v>
       </c>
       <c r="E61" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F61" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G61" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H61" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I61" s="3">
         <v>6.7</v>
-      </c>
-      <c r="I61" s="3">
-        <v>6.6</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C62" s="5">
         <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
-        <v>7.125</v>
+        <v>7.1250000000000009</v>
       </c>
       <c r="D62" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E62" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F62" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G62" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H62" s="3">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="I62" s="3">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>133</v>
+        <v>39</v>
       </c>
       <c r="C63" s="5">
         <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
-        <v>7.0875000000000004</v>
+        <v>7.125</v>
       </c>
       <c r="D63" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E63" s="1">
         <v>8</v>
       </c>
       <c r="F63" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G63" s="1">
         <v>7</v>
       </c>
       <c r="H63" s="3">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="I63" s="3">
-        <v>6.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="C64" s="5">
         <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
-        <v>7.0750000000000011</v>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D64" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E64" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F64" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G64" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H64" s="3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="I64" s="3">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C65" s="5">
         <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D65" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F65" s="1">
         <v>8</v>
       </c>
       <c r="G65" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H65" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I65" s="3">
         <v>6.2</v>
-      </c>
-      <c r="I65" s="3">
-        <v>5.2</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="C66" s="5">
         <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
-        <v>7.0750000000000002</v>
+        <v>7.0750000000000011</v>
       </c>
       <c r="D66" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E66" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F66" s="1">
         <v>8</v>
       </c>
       <c r="G66" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H66" s="3">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="I66" s="3">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="C67" s="5">
         <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D67" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E67" s="1">
         <v>7</v>
@@ -6115,55 +6118,55 @@
         <v>8</v>
       </c>
       <c r="G67" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H67" s="3">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="I67" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="C68" s="5">
         <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
-        <v>7.0749999999999993</v>
+        <v>7.0750000000000002</v>
       </c>
       <c r="D68" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E68" s="1">
         <v>7</v>
       </c>
       <c r="F68" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G68" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H68" s="3">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="I68" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C69" s="5">
         <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
-        <v>7.05</v>
+        <v>7.0749999999999993</v>
       </c>
       <c r="D69" s="1">
         <v>8</v>
       </c>
       <c r="E69" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" s="1">
         <v>7</v>
@@ -6172,46 +6175,46 @@
         <v>8</v>
       </c>
       <c r="H69" s="3">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="I69" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>221</v>
+        <v>176</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
-        <v>7.0250000000000004</v>
+        <v>7.05</v>
       </c>
       <c r="D70" s="1">
         <v>8</v>
       </c>
       <c r="E70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F70" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H70" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="I70" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>95</v>
+        <v>221</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
-        <v>6.9375</v>
+        <v>7.0250000000000004</v>
       </c>
       <c r="D71" s="1">
         <v>8</v>
@@ -6223,22 +6226,22 @@
         <v>8</v>
       </c>
       <c r="G71" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H71" s="3">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="I71" s="3">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>164</v>
+        <v>95</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
-        <v>6.9124999999999996</v>
+        <v>6.9375</v>
       </c>
       <c r="D72" s="1">
         <v>8</v>
@@ -6250,72 +6253,72 @@
         <v>8</v>
       </c>
       <c r="G72" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H72" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="I72" s="3">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
-        <v>6.8999999999999995</v>
+        <v>6.9124999999999996</v>
       </c>
       <c r="D73" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E73" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F73" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G73" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H73" s="3">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="I73" s="3">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>88</v>
+        <v>157</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
-        <v>6.8624999999999989</v>
+        <v>6.8999999999999995</v>
       </c>
       <c r="D74" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E74" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G74" s="1">
         <v>8</v>
       </c>
       <c r="H74" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I74" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
-        <v>184</v>
+        <v>88</v>
       </c>
       <c r="C75" s="5">
         <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
@@ -6342,179 +6345,179 @@
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="2" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="C76" s="5">
         <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
-        <v>6.85</v>
+        <v>6.8624999999999989</v>
       </c>
       <c r="D76" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E76" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F76" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G76" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H76" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I76" s="3">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C77" s="5">
         <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
-        <v>6.7999999999999989</v>
+        <v>6.85</v>
       </c>
       <c r="D77" s="1">
         <v>8</v>
       </c>
       <c r="E77" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G77" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H77" s="3">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="I77" s="3">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
-        <v>57</v>
+        <v>196</v>
       </c>
       <c r="C78" s="5">
         <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
-        <v>6.6999999999999993</v>
+        <v>6.7999999999999989</v>
       </c>
       <c r="D78" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E78" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F78" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G78" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H78" s="3">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="I78" s="3">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
-        <v>6.6875</v>
+        <v>6.6999999999999993</v>
       </c>
       <c r="D79" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E79" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G79" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H79" s="3">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="I79" s="3">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.6375000000000002</v>
+        <v>6.6875</v>
       </c>
       <c r="D80" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E80" s="1">
         <v>7</v>
       </c>
       <c r="F80" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G80" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H80" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I80" s="3">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
-        <v>6.6374999999999993</v>
+        <v>6.6375000000000002</v>
       </c>
       <c r="D81" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E81" s="1">
         <v>7</v>
       </c>
       <c r="F81" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G81" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H81" s="3">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="I81" s="3">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D82" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E82" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F82" s="1">
         <v>8</v>
@@ -6523,106 +6526,106 @@
         <v>7</v>
       </c>
       <c r="H82" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I82" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D83" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E83" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G83" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H83" s="3">
         <v>6.3</v>
       </c>
       <c r="I83" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D84" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E84" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F84" s="1">
         <v>7</v>
       </c>
       <c r="G84" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H84" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I84" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D85" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E85" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" s="1">
         <v>7</v>
       </c>
       <c r="G85" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H85" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I85" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D86" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E86" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F86" s="1">
         <v>7</v>
@@ -6631,76 +6634,76 @@
         <v>6</v>
       </c>
       <c r="H86" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I86" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D87" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E87" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" s="1">
         <v>7</v>
       </c>
       <c r="G87" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H87" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I87" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D88" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E88" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F88" s="1">
         <v>7</v>
       </c>
       <c r="G88" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H88" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I88" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D89" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E89" s="1">
         <v>6</v>
@@ -6712,25 +6715,25 @@
         <v>7</v>
       </c>
       <c r="H89" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I89" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D90" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E90" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" s="1">
         <v>7</v>
@@ -6739,79 +6742,79 @@
         <v>7</v>
       </c>
       <c r="H90" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I90" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D91" s="1">
         <v>7</v>
       </c>
       <c r="E91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F91" s="1">
         <v>7</v>
       </c>
       <c r="G91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H91" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I91" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
         <v>6.35</v>
       </c>
       <c r="D92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G92" s="1">
         <v>6</v>
       </c>
       <c r="H92" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I92" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F93" s="1">
         <v>6</v>
@@ -6820,42 +6823,42 @@
         <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I93" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E94" s="1">
         <v>6</v>
       </c>
       <c r="F94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H94" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I94" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
@@ -6865,163 +6868,163 @@
         <v>6</v>
       </c>
       <c r="E95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I95" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F96" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G96" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H96" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I96" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D97" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" s="1">
         <v>8</v>
       </c>
       <c r="G97" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H97" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I97" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D98" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F98" s="1">
         <v>8</v>
       </c>
       <c r="G98" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H98" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I98" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D99" s="1">
         <v>7</v>
       </c>
       <c r="E99" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G99" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H99" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I99" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D100" s="1">
         <v>7</v>
       </c>
       <c r="E100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H100" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I100" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D101" s="1">
         <v>7</v>
@@ -7030,25 +7033,25 @@
         <v>6</v>
       </c>
       <c r="F101" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G101" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H101" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I101" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D102" s="1">
         <v>7</v>
@@ -7060,49 +7063,49 @@
         <v>7</v>
       </c>
       <c r="G102" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H102" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I102" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
         <v>6.05</v>
       </c>
       <c r="D103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E103" s="1">
         <v>6</v>
       </c>
       <c r="F103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H103" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I103" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D104" s="1">
         <v>6</v>
@@ -7111,133 +7114,133 @@
         <v>6</v>
       </c>
       <c r="F104" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G104" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H104" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I104" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D105" s="1">
         <v>6</v>
       </c>
       <c r="E105" s="1">
+        <v>6</v>
+      </c>
+      <c r="F105" s="1">
+        <v>8</v>
+      </c>
+      <c r="G105" s="1">
         <v>5</v>
       </c>
-      <c r="F105" s="1">
-        <v>6</v>
-      </c>
-      <c r="G105" s="1">
-        <v>6</v>
-      </c>
       <c r="H105" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I105" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E106" s="1">
         <v>5</v>
       </c>
       <c r="F106" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H106" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I106" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D107" s="1">
         <v>7</v>
       </c>
       <c r="E107" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F107" s="1">
         <v>5</v>
       </c>
       <c r="G107" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H107" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I107" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D108" s="1">
         <v>7</v>
       </c>
       <c r="E108" s="1">
+        <v>6</v>
+      </c>
+      <c r="F108" s="1">
         <v>5</v>
       </c>
-      <c r="F108" s="1">
-        <v>4</v>
-      </c>
       <c r="G108" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H108" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I108" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D109" s="1">
         <v>7</v>
@@ -7249,37 +7252,37 @@
         <v>4</v>
       </c>
       <c r="G109" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H109" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I109" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D110" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E110" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F110" s="1">
+        <v>4</v>
+      </c>
+      <c r="G110" s="1">
         <v>5</v>
       </c>
-      <c r="G110" s="1">
-        <v>6</v>
-      </c>
       <c r="H110" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I110" s="3">
         <v>6.4</v>
@@ -7287,50 +7290,50 @@
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D111" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E111" s="1">
+        <v>3</v>
+      </c>
+      <c r="F111" s="1">
         <v>5</v>
       </c>
-      <c r="F111" s="1">
-        <v>6</v>
-      </c>
       <c r="G111" s="1">
         <v>6</v>
       </c>
       <c r="H111" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I111" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D112" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F112" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H112" s="3">
         <v>5.8</v>
@@ -7341,287 +7344,287 @@
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D113" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E113" s="1">
         <v>6</v>
       </c>
       <c r="F113" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H113" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I113" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E114" s="1">
         <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I114" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D115" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E115" s="1">
+        <v>6</v>
+      </c>
+      <c r="F115" s="1">
         <v>5</v>
       </c>
-      <c r="F115" s="1">
-        <v>6</v>
-      </c>
       <c r="G115" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H115" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I115" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D116" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E116" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F116" s="1">
         <v>6</v>
       </c>
       <c r="G116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H116" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I116" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D117" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I117" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D118" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E118" s="1">
         <v>5</v>
       </c>
       <c r="F118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H118" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I118" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D119" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E119" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F119" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G119" s="1">
         <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I119" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B120" s="9" t="s">
-        <v>223</v>
+      <c r="B120" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E120" s="1">
         <v>4</v>
       </c>
       <c r="F120" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I120" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D121" s="1">
         <v>5</v>
       </c>
       <c r="E121" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F121" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G121" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H121" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I121" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D122" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E122" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F122" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H122" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I122" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D123" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E123" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F123" s="1">
         <v>5</v>
@@ -7630,397 +7633,397 @@
         <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I123" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D124" s="1">
+        <v>6</v>
+      </c>
+      <c r="E124" s="1">
+        <v>3</v>
+      </c>
+      <c r="F124" s="1">
         <v>5</v>
       </c>
-      <c r="E124" s="1">
-        <v>5</v>
-      </c>
-      <c r="F124" s="1">
-        <v>3</v>
-      </c>
       <c r="G124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H124" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I124" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D125" s="1">
         <v>5</v>
       </c>
       <c r="E125" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F125" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G125" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H125" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I125" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I125" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D126" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E126" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F126" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G126" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H126" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I126" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D127" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E127" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F127" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G127" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H127" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I127" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D128" s="1">
         <v>5</v>
       </c>
       <c r="E128" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F128" s="1">
         <v>5</v>
       </c>
       <c r="G128" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H128" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I128" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D129" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E129" s="1">
         <v>4</v>
       </c>
       <c r="F129" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G129" s="1">
         <v>5</v>
       </c>
       <c r="H129" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I129" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D130" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E130" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F130" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G130" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H130" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I130" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D131" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E131" s="1">
+        <v>0</v>
+      </c>
+      <c r="F131" s="1">
         <v>2</v>
       </c>
-      <c r="F131" s="1">
-        <v>4</v>
-      </c>
       <c r="G131" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H131" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I131" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D132" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E132" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F132" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G132" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H132" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I132" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D133" s="1">
+        <v>5</v>
+      </c>
+      <c r="E133" s="1">
         <v>3</v>
       </c>
-      <c r="E133" s="1">
-        <v>4</v>
-      </c>
       <c r="F133" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G133" s="1">
         <v>4</v>
       </c>
       <c r="H133" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I133" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D134" s="1">
+        <v>3</v>
+      </c>
+      <c r="E134" s="1">
         <v>4</v>
       </c>
-      <c r="E134" s="1">
-        <v>3</v>
-      </c>
       <c r="F134" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G134" s="1">
         <v>4</v>
       </c>
       <c r="H134" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I134" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D135" s="1">
         <v>4</v>
       </c>
       <c r="E135" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F135" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G135" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H135" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I135" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D136" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E136" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F136" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H136" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I136" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D137" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E137" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F137" s="1">
         <v>2</v>
       </c>
       <c r="G137" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H137" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I137" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D138" s="1">
         <v>3</v>
@@ -8029,150 +8032,177 @@
         <v>3</v>
       </c>
       <c r="F138" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G138" s="1">
         <v>4</v>
       </c>
       <c r="H138" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I138" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I138" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D139" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E139" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F139" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G139" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H139" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I139" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D140" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E140" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F140" s="1">
         <v>2</v>
       </c>
       <c r="G140" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H140" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I140" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D141" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E141" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F141" s="1">
         <v>2</v>
       </c>
       <c r="G141" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H141" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I141" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D142" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F142" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G142" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H142" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I142" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D143" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E143" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F143" s="1">
         <v>0</v>
       </c>
       <c r="G143" s="1">
+        <v>1</v>
+      </c>
+      <c r="H143" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I143" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="144" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B144" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C144" s="5">
+        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D144" s="1">
         <v>0</v>
       </c>
-      <c r="H143" s="3">
+      <c r="E144" s="1">
+        <v>0</v>
+      </c>
+      <c r="F144" s="1">
+        <v>0</v>
+      </c>
+      <c r="G144" s="1">
+        <v>0</v>
+      </c>
+      <c r="H144" s="3">
         <v>7.6</v>
       </c>
-      <c r="I143" s="3">
+      <c r="I144" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 125 "Bullet Train"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D353CC29-28E2-4ABE-ADAA-47235A9ACEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56C5991-37CA-4221-BE2A-C0701AB6649F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="226">
   <si>
     <t>Película</t>
   </si>
@@ -1251,6 +1251,9 @@
   </si>
   <si>
     <t>Ready Player One</t>
+  </si>
+  <si>
+    <t>Bullet Train</t>
   </si>
 </sst>
 </file>
@@ -1603,10 +1606,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I145" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I145" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I145">
-    <sortCondition descending="1" ref="C2:C145"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I146" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I146" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I146">
+    <sortCondition descending="1" ref="C2:C146"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4328,7 +4331,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K145"/>
+  <dimension ref="B2:K146"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5777,18 +5780,18 @@
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="2" t="s">
-        <v>147</v>
+      <c r="B55" s="9" t="s">
+        <v>225</v>
       </c>
       <c r="C55" s="5">
         <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
-        <v>7.2374999999999998</v>
+        <v>7.2624999999999993</v>
       </c>
       <c r="D55" s="1">
         <v>7</v>
       </c>
       <c r="E55" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F55" s="1">
         <v>8</v>
@@ -5797,127 +5800,127 @@
         <v>8</v>
       </c>
       <c r="H55" s="3">
-        <v>6</v>
+        <v>7.3</v>
       </c>
       <c r="I55" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="C56" s="5">
         <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
-        <v>7.2250000000000005</v>
+        <v>7.2374999999999998</v>
       </c>
       <c r="D56" s="1">
         <v>7</v>
       </c>
       <c r="E56" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F56" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G56" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H56" s="3">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="I56" s="3">
-        <v>7.6</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C57" s="5">
         <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
-        <v>7.2125000000000004</v>
+        <v>7.2250000000000005</v>
       </c>
       <c r="D57" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E57" s="1">
         <v>7</v>
       </c>
       <c r="F57" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G57" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H57" s="3">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="I57" s="3">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>146</v>
+        <v>65</v>
       </c>
       <c r="C58" s="5">
         <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
-        <v>7.2124999999999995</v>
+        <v>7.2125000000000004</v>
       </c>
       <c r="D58" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E58" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F58" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G58" s="1">
         <v>8</v>
       </c>
       <c r="H58" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I58" s="3">
         <v>6.3</v>
-      </c>
-      <c r="I58" s="3">
-        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="C59" s="5">
         <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
-        <v>7.1999999999999993</v>
+        <v>7.2124999999999995</v>
       </c>
       <c r="D59" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E59" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F59" s="1">
         <v>9</v>
       </c>
       <c r="G59" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H59" s="3">
         <v>6.3</v>
       </c>
       <c r="I59" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="C60" s="5">
         <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
-        <v>7.1499999999999995</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D60" s="1">
         <v>8</v>
@@ -5926,217 +5929,217 @@
         <v>7</v>
       </c>
       <c r="F60" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G60" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H60" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I60" s="3">
-        <v>6.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="C61" s="5">
         <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
-        <v>7.1375000000000011</v>
+        <v>7.1499999999999995</v>
       </c>
       <c r="D61" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E61" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F61" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G61" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H61" s="3">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="I61" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="C62" s="5">
         <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
-        <v>7.1250000000000009</v>
+        <v>7.1375000000000011</v>
       </c>
       <c r="D62" s="1">
         <v>7</v>
       </c>
       <c r="E62" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F62" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G62" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H62" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I62" s="3">
         <v>6.7</v>
-      </c>
-      <c r="I62" s="3">
-        <v>6.6</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C63" s="5">
         <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
-        <v>7.125</v>
+        <v>7.1250000000000009</v>
       </c>
       <c r="D63" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E63" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F63" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G63" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H63" s="3">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="I63" s="3">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>133</v>
+        <v>39</v>
       </c>
       <c r="C64" s="5">
         <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
-        <v>7.0875000000000004</v>
+        <v>7.125</v>
       </c>
       <c r="D64" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" s="1">
         <v>8</v>
       </c>
       <c r="F64" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G64" s="1">
         <v>7</v>
       </c>
       <c r="H64" s="3">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="I64" s="3">
-        <v>6.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="C65" s="5">
         <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
-        <v>7.0750000000000011</v>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D65" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E65" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F65" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G65" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H65" s="3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="I65" s="3">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C66" s="5">
         <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D66" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E66" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" s="1">
         <v>8</v>
       </c>
       <c r="G66" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H66" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I66" s="3">
         <v>6.2</v>
-      </c>
-      <c r="I66" s="3">
-        <v>5.2</v>
       </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="C67" s="5">
         <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
-        <v>7.0750000000000002</v>
+        <v>7.0750000000000011</v>
       </c>
       <c r="D67" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E67" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F67" s="1">
         <v>8</v>
       </c>
       <c r="G67" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H67" s="3">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="I67" s="3">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="C68" s="5">
         <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D68" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E68" s="1">
         <v>7</v>
@@ -6145,55 +6148,55 @@
         <v>8</v>
       </c>
       <c r="G68" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H68" s="3">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="I68" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="C69" s="5">
         <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
-        <v>7.0749999999999993</v>
+        <v>7.0750000000000002</v>
       </c>
       <c r="D69" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E69" s="1">
         <v>7</v>
       </c>
       <c r="F69" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G69" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H69" s="3">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="I69" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
-        <v>7.05</v>
+        <v>7.0749999999999993</v>
       </c>
       <c r="D70" s="1">
         <v>8</v>
       </c>
       <c r="E70" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" s="1">
         <v>7</v>
@@ -6202,46 +6205,46 @@
         <v>8</v>
       </c>
       <c r="H70" s="3">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="I70" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>221</v>
+        <v>176</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
-        <v>7.0250000000000004</v>
+        <v>7.05</v>
       </c>
       <c r="D71" s="1">
         <v>8</v>
       </c>
       <c r="E71" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F71" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G71" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H71" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="I71" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>95</v>
+        <v>221</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
-        <v>6.9375</v>
+        <v>7.0250000000000004</v>
       </c>
       <c r="D72" s="1">
         <v>8</v>
@@ -6253,22 +6256,22 @@
         <v>8</v>
       </c>
       <c r="G72" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H72" s="3">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="I72" s="3">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>164</v>
+        <v>95</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
-        <v>6.9124999999999996</v>
+        <v>6.9375</v>
       </c>
       <c r="D73" s="1">
         <v>8</v>
@@ -6280,72 +6283,72 @@
         <v>8</v>
       </c>
       <c r="G73" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H73" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="I73" s="3">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
-        <v>6.8999999999999995</v>
+        <v>6.9124999999999996</v>
       </c>
       <c r="D74" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E74" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F74" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G74" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H74" s="3">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="I74" s="3">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
-        <v>88</v>
+        <v>157</v>
       </c>
       <c r="C75" s="5">
         <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
-        <v>6.8624999999999989</v>
+        <v>6.8999999999999995</v>
       </c>
       <c r="D75" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E75" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G75" s="1">
         <v>8</v>
       </c>
       <c r="H75" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I75" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="2" t="s">
-        <v>184</v>
+        <v>88</v>
       </c>
       <c r="C76" s="5">
         <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
@@ -6372,179 +6375,179 @@
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="C77" s="5">
         <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
-        <v>6.85</v>
+        <v>6.8624999999999989</v>
       </c>
       <c r="D77" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E77" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F77" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G77" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H77" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I77" s="3">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C78" s="5">
         <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
-        <v>6.7999999999999989</v>
+        <v>6.85</v>
       </c>
       <c r="D78" s="1">
         <v>8</v>
       </c>
       <c r="E78" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G78" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H78" s="3">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="I78" s="3">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" s="2" t="s">
-        <v>57</v>
+        <v>196</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
-        <v>6.6999999999999993</v>
+        <v>6.7999999999999989</v>
       </c>
       <c r="D79" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E79" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F79" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G79" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H79" s="3">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="I79" s="3">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.6875</v>
+        <v>6.6999999999999993</v>
       </c>
       <c r="D80" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E80" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G80" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H80" s="3">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="I80" s="3">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
-        <v>6.6375000000000002</v>
+        <v>6.6875</v>
       </c>
       <c r="D81" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E81" s="1">
         <v>7</v>
       </c>
       <c r="F81" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G81" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H81" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I81" s="3">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
-        <v>6.6374999999999993</v>
+        <v>6.6375000000000002</v>
       </c>
       <c r="D82" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E82" s="1">
         <v>7</v>
       </c>
       <c r="F82" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G82" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H82" s="3">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="I82" s="3">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D83" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E83" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F83" s="1">
         <v>8</v>
@@ -6553,106 +6556,106 @@
         <v>7</v>
       </c>
       <c r="H83" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I83" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D84" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G84" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H84" s="3">
         <v>6.3</v>
       </c>
       <c r="I84" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D85" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E85" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F85" s="1">
         <v>7</v>
       </c>
       <c r="G85" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H85" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I85" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D86" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E86" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" s="1">
         <v>7</v>
       </c>
       <c r="G86" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H86" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I86" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D87" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E87" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F87" s="1">
         <v>7</v>
@@ -6661,76 +6664,76 @@
         <v>6</v>
       </c>
       <c r="H87" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I87" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D88" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E88" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" s="1">
         <v>7</v>
       </c>
       <c r="G88" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H88" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I88" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D89" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F89" s="1">
         <v>7</v>
       </c>
       <c r="G89" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H89" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I89" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D90" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E90" s="1">
         <v>6</v>
@@ -6742,25 +6745,25 @@
         <v>7</v>
       </c>
       <c r="H90" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I90" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D91" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" s="1">
         <v>7</v>
@@ -6769,79 +6772,79 @@
         <v>7</v>
       </c>
       <c r="H91" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I91" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D92" s="1">
         <v>7</v>
       </c>
       <c r="E92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F92" s="1">
         <v>7</v>
       </c>
       <c r="G92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H92" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I92" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
         <v>6.35</v>
       </c>
       <c r="D93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G93" s="1">
         <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I93" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F94" s="1">
         <v>6</v>
@@ -6850,42 +6853,42 @@
         <v>6</v>
       </c>
       <c r="H94" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I94" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E95" s="1">
         <v>6</v>
       </c>
       <c r="F95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H95" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I95" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
@@ -6895,163 +6898,163 @@
         <v>6</v>
       </c>
       <c r="E96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H96" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I96" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F97" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G97" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H97" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I97" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D98" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" s="1">
         <v>8</v>
       </c>
       <c r="G98" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H98" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I98" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D99" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F99" s="1">
         <v>8</v>
       </c>
       <c r="G99" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I99" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D100" s="1">
         <v>7</v>
       </c>
       <c r="E100" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G100" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H100" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I100" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D101" s="1">
         <v>7</v>
       </c>
       <c r="E101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H101" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I101" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D102" s="1">
         <v>7</v>
@@ -7060,25 +7063,25 @@
         <v>6</v>
       </c>
       <c r="F102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G102" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I102" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D103" s="1">
         <v>7</v>
@@ -7090,49 +7093,49 @@
         <v>7</v>
       </c>
       <c r="G103" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H103" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I103" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
         <v>6.05</v>
       </c>
       <c r="D104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E104" s="1">
         <v>6</v>
       </c>
       <c r="F104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H104" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I104" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D105" s="1">
         <v>6</v>
@@ -7141,133 +7144,133 @@
         <v>6</v>
       </c>
       <c r="F105" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G105" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I105" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D106" s="1">
         <v>6</v>
       </c>
       <c r="E106" s="1">
+        <v>6</v>
+      </c>
+      <c r="F106" s="1">
+        <v>8</v>
+      </c>
+      <c r="G106" s="1">
         <v>5</v>
       </c>
-      <c r="F106" s="1">
-        <v>6</v>
-      </c>
-      <c r="G106" s="1">
-        <v>6</v>
-      </c>
       <c r="H106" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I106" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D107" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E107" s="1">
         <v>5</v>
       </c>
       <c r="F107" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G107" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H107" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I107" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D108" s="1">
         <v>7</v>
       </c>
       <c r="E108" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F108" s="1">
         <v>5</v>
       </c>
       <c r="G108" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H108" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I108" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D109" s="1">
         <v>7</v>
       </c>
       <c r="E109" s="1">
+        <v>6</v>
+      </c>
+      <c r="F109" s="1">
         <v>5</v>
       </c>
-      <c r="F109" s="1">
-        <v>4</v>
-      </c>
       <c r="G109" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H109" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I109" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D110" s="1">
         <v>7</v>
@@ -7279,37 +7282,37 @@
         <v>4</v>
       </c>
       <c r="G110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I110" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D111" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E111" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F111" s="1">
+        <v>4</v>
+      </c>
+      <c r="G111" s="1">
         <v>5</v>
       </c>
-      <c r="G111" s="1">
-        <v>6</v>
-      </c>
       <c r="H111" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I111" s="3">
         <v>6.4</v>
@@ -7317,50 +7320,50 @@
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D112" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E112" s="1">
+        <v>3</v>
+      </c>
+      <c r="F112" s="1">
         <v>5</v>
       </c>
-      <c r="F112" s="1">
-        <v>6</v>
-      </c>
       <c r="G112" s="1">
         <v>6</v>
       </c>
       <c r="H112" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I112" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D113" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F113" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
         <v>5.8</v>
@@ -7371,287 +7374,287 @@
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D114" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E114" s="1">
         <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H114" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I114" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E115" s="1">
         <v>6</v>
       </c>
       <c r="F115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H115" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I115" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D116" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E116" s="1">
+        <v>6</v>
+      </c>
+      <c r="F116" s="1">
         <v>5</v>
       </c>
-      <c r="F116" s="1">
-        <v>6</v>
-      </c>
       <c r="G116" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H116" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I116" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D117" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E117" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F117" s="1">
         <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H117" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I117" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D118" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I118" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D119" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E119" s="1">
         <v>5</v>
       </c>
       <c r="F119" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G119" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H119" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I119" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E120" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F120" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
         <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I120" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E121" s="1">
         <v>4</v>
       </c>
       <c r="F121" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I121" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D122" s="1">
         <v>5</v>
       </c>
       <c r="E122" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F122" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G122" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H122" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I122" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D123" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E123" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F123" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G123" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H123" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I123" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D124" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E124" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
         <v>5</v>
@@ -7660,397 +7663,397 @@
         <v>6</v>
       </c>
       <c r="H124" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I124" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D125" s="1">
+        <v>6</v>
+      </c>
+      <c r="E125" s="1">
+        <v>3</v>
+      </c>
+      <c r="F125" s="1">
         <v>5</v>
       </c>
-      <c r="E125" s="1">
-        <v>5</v>
-      </c>
-      <c r="F125" s="1">
-        <v>3</v>
-      </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H125" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I125" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D126" s="1">
         <v>5</v>
       </c>
       <c r="E126" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G126" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H126" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I126" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I126" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D127" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E127" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F127" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G127" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H127" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I127" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D128" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E128" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F128" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G128" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H128" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I128" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D129" s="1">
         <v>5</v>
       </c>
       <c r="E129" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F129" s="1">
         <v>5</v>
       </c>
       <c r="G129" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H129" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I129" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D130" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E130" s="1">
         <v>4</v>
       </c>
       <c r="F130" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G130" s="1">
         <v>5</v>
       </c>
       <c r="H130" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I130" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D131" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E131" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F131" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H131" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I131" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D132" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E132" s="1">
+        <v>0</v>
+      </c>
+      <c r="F132" s="1">
         <v>2</v>
       </c>
-      <c r="F132" s="1">
-        <v>4</v>
-      </c>
       <c r="G132" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H132" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I132" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D133" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E133" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F133" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G133" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H133" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I133" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D134" s="1">
+        <v>5</v>
+      </c>
+      <c r="E134" s="1">
         <v>3</v>
       </c>
-      <c r="E134" s="1">
-        <v>4</v>
-      </c>
       <c r="F134" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G134" s="1">
         <v>4</v>
       </c>
       <c r="H134" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I134" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D135" s="1">
+        <v>3</v>
+      </c>
+      <c r="E135" s="1">
         <v>4</v>
       </c>
-      <c r="E135" s="1">
-        <v>3</v>
-      </c>
       <c r="F135" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G135" s="1">
         <v>4</v>
       </c>
       <c r="H135" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I135" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D136" s="1">
         <v>4</v>
       </c>
       <c r="E136" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F136" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G136" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H136" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I136" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D137" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E137" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F137" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H137" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I137" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D138" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E138" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F138" s="1">
         <v>2</v>
       </c>
       <c r="G138" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H138" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I138" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D139" s="1">
         <v>3</v>
@@ -8059,25 +8062,25 @@
         <v>3</v>
       </c>
       <c r="F139" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G139" s="1">
         <v>4</v>
       </c>
       <c r="H139" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I139" s="3">
         <v>4.8</v>
       </c>
-      <c r="I139" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B140" s="9">
-        <v>180</v>
+      <c r="B140" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D140" s="1">
         <v>3</v>
@@ -8089,147 +8092,174 @@
         <v>3</v>
       </c>
       <c r="G140" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H140" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I140" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B141" s="2" t="s">
-        <v>216</v>
+      <c r="B141" s="2">
+        <v>180</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D141" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E141" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F141" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G141" s="1">
         <v>3</v>
       </c>
       <c r="H141" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I141" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D142" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E142" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F142" s="1">
         <v>2</v>
       </c>
       <c r="G142" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H142" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I142" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D143" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E143" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F143" s="1">
         <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H143" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I143" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D144" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G144" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H144" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I144" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D145" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E145" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F145" s="1">
         <v>0</v>
       </c>
       <c r="G145" s="1">
+        <v>1</v>
+      </c>
+      <c r="H145" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I145" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="146" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B146" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C146" s="5">
+        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D146" s="1">
         <v>0</v>
       </c>
-      <c r="H145" s="3">
+      <c r="E146" s="1">
+        <v>0</v>
+      </c>
+      <c r="F146" s="1">
+        <v>0</v>
+      </c>
+      <c r="G146" s="1">
+        <v>0</v>
+      </c>
+      <c r="H146" s="3">
         <v>7.6</v>
       </c>
-      <c r="I145" s="3">
+      <c r="I146" s="3">
         <v>5.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 126 "Superagente Makey"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56C5991-37CA-4221-BE2A-C0701AB6649F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23F80F7-65FF-4A70-A24A-9B640D9210B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="227">
   <si>
     <t>Película</t>
   </si>
@@ -1254,6 +1254,9 @@
   </si>
   <si>
     <t>Bullet Train</t>
+  </si>
+  <si>
+    <t>Superagente Makey</t>
   </si>
 </sst>
 </file>
@@ -1606,10 +1609,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I146" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I146" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I146">
-    <sortCondition descending="1" ref="C2:C146"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I147" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I147" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I147">
+    <sortCondition descending="1" ref="C2:C147"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4331,7 +4334,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K146"/>
+  <dimension ref="B2:K147"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5780,7 +5783,7 @@
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="9" t="s">
+      <c r="B55" s="2" t="s">
         <v>225</v>
       </c>
       <c r="C55" s="5">
@@ -8261,6 +8264,33 @@
       </c>
       <c r="I146" s="3">
         <v>5.9</v>
+      </c>
+    </row>
+    <row r="147" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B147" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="C147" s="5">
+        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <v>2.5125000000000002</v>
+      </c>
+      <c r="D147" s="1">
+        <v>2</v>
+      </c>
+      <c r="E147" s="1">
+        <v>1</v>
+      </c>
+      <c r="F147" s="1">
+        <v>2</v>
+      </c>
+      <c r="G147" s="1">
+        <v>2</v>
+      </c>
+      <c r="H147" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="I147" s="3">
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V. 127 "Machos alfa"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23F80F7-65FF-4A70-A24A-9B640D9210B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67028EBE-AA42-4C49-A9A6-3805D248FA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -78,6 +78,7 @@
     <author>tc={3E762906-7E78-4A82-82BD-91226BEEE65F}</author>
     <author>tc={A836A830-A167-47D8-ADFF-FC6A88D1B4AF}</author>
     <author>tc={153818FB-95E4-42BD-AB45-ADAC7CCB6F82}</author>
+    <author>tc={83190950-04EC-4A0B-AFCD-A5040D1110EE}</author>
     <author>tc={3D8C30B1-4F7A-4A97-801E-73E85EF747E6}</author>
     <author>tc={008FAA73-DE5D-4913-AE22-80AE836D5D61}</author>
     <author>tc={5698F250-EDD4-45DE-B2E5-000AD058A767}</author>
@@ -405,7 +406,15 @@
     14 temporadas</t>
       </text>
     </comment>
-    <comment ref="B49" authorId="39" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+    <comment ref="B49" authorId="39" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    5 temporadas</t>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -413,7 +422,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -421,7 +430,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="41" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+    <comment ref="B54" authorId="42" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -429,7 +438,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B54" authorId="42" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+    <comment ref="B55" authorId="43" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -437,7 +446,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B55" authorId="43" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+    <comment ref="B56" authorId="44" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -445,7 +454,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B56" authorId="44" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -453,7 +462,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -461,7 +470,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B63" authorId="46" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+    <comment ref="B64" authorId="47" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -469,7 +478,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B64" authorId="47" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B65" authorId="48" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -477,7 +486,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B65" authorId="48" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B66" authorId="49" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -485,7 +494,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B66" authorId="49" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -493,7 +502,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -501,7 +510,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -576,7 +585,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="228">
   <si>
     <t>Película</t>
   </si>
@@ -1257,6 +1266,9 @@
   </si>
   <si>
     <t>Superagente Makey</t>
+  </si>
+  <si>
+    <t>Machos alfa</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1278,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1302,6 +1314,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1345,7 +1363,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1368,9 +1386,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1583,10 +1598,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M68" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M68" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M68">
-    <sortCondition descending="1" ref="C2:C68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M69" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M69" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M69">
+    <sortCondition descending="1" ref="C2:C69"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -2010,43 +2025,46 @@
   <threadedComment ref="B47" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
     <text>14 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B49" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+  <threadedComment ref="B49" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+    <text>5 temporadas</text>
+  </threadedComment>
+  <threadedComment ref="B50" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B50" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+  <threadedComment ref="B51" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B53" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+  <threadedComment ref="B54" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B54" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+  <threadedComment ref="B55" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B55" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+  <threadedComment ref="B56" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B56" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+  <threadedComment ref="B57" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B57" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+  <threadedComment ref="B58" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B63" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+  <threadedComment ref="B64" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B64" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B65" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B65" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B66" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B66" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B67" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B67" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B68" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B68" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B69" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2058,7 +2076,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O68"/>
+  <dimension ref="B2:O69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -2120,7 +2138,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2154,7 +2172,7 @@
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2187,7 +2205,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2223,7 +2241,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2259,7 +2277,7 @@
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2293,7 +2311,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2326,7 +2344,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2359,7 +2377,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2392,7 +2410,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2425,7 +2443,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2460,7 +2478,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2495,7 +2513,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2528,7 +2546,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2561,7 +2579,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2596,7 +2614,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2629,7 +2647,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2662,7 +2680,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2695,7 +2713,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2726,7 +2744,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2759,7 +2777,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2792,7 +2810,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2825,7 +2843,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2858,7 +2876,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
         <v>7.8750000000000009</v>
       </c>
       <c r="D25" s="1">
@@ -2891,7 +2909,7 @@
         <v>43</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
         <v>7.8125000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -2924,7 +2942,7 @@
         <v>138</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
         <v>7.8125</v>
       </c>
       <c r="D27" s="1">
@@ -2957,7 +2975,7 @@
         <v>82</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
         <v>7.7874999999999996</v>
       </c>
       <c r="D28" s="1">
@@ -2990,7 +3008,7 @@
         <v>73</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
         <v>7.7250000000000005</v>
       </c>
       <c r="D29" s="1">
@@ -3025,7 +3043,7 @@
         <v>142</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D30" s="1">
@@ -3058,7 +3076,7 @@
         <v>192</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3091,7 +3109,7 @@
         <v>47</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
         <v>7.6000000000000005</v>
       </c>
       <c r="D32" s="1">
@@ -3124,7 +3142,7 @@
         <v>198</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
         <v>7.5625</v>
       </c>
       <c r="D33" s="1">
@@ -3157,7 +3175,7 @@
         <v>15</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D34" s="1">
@@ -3193,7 +3211,7 @@
         <v>210</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3226,7 +3244,7 @@
         <v>105</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D36" s="1">
@@ -3261,7 +3279,7 @@
         <v>141</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3294,7 +3312,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
         <v>7.4874999999999989</v>
       </c>
       <c r="D38" s="1">
@@ -3326,7 +3344,7 @@
         <v>50</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
         <v>7.35</v>
       </c>
       <c r="D39" s="1">
@@ -3358,7 +3376,7 @@
         <v>185</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
         <v>7.3</v>
       </c>
       <c r="D40" s="1">
@@ -3391,7 +3409,7 @@
         <v>80</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
         <v>7.2500000000000009</v>
       </c>
       <c r="D41" s="1">
@@ -3424,7 +3442,7 @@
         <v>115</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
         <v>7.25</v>
       </c>
       <c r="D42" s="1">
@@ -3457,7 +3475,7 @@
         <v>29</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
         <v>7.2</v>
       </c>
       <c r="D43" s="1">
@@ -3492,7 +3510,7 @@
         <v>22</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
         <v>7.2</v>
       </c>
       <c r="D44" s="1">
@@ -3524,7 +3542,7 @@
         <v>140</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
         <v>7.1875000000000009</v>
       </c>
       <c r="D45" s="1">
@@ -3557,7 +3575,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
         <v>7.1875</v>
       </c>
       <c r="D46" s="1">
@@ -3590,7 +3608,7 @@
         <v>27</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -3624,7 +3642,7 @@
         <v>49</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D48" s="1">
@@ -3654,17 +3672,17 @@
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>71</v>
+        <v>227</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9750000000000005</v>
+        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D49" s="1">
         <v>6</v>
       </c>
       <c r="E49" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F49" s="1">
         <v>7</v>
@@ -3676,107 +3694,108 @@
         <v>7.7</v>
       </c>
       <c r="I49" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="J49" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K49" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9</v>
+        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
+        <v>6.9750000000000005</v>
       </c>
       <c r="D50" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F50" s="1">
         <v>7</v>
       </c>
       <c r="G50" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H50" s="3">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="I50" s="3">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="J50" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K50" s="1"/>
+      <c r="K50" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8750000000000009</v>
+        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <v>6.9</v>
       </c>
       <c r="D51" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E51" s="1">
         <v>6</v>
       </c>
       <c r="F51" s="1">
+        <v>7</v>
+      </c>
+      <c r="G51" s="1">
         <v>5</v>
       </c>
-      <c r="G51" s="1">
-        <v>7</v>
-      </c>
       <c r="H51" s="3">
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
       <c r="I51" s="3">
-        <v>8.6</v>
-      </c>
-      <c r="J51" s="1"/>
+        <v>7.2</v>
+      </c>
+      <c r="J51" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K51" s="1"/>
-      <c r="L51" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8</v>
+        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <v>6.8750000000000009</v>
       </c>
       <c r="D52" s="1">
         <v>6</v>
       </c>
       <c r="E52" s="1">
+        <v>6</v>
+      </c>
+      <c r="F52" s="1">
         <v>5</v>
       </c>
-      <c r="F52" s="1">
-        <v>6</v>
-      </c>
       <c r="G52" s="1">
         <v>7</v>
       </c>
       <c r="H52" s="3">
-        <v>8.5</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="I52" s="3">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
@@ -3786,17 +3805,17 @@
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7750000000000004</v>
+        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <v>6.8</v>
       </c>
       <c r="D53" s="1">
         <v>6</v>
       </c>
       <c r="E53" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F53" s="1">
         <v>6</v>
@@ -3805,43 +3824,42 @@
         <v>7</v>
       </c>
       <c r="H53" s="3">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="I53" s="3">
-        <v>6.8</v>
-      </c>
-      <c r="J53" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+      <c r="L53" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
-        <v>6.75</v>
+        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <v>6.7750000000000004</v>
       </c>
       <c r="D54" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E54" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F54" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G54" s="1">
         <v>7</v>
       </c>
       <c r="H54" s="3">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I54" s="3">
-        <v>4.2</v>
+        <v>6.8</v>
       </c>
       <c r="J54" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3852,61 +3870,62 @@
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7250000000000005</v>
+        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <v>6.75</v>
       </c>
       <c r="D55" s="1">
         <v>8</v>
       </c>
       <c r="E55" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F55" s="1">
         <v>7</v>
       </c>
       <c r="G55" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H55" s="3">
-        <v>7.7</v>
+        <v>5.9</v>
       </c>
       <c r="I55" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J55" s="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="J55" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K55" s="1"/>
-      <c r="L55" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7</v>
+        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <v>6.7250000000000005</v>
       </c>
       <c r="D56" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F56" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G56" s="1">
         <v>6</v>
       </c>
       <c r="H56" s="3">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
       <c r="I56" s="3">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
@@ -3916,79 +3935,76 @@
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
-        <v>6.55</v>
+        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <v>6.7</v>
       </c>
       <c r="D57" s="1">
         <v>5</v>
       </c>
       <c r="E57" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F57" s="1">
         <v>6</v>
       </c>
       <c r="G57" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H57" s="3">
-        <v>7</v>
+        <v>8.6</v>
       </c>
       <c r="I57" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J57" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K57" s="1"/>
-      <c r="L57" s="1"/>
-      <c r="M57" s="1"/>
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4875000000000007</v>
+        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <v>6.55</v>
       </c>
       <c r="D58" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E58" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F58" s="1">
         <v>6</v>
       </c>
       <c r="G58" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H58" s="3">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="I58" s="3">
-        <v>7.7</v>
-      </c>
-      <c r="J58" s="1"/>
-      <c r="K58" t="e" vm="2">
+        <v>5.4</v>
+      </c>
+      <c r="J58" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K58" s="1"/>
       <c r="L58" s="1"/>
-      <c r="M58" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="M58" s="1"/>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4</v>
+        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <v>6.4875000000000007</v>
       </c>
       <c r="D59" s="1">
         <v>6</v>
@@ -4000,46 +4016,48 @@
         <v>6</v>
       </c>
       <c r="G59" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H59" s="3">
         <v>8.1</v>
       </c>
       <c r="I59" s="3">
-        <v>6</v>
-      </c>
-      <c r="J59" t="e" vm="1">
+        <v>7.7</v>
+      </c>
+      <c r="J59" s="1"/>
+      <c r="K59" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K59" s="1"/>
       <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
+      <c r="M59" s="1" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <v>6.4</v>
       </c>
       <c r="D60" s="1">
         <v>6</v>
       </c>
       <c r="E60" s="1">
+        <v>6</v>
+      </c>
+      <c r="F60" s="1">
+        <v>6</v>
+      </c>
+      <c r="G60" s="1">
         <v>5</v>
       </c>
-      <c r="F60" s="1">
-        <v>6</v>
-      </c>
-      <c r="G60" s="1">
-        <v>6</v>
-      </c>
       <c r="H60" s="3">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="I60" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="J60" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4050,66 +4068,66 @@
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
-        <v>6.2250000000000005</v>
+        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D61" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E61" s="1">
         <v>5</v>
       </c>
       <c r="F61" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G61" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H61" s="3">
-        <v>8.1999999999999993</v>
+        <v>7.8</v>
       </c>
       <c r="I61" s="3">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="J61" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K61" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K61" s="1"/>
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1750000000000007</v>
+        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D62" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E62" s="1">
         <v>5</v>
       </c>
       <c r="F62" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G62" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H62" s="3">
-        <v>6.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I62" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="J62" s="1"/>
+        <v>6.4</v>
+      </c>
+      <c r="J62" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K62" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -4118,62 +4136,62 @@
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1624999999999996</v>
+        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <v>6.1750000000000007</v>
       </c>
       <c r="D63" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E63" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F63" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G63" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H63" s="3">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="I63" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="J63" t="e" vm="1">
+        <v>6.2</v>
+      </c>
+      <c r="J63" s="1"/>
+      <c r="K63" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K63" s="1"/>
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
-        <v>5.9749999999999996</v>
+        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D64" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E64" s="1">
         <v>7</v>
       </c>
       <c r="F64" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G64" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H64" s="3">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I64" s="3">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J64" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4184,29 +4202,29 @@
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
-        <v>5.7750000000000004</v>
+        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D65" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1">
         <v>7</v>
       </c>
       <c r="F65" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G65" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H65" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I65" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J65" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4217,29 +4235,29 @@
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
-        <v>5.7625000000000002</v>
+        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D66" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E66" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" s="1">
+        <v>7</v>
+      </c>
+      <c r="G66" s="1">
+        <v>3</v>
+      </c>
+      <c r="H66" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I66" s="3">
         <v>5</v>
-      </c>
-      <c r="G66" s="1">
-        <v>5</v>
-      </c>
-      <c r="H66" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I66" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J66" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4250,68 +4268,101 @@
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C68" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
-        <v>5.4625000000000004</v>
+        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D67" s="1">
+        <v>8</v>
+      </c>
+      <c r="E67" s="1">
+        <v>8</v>
+      </c>
+      <c r="F67" s="1">
         <v>5</v>
       </c>
-      <c r="E67" s="1">
-        <v>7</v>
-      </c>
-      <c r="F67" s="1">
-        <v>6</v>
-      </c>
       <c r="G67" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H67" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I67" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I67" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J67" s="1"/>
+      <c r="J67" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K67" s="1"/>
-      <c r="L67" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L67" s="1"/>
+      <c r="M67" s="1"/>
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C68" s="5">
+        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D68" s="1">
+        <v>5</v>
+      </c>
+      <c r="E68" s="1">
+        <v>7</v>
+      </c>
+      <c r="F68" s="1">
+        <v>6</v>
+      </c>
+      <c r="G68" s="1">
+        <v>7</v>
+      </c>
+      <c r="H68" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I68" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="L68" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B69" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C68" s="5">
-        <f t="shared" si="2"/>
+      <c r="C69" s="5">
+        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D69" s="1">
         <v>2</v>
       </c>
-      <c r="E68" s="1">
+      <c r="E69" s="1">
         <v>4</v>
       </c>
-      <c r="F68" s="1">
+      <c r="F69" s="1">
         <v>2</v>
       </c>
-      <c r="G68" s="1">
+      <c r="G69" s="1">
         <v>5</v>
       </c>
-      <c r="H68" s="3">
+      <c r="H69" s="3">
         <v>7.7</v>
       </c>
-      <c r="I68" s="3">
+      <c r="I69" s="3">
         <v>6.3</v>
       </c>
-      <c r="J68" t="e" vm="1">
+      <c r="J69" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
+      <c r="K69" s="1"/>
+      <c r="L69" s="1"/>
+      <c r="M69" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4381,7 +4432,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4409,7 +4460,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4437,7 +4488,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4464,7 +4515,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4491,7 +4542,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4518,7 +4569,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4545,7 +4596,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4572,7 +4623,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4599,7 +4650,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4626,7 +4677,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -4653,7 +4704,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -4680,7 +4731,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -4707,7 +4758,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -4734,7 +4785,7 @@
         <v>125</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.1750000000000007</v>
       </c>
       <c r="D16" s="1">
@@ -4761,7 +4812,7 @@
         <v>81</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.1624999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -4788,7 +4839,7 @@
         <v>77</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.15</v>
       </c>
       <c r="D18" s="1">
@@ -4815,7 +4866,7 @@
         <v>54</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D19" s="1">
@@ -4842,7 +4893,7 @@
         <v>126</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.0750000000000011</v>
       </c>
       <c r="D20" s="1">
@@ -4869,7 +4920,7 @@
         <v>58</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8.0625</v>
       </c>
       <c r="D21" s="1">
@@ -4896,7 +4947,7 @@
         <v>23</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>7.9249999999999998</v>
       </c>
       <c r="D22" s="1">
@@ -4923,7 +4974,7 @@
         <v>122</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>7.9124999999999996</v>
       </c>
       <c r="D23" s="1">
@@ -4950,7 +5001,7 @@
         <v>108</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>7.8999999999999995</v>
       </c>
       <c r="D24" s="1">
@@ -4977,7 +5028,7 @@
         <v>78</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.875</v>
       </c>
       <c r="D25" s="1">
@@ -5004,7 +5055,7 @@
         <v>109</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D26" s="1">
@@ -5031,7 +5082,7 @@
         <v>61</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5058,7 +5109,7 @@
         <v>193</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7750000000000004</v>
       </c>
       <c r="D28" s="1">
@@ -5085,7 +5136,7 @@
         <v>60</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7375000000000007</v>
       </c>
       <c r="D29" s="1">
@@ -5112,7 +5163,7 @@
         <v>38</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7000000000000011</v>
       </c>
       <c r="D30" s="1">
@@ -5139,7 +5190,7 @@
         <v>63</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999993</v>
       </c>
       <c r="D31" s="1">
@@ -5166,7 +5217,7 @@
         <v>123</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.5874999999999995</v>
       </c>
       <c r="D32" s="1">
@@ -5193,7 +5244,7 @@
         <v>37</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000011</v>
       </c>
       <c r="D33" s="1">
@@ -5220,7 +5271,7 @@
         <v>67</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000002</v>
       </c>
       <c r="D34" s="1">
@@ -5247,7 +5298,7 @@
         <v>62</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5625</v>
       </c>
       <c r="D35" s="1">
@@ -5274,7 +5325,7 @@
         <v>217</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5301,7 +5352,7 @@
         <v>55</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5624999999999991</v>
       </c>
       <c r="D37" s="1">
@@ -5328,7 +5379,7 @@
         <v>201</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.55</v>
       </c>
       <c r="D38" s="1">
@@ -5355,7 +5406,7 @@
         <v>69</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D39" s="1">
@@ -5382,7 +5433,7 @@
         <v>132</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.5125000000000002</v>
       </c>
       <c r="D40" s="1">
@@ -5409,7 +5460,7 @@
         <v>205</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.4875000000000007</v>
       </c>
       <c r="D41" s="1">
@@ -5436,7 +5487,7 @@
         <v>172</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.4749999999999996</v>
       </c>
       <c r="D42" s="1">
@@ -5463,7 +5514,7 @@
         <v>130</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D43" s="1">
@@ -5490,7 +5541,7 @@
         <v>97</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.4375</v>
       </c>
       <c r="D44" s="1">
@@ -5517,7 +5568,7 @@
         <v>100</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.4249999999999998</v>
       </c>
       <c r="D45" s="1">
@@ -5544,7 +5595,7 @@
         <v>131</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.4124999999999996</v>
       </c>
       <c r="D46" s="1">
@@ -5571,7 +5622,7 @@
         <v>220</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -5598,7 +5649,7 @@
         <v>175</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999989</v>
       </c>
       <c r="D48" s="1">
@@ -5625,7 +5676,7 @@
         <v>52</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.3500000000000005</v>
       </c>
       <c r="D49" s="1">
@@ -5652,7 +5703,7 @@
         <v>165</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.3249999999999993</v>
       </c>
       <c r="D50" s="1">
@@ -5679,7 +5730,7 @@
         <v>224</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.3125</v>
       </c>
       <c r="D51" s="1">
@@ -5706,7 +5757,7 @@
         <v>111</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D52" s="1">
@@ -5733,7 +5784,7 @@
         <v>103</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D53" s="1">
@@ -5760,7 +5811,7 @@
         <v>181</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D54" s="1">
@@ -5787,7 +5838,7 @@
         <v>225</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>7.2624999999999993</v>
       </c>
       <c r="D55" s="1">
@@ -5814,7 +5865,7 @@
         <v>147</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>7.2374999999999998</v>
       </c>
       <c r="D56" s="1">
@@ -5841,7 +5892,7 @@
         <v>59</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>7.2250000000000005</v>
       </c>
       <c r="D57" s="1">
@@ -5868,7 +5919,7 @@
         <v>65</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>7.2125000000000004</v>
       </c>
       <c r="D58" s="1">
@@ -5895,7 +5946,7 @@
         <v>146</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>7.2124999999999995</v>
       </c>
       <c r="D59" s="1">
@@ -5922,7 +5973,7 @@
         <v>94</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
       <c r="D60" s="1">
@@ -5949,7 +6000,7 @@
         <v>53</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="D61" s="1">
@@ -5976,7 +6027,7 @@
         <v>104</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>7.1375000000000011</v>
       </c>
       <c r="D62" s="1">
@@ -6003,7 +6054,7 @@
         <v>40</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>7.1250000000000009</v>
       </c>
       <c r="D63" s="1">
@@ -6030,7 +6081,7 @@
         <v>39</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>7.125</v>
       </c>
       <c r="D64" s="1">
@@ -6057,7 +6108,7 @@
         <v>133</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D65" s="1">
@@ -6084,7 +6135,7 @@
         <v>98</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D66" s="1">
@@ -6111,7 +6162,7 @@
         <v>171</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D67" s="1">
@@ -6138,7 +6189,7 @@
         <v>110</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D68" s="1">
@@ -6165,7 +6216,7 @@
         <v>143</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D69" s="1">
@@ -6192,7 +6243,7 @@
         <v>177</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>7.0749999999999993</v>
       </c>
       <c r="D70" s="1">
@@ -6219,7 +6270,7 @@
         <v>176</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="D71" s="1">
@@ -6246,7 +6297,7 @@
         <v>221</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="D72" s="1">
@@ -6273,7 +6324,7 @@
         <v>95</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>6.9375</v>
       </c>
       <c r="D73" s="1">
@@ -6300,7 +6351,7 @@
         <v>164</v>
       </c>
       <c r="C74" s="5">
-        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
+        <f t="shared" si="2"/>
         <v>6.9124999999999996</v>
       </c>
       <c r="D74" s="1">
@@ -6327,7 +6378,7 @@
         <v>157</v>
       </c>
       <c r="C75" s="5">
-        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
+        <f t="shared" si="2"/>
         <v>6.8999999999999995</v>
       </c>
       <c r="D75" s="1">
@@ -6354,7 +6405,7 @@
         <v>88</v>
       </c>
       <c r="C76" s="5">
-        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D76" s="1">
@@ -6381,7 +6432,7 @@
         <v>184</v>
       </c>
       <c r="C77" s="5">
-        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D77" s="1">
@@ -6408,7 +6459,7 @@
         <v>119</v>
       </c>
       <c r="C78" s="5">
-        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
+        <f t="shared" si="2"/>
         <v>6.85</v>
       </c>
       <c r="D78" s="1">
@@ -6435,7 +6486,7 @@
         <v>196</v>
       </c>
       <c r="C79" s="5">
-        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
+        <f t="shared" si="2"/>
         <v>6.7999999999999989</v>
       </c>
       <c r="D79" s="1">
@@ -6462,7 +6513,7 @@
         <v>57</v>
       </c>
       <c r="C80" s="5">
-        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
+        <f t="shared" si="2"/>
         <v>6.6999999999999993</v>
       </c>
       <c r="D80" s="1">
@@ -6489,7 +6540,7 @@
         <v>87</v>
       </c>
       <c r="C81" s="5">
-        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
+        <f t="shared" si="2"/>
         <v>6.6875</v>
       </c>
       <c r="D81" s="1">
@@ -6516,7 +6567,7 @@
         <v>211</v>
       </c>
       <c r="C82" s="5">
-        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
+        <f t="shared" si="2"/>
         <v>6.6375000000000002</v>
       </c>
       <c r="D82" s="1">
@@ -6543,7 +6594,7 @@
         <v>219</v>
       </c>
       <c r="C83" s="5">
-        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
+        <f t="shared" si="2"/>
         <v>6.6374999999999993</v>
       </c>
       <c r="D83" s="1">
@@ -6570,7 +6621,7 @@
         <v>41</v>
       </c>
       <c r="C84" s="5">
-        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999989</v>
       </c>
       <c r="D84" s="1">
@@ -6597,7 +6648,7 @@
         <v>117</v>
       </c>
       <c r="C85" s="5">
-        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D85" s="1">
@@ -6624,7 +6675,7 @@
         <v>179</v>
       </c>
       <c r="C86" s="5">
-        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D86" s="1">
@@ -6651,7 +6702,7 @@
         <v>215</v>
       </c>
       <c r="C87" s="5">
-        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
+        <f t="shared" si="2"/>
         <v>6.5750000000000002</v>
       </c>
       <c r="D87" s="1">
@@ -6678,7 +6729,7 @@
         <v>168</v>
       </c>
       <c r="C88" s="5">
-        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
+        <f t="shared" si="2"/>
         <v>6.5499999999999989</v>
       </c>
       <c r="D88" s="1">
@@ -6705,7 +6756,7 @@
         <v>197</v>
       </c>
       <c r="C89" s="5">
-        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
+        <f t="shared" si="2"/>
         <v>6.5375000000000005</v>
       </c>
       <c r="D89" s="1">
@@ -6732,7 +6783,7 @@
         <v>202</v>
       </c>
       <c r="C90" s="5">
-        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D90" s="1">
@@ -6759,7 +6810,7 @@
         <v>183</v>
       </c>
       <c r="C91" s="5">
-        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D91" s="1">
@@ -6786,7 +6837,7 @@
         <v>200</v>
       </c>
       <c r="C92" s="5">
-        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D92" s="1">
@@ -6813,7 +6864,7 @@
         <v>188</v>
       </c>
       <c r="C93" s="5">
-        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D93" s="1">
@@ -6840,7 +6891,7 @@
         <v>208</v>
       </c>
       <c r="C94" s="5">
-        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D94" s="1">
@@ -6867,7 +6918,7 @@
         <v>134</v>
       </c>
       <c r="C95" s="5">
-        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
+        <f t="shared" si="2"/>
         <v>6.3125</v>
       </c>
       <c r="D95" s="1">
@@ -6894,7 +6945,7 @@
         <v>144</v>
       </c>
       <c r="C96" s="5">
-        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <f t="shared" si="2"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D96" s="1">
@@ -6921,7 +6972,7 @@
         <v>64</v>
       </c>
       <c r="C97" s="5">
-        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
+        <f t="shared" si="2"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D97" s="1">
@@ -6948,7 +6999,7 @@
         <v>75</v>
       </c>
       <c r="C98" s="5">
-        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <f t="shared" si="2"/>
         <v>6.2125000000000004</v>
       </c>
       <c r="D98" s="1">
@@ -6975,7 +7026,7 @@
         <v>19</v>
       </c>
       <c r="C99" s="5">
-        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.2124999999999995</v>
       </c>
       <c r="D99" s="1">
@@ -7002,7 +7053,7 @@
         <v>101</v>
       </c>
       <c r="C100" s="5">
-        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
+        <f t="shared" si="3"/>
         <v>6.15</v>
       </c>
       <c r="D100" s="1">
@@ -7029,7 +7080,7 @@
         <v>158</v>
       </c>
       <c r="C101" s="5">
-        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <f t="shared" si="3"/>
         <v>6.0874999999999995</v>
       </c>
       <c r="D101" s="1">
@@ -7056,7 +7107,7 @@
         <v>222</v>
       </c>
       <c r="C102" s="5">
-        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <f t="shared" si="3"/>
         <v>6.0625</v>
       </c>
       <c r="D102" s="1">
@@ -7083,7 +7134,7 @@
         <v>214</v>
       </c>
       <c r="C103" s="5">
-        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <f t="shared" si="3"/>
         <v>6.0500000000000007</v>
       </c>
       <c r="D103" s="1">
@@ -7110,7 +7161,7 @@
         <v>160</v>
       </c>
       <c r="C104" s="5">
-        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D104" s="1">
@@ -7137,7 +7188,7 @@
         <v>206</v>
       </c>
       <c r="C105" s="5">
-        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D105" s="1">
@@ -7164,7 +7215,7 @@
         <v>159</v>
       </c>
       <c r="C106" s="5">
-        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <f t="shared" si="3"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="D106" s="1">
@@ -7191,7 +7242,7 @@
         <v>195</v>
       </c>
       <c r="C107" s="5">
-        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <f t="shared" si="3"/>
         <v>5.8875000000000011</v>
       </c>
       <c r="D107" s="1">
@@ -7218,7 +7269,7 @@
         <v>186</v>
       </c>
       <c r="C108" s="5">
-        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <f t="shared" si="3"/>
         <v>5.8125000000000009</v>
       </c>
       <c r="D108" s="1">
@@ -7245,7 +7296,7 @@
         <v>209</v>
       </c>
       <c r="C109" s="5">
-        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
+        <f t="shared" si="3"/>
         <v>5.8000000000000007</v>
       </c>
       <c r="D109" s="1">
@@ -7272,7 +7323,7 @@
         <v>113</v>
       </c>
       <c r="C110" s="5">
-        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <f t="shared" si="3"/>
         <v>5.7374999999999989</v>
       </c>
       <c r="D110" s="1">
@@ -7299,7 +7350,7 @@
         <v>187</v>
       </c>
       <c r="C111" s="5">
-        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <f t="shared" si="3"/>
         <v>5.7250000000000005</v>
       </c>
       <c r="D111" s="1">
@@ -7326,7 +7377,7 @@
         <v>26</v>
       </c>
       <c r="C112" s="5">
-        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <f t="shared" si="3"/>
         <v>5.6749999999999998</v>
       </c>
       <c r="D112" s="1">
@@ -7353,7 +7404,7 @@
         <v>149</v>
       </c>
       <c r="C113" s="5">
-        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D113" s="1">
@@ -7380,7 +7431,7 @@
         <v>156</v>
       </c>
       <c r="C114" s="5">
-        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D114" s="1">
@@ -7407,7 +7458,7 @@
         <v>166</v>
       </c>
       <c r="C115" s="5">
-        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D115" s="1">
@@ -7434,7 +7485,7 @@
         <v>191</v>
       </c>
       <c r="C116" s="5">
-        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D116" s="1">
@@ -7461,7 +7512,7 @@
         <v>204</v>
       </c>
       <c r="C117" s="5">
-        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <f t="shared" si="3"/>
         <v>5.3750000000000009</v>
       </c>
       <c r="D117" s="1">
@@ -7488,7 +7539,7 @@
         <v>190</v>
       </c>
       <c r="C118" s="5">
-        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
+        <f t="shared" si="3"/>
         <v>5.375</v>
       </c>
       <c r="D118" s="1">
@@ -7515,7 +7566,7 @@
         <v>182</v>
       </c>
       <c r="C119" s="5">
-        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <f t="shared" si="3"/>
         <v>5.2875000000000005</v>
       </c>
       <c r="D119" s="1">
@@ -7542,7 +7593,7 @@
         <v>74</v>
       </c>
       <c r="C120" s="5">
-        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <f t="shared" si="3"/>
         <v>5.1875</v>
       </c>
       <c r="D120" s="1">
@@ -7569,7 +7620,7 @@
         <v>145</v>
       </c>
       <c r="C121" s="5">
-        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <f t="shared" si="3"/>
         <v>5.1124999999999998</v>
       </c>
       <c r="D121" s="1">
@@ -7596,7 +7647,7 @@
         <v>223</v>
       </c>
       <c r="C122" s="5">
-        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
+        <f t="shared" si="3"/>
         <v>5.0750000000000002</v>
       </c>
       <c r="D122" s="1">
@@ -7623,7 +7674,7 @@
         <v>21</v>
       </c>
       <c r="C123" s="5">
-        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <f t="shared" si="3"/>
         <v>5.05</v>
       </c>
       <c r="D123" s="1">
@@ -7650,7 +7701,7 @@
         <v>203</v>
       </c>
       <c r="C124" s="5">
-        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <f t="shared" si="3"/>
         <v>4.9875000000000007</v>
       </c>
       <c r="D124" s="1">
@@ -7677,7 +7728,7 @@
         <v>169</v>
       </c>
       <c r="C125" s="5">
-        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <f t="shared" si="3"/>
         <v>4.9874999999999998</v>
       </c>
       <c r="D125" s="1">
@@ -7704,7 +7755,7 @@
         <v>163</v>
       </c>
       <c r="C126" s="5">
-        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <f t="shared" si="3"/>
         <v>4.8499999999999996</v>
       </c>
       <c r="D126" s="1">
@@ -7731,7 +7782,7 @@
         <v>162</v>
       </c>
       <c r="C127" s="5">
-        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <f t="shared" si="3"/>
         <v>4.7875000000000005</v>
       </c>
       <c r="D127" s="1">
@@ -7758,7 +7809,7 @@
         <v>213</v>
       </c>
       <c r="C128" s="5">
-        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <f t="shared" si="3"/>
         <v>4.6124999999999998</v>
       </c>
       <c r="D128" s="1">
@@ -7785,7 +7836,7 @@
         <v>154</v>
       </c>
       <c r="C129" s="5">
-        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <f t="shared" si="3"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="D129" s="1">
@@ -7812,7 +7863,7 @@
         <v>135</v>
       </c>
       <c r="C130" s="5">
-        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <f t="shared" si="3"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D130" s="1">
@@ -7839,7 +7890,7 @@
         <v>161</v>
       </c>
       <c r="C131" s="5">
-        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>4.4249999999999998</v>
       </c>
       <c r="D131" s="1">
@@ -7866,7 +7917,7 @@
         <v>114</v>
       </c>
       <c r="C132" s="5">
-        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <f t="shared" si="4"/>
         <v>4.4124999999999996</v>
       </c>
       <c r="D132" s="1">
@@ -7893,7 +7944,7 @@
         <v>207</v>
       </c>
       <c r="C133" s="5">
-        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <f t="shared" si="4"/>
         <v>4.3375000000000004</v>
       </c>
       <c r="D133" s="1">
@@ -7920,7 +7971,7 @@
         <v>150</v>
       </c>
       <c r="C134" s="5">
-        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <f t="shared" si="4"/>
         <v>4.3374999999999995</v>
       </c>
       <c r="D134" s="1">
@@ -7947,7 +7998,7 @@
         <v>173</v>
       </c>
       <c r="C135" s="5">
-        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <f t="shared" si="4"/>
         <v>4.3125</v>
       </c>
       <c r="D135" s="1">
@@ -7974,7 +8025,7 @@
         <v>212</v>
       </c>
       <c r="C136" s="5">
-        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <f t="shared" si="4"/>
         <v>4.3</v>
       </c>
       <c r="D136" s="1">
@@ -8001,7 +8052,7 @@
         <v>167</v>
       </c>
       <c r="C137" s="5">
-        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <f t="shared" si="4"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="D137" s="1">
@@ -8028,7 +8079,7 @@
         <v>68</v>
       </c>
       <c r="C138" s="5">
-        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <f t="shared" si="4"/>
         <v>4.1124999999999998</v>
       </c>
       <c r="D138" s="1">
@@ -8055,7 +8106,7 @@
         <v>218</v>
       </c>
       <c r="C139" s="5">
-        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <f t="shared" si="4"/>
         <v>3.9499999999999997</v>
       </c>
       <c r="D139" s="1">
@@ -8082,7 +8133,7 @@
         <v>199</v>
       </c>
       <c r="C140" s="5">
-        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <f t="shared" si="4"/>
         <v>3.7375000000000003</v>
       </c>
       <c r="D140" s="1">
@@ -8109,7 +8160,7 @@
         <v>180</v>
       </c>
       <c r="C141" s="5">
-        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <f t="shared" si="4"/>
         <v>3.5625000000000004</v>
       </c>
       <c r="D141" s="1">
@@ -8136,7 +8187,7 @@
         <v>216</v>
       </c>
       <c r="C142" s="5">
-        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <f t="shared" si="4"/>
         <v>3.5375000000000005</v>
       </c>
       <c r="D142" s="1">
@@ -8163,7 +8214,7 @@
         <v>189</v>
       </c>
       <c r="C143" s="5">
-        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <f t="shared" si="4"/>
         <v>3.3250000000000002</v>
       </c>
       <c r="D143" s="1">
@@ -8190,7 +8241,7 @@
         <v>194</v>
       </c>
       <c r="C144" s="5">
-        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <f t="shared" si="4"/>
         <v>3.2749999999999995</v>
       </c>
       <c r="D144" s="1">
@@ -8217,7 +8268,7 @@
         <v>155</v>
       </c>
       <c r="C145" s="5">
-        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <f t="shared" si="4"/>
         <v>2.9124999999999996</v>
       </c>
       <c r="D145" s="1">
@@ -8244,7 +8295,7 @@
         <v>174</v>
       </c>
       <c r="C146" s="5">
-        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <f t="shared" si="4"/>
         <v>2.6375000000000002</v>
       </c>
       <c r="D146" s="1">
@@ -8267,11 +8318,11 @@
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B147" s="9" t="s">
+      <c r="B147" s="2" t="s">
         <v>226</v>
       </c>
       <c r="C147" s="5">
-        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <f t="shared" si="4"/>
         <v>2.5125000000000002</v>
       </c>
       <c r="D147" s="1">

</xml_diff>

<commit_message>
V. 129 "Juego de armas"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAADD3B-F09F-4FCA-BF44-EF067D9174E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E408BF-7326-4328-BDE0-CF3B2DBD99E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="6015" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="233">
   <si>
     <t>Película</t>
   </si>
@@ -1290,6 +1290,9 @@
   </si>
   <si>
     <t>Berlín y la dama del armiño</t>
+  </si>
+  <si>
+    <t>Juego de armas</t>
   </si>
 </sst>
 </file>
@@ -1299,7 +1302,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1335,12 +1338,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1399,13 +1396,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1417,45 +1414,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1496,6 +1454,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1622,48 +1619,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M70" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M70" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M70" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M70">
     <sortCondition descending="1" ref="C2:C70"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I150" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I150" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I150">
-    <sortCondition descending="1" ref="C2:C150"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I151" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I151" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I151">
+    <sortCondition descending="1" ref="C2:C151"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2156,7 +2153,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2165,7 +2162,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2192,14 +2189,14 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2232,7 +2229,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2259,7 +2256,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2268,7 +2265,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2297,14 +2294,14 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2331,14 +2328,14 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2371,7 +2368,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2404,7 +2401,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2437,7 +2434,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2470,7 +2467,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2505,7 +2502,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2540,7 +2537,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2573,7 +2570,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2606,7 +2603,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2641,7 +2638,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2674,7 +2671,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2707,7 +2704,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2740,7 +2737,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2771,7 +2768,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2804,7 +2801,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2837,7 +2834,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2870,7 +2867,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2903,7 +2900,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.8750000000000009</v>
       </c>
       <c r="D25" s="1">
@@ -2936,7 +2933,7 @@
         <v>43</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.8125000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -2969,7 +2966,7 @@
         <v>138</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.8125</v>
       </c>
       <c r="D27" s="1">
@@ -3002,7 +2999,7 @@
         <v>82</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7874999999999996</v>
       </c>
       <c r="D28" s="1">
@@ -3035,7 +3032,7 @@
         <v>73</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7250000000000005</v>
       </c>
       <c r="D29" s="1">
@@ -3070,7 +3067,7 @@
         <v>142</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.6624999999999996</v>
       </c>
       <c r="D30" s="1">
@@ -3103,7 +3100,7 @@
         <v>192</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3136,7 +3133,7 @@
         <v>47</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.6000000000000005</v>
       </c>
       <c r="D32" s="1">
@@ -3169,7 +3166,7 @@
         <v>198</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5625</v>
       </c>
       <c r="D33" s="1">
@@ -3202,7 +3199,7 @@
         <v>15</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D34" s="1">
@@ -3238,7 +3235,7 @@
         <v>210</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3271,7 +3268,7 @@
         <v>105</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5249999999999995</v>
       </c>
       <c r="D36" s="1">
@@ -3306,7 +3303,7 @@
         <v>141</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3339,7 +3336,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.4874999999999989</v>
       </c>
       <c r="D38" s="1">
@@ -3371,7 +3368,7 @@
         <v>50</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.35</v>
       </c>
       <c r="D39" s="1">
@@ -3403,7 +3400,7 @@
         <v>185</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D40" s="1">
@@ -3436,7 +3433,7 @@
         <v>80</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.2500000000000009</v>
       </c>
       <c r="D41" s="1">
@@ -3469,7 +3466,7 @@
         <v>115</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.25</v>
       </c>
       <c r="D42" s="1">
@@ -3502,7 +3499,7 @@
         <v>29</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.2</v>
       </c>
       <c r="D43" s="1">
@@ -3537,7 +3534,7 @@
         <v>22</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.2</v>
       </c>
       <c r="D44" s="1">
@@ -3569,7 +3566,7 @@
         <v>140</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.1875000000000009</v>
       </c>
       <c r="D45" s="1">
@@ -3602,7 +3599,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.1875</v>
       </c>
       <c r="D46" s="1">
@@ -3635,7 +3632,7 @@
         <v>27</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.1749999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -3669,7 +3666,7 @@
         <v>49</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.1749999999999998</v>
       </c>
       <c r="D48" s="1">
@@ -3702,7 +3699,7 @@
         <v>227</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D49" s="1">
@@ -3735,7 +3732,7 @@
         <v>231</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D50" s="1">
@@ -3766,7 +3763,7 @@
         <v>71</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>6.9750000000000005</v>
       </c>
       <c r="D51" s="1">
@@ -3801,7 +3798,7 @@
         <v>76</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>6.9</v>
       </c>
       <c r="D52" s="1">
@@ -3834,7 +3831,7 @@
         <v>44</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>6.8750000000000009</v>
       </c>
       <c r="D53" s="1">
@@ -3866,7 +3863,7 @@
         <v>48</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>6.8</v>
       </c>
       <c r="D54" s="1">
@@ -3898,7 +3895,7 @@
         <v>148</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>6.7750000000000004</v>
       </c>
       <c r="D55" s="1">
@@ -3931,7 +3928,7 @@
         <v>153</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>6.75</v>
       </c>
       <c r="D56" s="1">
@@ -3964,7 +3961,7 @@
         <v>17</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>6.7250000000000005</v>
       </c>
       <c r="D57" s="1">
@@ -3996,7 +3993,7 @@
         <v>18</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>6.7</v>
       </c>
       <c r="D58" s="1">
@@ -4028,7 +4025,7 @@
         <v>9</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>6.55</v>
       </c>
       <c r="D59" s="1">
@@ -4061,7 +4058,7 @@
         <v>106</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>6.4875000000000007</v>
       </c>
       <c r="D60" s="1">
@@ -4096,7 +4093,7 @@
         <v>30</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>6.4</v>
       </c>
       <c r="D61" s="1">
@@ -4129,7 +4126,7 @@
         <v>13</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D62" s="1">
@@ -4162,7 +4159,7 @@
         <v>32</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>6.2250000000000005</v>
       </c>
       <c r="D63" s="1">
@@ -4197,7 +4194,7 @@
         <v>42</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>6.1750000000000007</v>
       </c>
       <c r="D64" s="1">
@@ -4230,7 +4227,7 @@
         <v>11</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>6.1624999999999996</v>
       </c>
       <c r="D65" s="1">
@@ -4263,7 +4260,7 @@
         <v>89</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>5.9749999999999996</v>
       </c>
       <c r="D66" s="1">
@@ -4296,7 +4293,7 @@
         <v>99</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>5.7750000000000004</v>
       </c>
       <c r="D67" s="1">
@@ -4329,7 +4326,7 @@
         <v>180</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>5.7625000000000002</v>
       </c>
       <c r="D68" s="1">
@@ -4362,7 +4359,7 @@
         <v>91</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>5.4625000000000004</v>
       </c>
       <c r="D69" s="1">
@@ -4394,7 +4391,7 @@
         <v>36</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D70" s="1">
@@ -4429,7 +4426,7 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="53" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="47" orientation="landscape" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>
@@ -4443,7 +4440,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K150"/>
+  <dimension ref="B2:K151"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4481,7 +4478,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4511,7 +4508,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4539,7 +4536,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -5514,7 +5511,7 @@
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C41" s="5">
@@ -7539,7 +7536,7 @@
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B116" s="9" t="s">
+      <c r="B116" s="2" t="s">
         <v>229</v>
       </c>
       <c r="C116" s="5">
@@ -7620,7 +7617,7 @@
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B119" s="9" t="s">
+      <c r="B119" s="2" t="s">
         <v>228</v>
       </c>
       <c r="C119" s="5">
@@ -7728,153 +7725,153 @@
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B123" s="2" t="s">
-        <v>74</v>
+      <c r="B123" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.1875</v>
+        <v>5.2</v>
       </c>
       <c r="D123" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E123" s="1">
+        <v>4</v>
+      </c>
+      <c r="F123" s="1">
+        <v>2</v>
+      </c>
+      <c r="G123" s="1">
         <v>5</v>
       </c>
-      <c r="F123" s="1">
-        <v>6</v>
-      </c>
-      <c r="G123" s="1">
-        <v>6</v>
-      </c>
       <c r="H123" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I123" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D124" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E124" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G124" s="1">
         <v>6</v>
       </c>
       <c r="H124" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I124" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E125" s="1">
         <v>4</v>
       </c>
       <c r="F125" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H125" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I125" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D126" s="1">
         <v>5</v>
       </c>
       <c r="E126" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F126" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G126" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H126" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I126" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D127" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E127" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F127" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G127" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H127" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I127" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D128" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E128" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F128" s="1">
         <v>5</v>
@@ -7883,397 +7880,397 @@
         <v>6</v>
       </c>
       <c r="H128" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I128" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D129" s="1">
+        <v>6</v>
+      </c>
+      <c r="E129" s="1">
+        <v>3</v>
+      </c>
+      <c r="F129" s="1">
         <v>5</v>
       </c>
-      <c r="E129" s="1">
-        <v>5</v>
-      </c>
-      <c r="F129" s="1">
-        <v>3</v>
-      </c>
       <c r="G129" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H129" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I129" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D130" s="1">
         <v>5</v>
       </c>
       <c r="E130" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F130" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G130" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H130" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I130" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I130" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D131" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E131" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F131" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H131" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I131" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D132" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E132" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F132" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G132" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H132" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I132" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D133" s="1">
         <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F133" s="1">
         <v>5</v>
       </c>
       <c r="G133" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H133" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I133" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D134" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E134" s="1">
         <v>4</v>
       </c>
       <c r="F134" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G134" s="1">
         <v>5</v>
       </c>
       <c r="H134" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I134" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D135" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E135" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F135" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G135" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H135" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I135" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D136" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E136" s="1">
+        <v>0</v>
+      </c>
+      <c r="F136" s="1">
         <v>2</v>
       </c>
-      <c r="F136" s="1">
-        <v>4</v>
-      </c>
       <c r="G136" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H136" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I136" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D137" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E137" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F137" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G137" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H137" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I137" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D138" s="1">
+        <v>5</v>
+      </c>
+      <c r="E138" s="1">
         <v>3</v>
       </c>
-      <c r="E138" s="1">
-        <v>4</v>
-      </c>
       <c r="F138" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G138" s="1">
         <v>4</v>
       </c>
       <c r="H138" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I138" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D139" s="1">
+        <v>3</v>
+      </c>
+      <c r="E139" s="1">
         <v>4</v>
       </c>
-      <c r="E139" s="1">
-        <v>3</v>
-      </c>
       <c r="F139" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G139" s="1">
         <v>4</v>
       </c>
       <c r="H139" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I139" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D140" s="1">
         <v>4</v>
       </c>
       <c r="E140" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F140" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G140" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H140" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I140" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D141" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E141" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F141" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G141" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H141" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I141" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D142" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E142" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F142" s="1">
         <v>2</v>
       </c>
       <c r="G142" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H142" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I142" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D143" s="1">
         <v>3</v>
@@ -8282,25 +8279,25 @@
         <v>3</v>
       </c>
       <c r="F143" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G143" s="1">
         <v>4</v>
       </c>
       <c r="H143" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I143" s="3">
         <v>4.8</v>
       </c>
-      <c r="I143" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B144" s="2">
-        <v>180</v>
+      <c r="B144" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D144" s="1">
         <v>3</v>
@@ -8312,145 +8309,145 @@
         <v>3</v>
       </c>
       <c r="G144" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H144" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I144" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B145" s="2" t="s">
-        <v>216</v>
+      <c r="B145" s="2">
+        <v>180</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D145" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E145" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F145" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G145" s="1">
         <v>3</v>
       </c>
       <c r="H145" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I145" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D146" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E146" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F146" s="1">
         <v>2</v>
       </c>
       <c r="G146" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H146" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I146" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D147" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E147" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" s="1">
         <v>2</v>
       </c>
       <c r="G147" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H147" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I147" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D148" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E148" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F148" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G148" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H148" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I148" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D149" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E149" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F149" s="1">
         <v>0</v>
       </c>
       <c r="G149" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H149" s="3">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="I149" s="3">
         <v>5.9</v>
@@ -8458,28 +8455,55 @@
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D150" s="1">
+        <v>0</v>
+      </c>
+      <c r="E150" s="1">
+        <v>0</v>
+      </c>
+      <c r="F150" s="1">
+        <v>0</v>
+      </c>
+      <c r="G150" s="1">
+        <v>0</v>
+      </c>
+      <c r="H150" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I150" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="151" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B151" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C151" s="5">
+        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D151" s="1">
         <v>2</v>
       </c>
-      <c r="E150" s="1">
+      <c r="E151" s="1">
         <v>1</v>
       </c>
-      <c r="F150" s="1">
+      <c r="F151" s="1">
         <v>2</v>
       </c>
-      <c r="G150" s="1">
+      <c r="G151" s="1">
         <v>2</v>
       </c>
-      <c r="H150" s="3">
+      <c r="H151" s="3">
         <v>4.3</v>
       </c>
-      <c r="I150" s="3">
+      <c r="I151" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 130 "Las damas primero"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E408BF-7326-4328-BDE0-CF3B2DBD99E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558F1314-1B16-449D-A73C-CE804AA33B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="234">
   <si>
     <t>Película</t>
   </si>
@@ -1293,6 +1293,9 @@
   </si>
   <si>
     <t>Juego de armas</t>
+  </si>
+  <si>
+    <t>Las damas primero</t>
   </si>
 </sst>
 </file>
@@ -1645,10 +1648,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I151" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I151" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I151">
-    <sortCondition descending="1" ref="C2:C151"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I152" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I152" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I152">
+    <sortCondition descending="1" ref="C2:C152"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4293,7 +4296,7 @@
         <v>99</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C70" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>5.7750000000000004</v>
       </c>
       <c r="D67" s="1">
@@ -4440,7 +4443,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K151"/>
+  <dimension ref="B2:K152"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -7725,7 +7728,7 @@
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B123" s="9" t="s">
+      <c r="B123" s="2" t="s">
         <v>232</v>
       </c>
       <c r="C123" s="5">
@@ -8238,66 +8241,66 @@
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B142" s="2" t="s">
-        <v>68</v>
+      <c r="B142" s="9" t="s">
+        <v>233</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D142" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E142" s="1">
+        <v>3</v>
+      </c>
+      <c r="F142" s="1">
+        <v>3</v>
+      </c>
+      <c r="G142" s="1">
         <v>4</v>
       </c>
-      <c r="F142" s="1">
-        <v>2</v>
-      </c>
-      <c r="G142" s="1">
-        <v>5</v>
-      </c>
       <c r="H142" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I142" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D143" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E143" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F143" s="1">
         <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H143" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I143" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D144" s="1">
         <v>3</v>
@@ -8306,25 +8309,25 @@
         <v>3</v>
       </c>
       <c r="F144" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G144" s="1">
         <v>4</v>
       </c>
       <c r="H144" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I144" s="3">
         <v>4.8</v>
       </c>
-      <c r="I144" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B145" s="2">
-        <v>180</v>
+      <c r="B145" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D145" s="1">
         <v>3</v>
@@ -8336,145 +8339,145 @@
         <v>3</v>
       </c>
       <c r="G145" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H145" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I145" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B146" s="2" t="s">
-        <v>216</v>
+      <c r="B146" s="2">
+        <v>180</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D146" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E146" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F146" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G146" s="1">
         <v>3</v>
       </c>
       <c r="H146" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I146" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E147" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F147" s="1">
         <v>2</v>
       </c>
       <c r="G147" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H147" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I147" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D148" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E148" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F148" s="1">
         <v>2</v>
       </c>
       <c r="G148" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H148" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I148" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D149" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E149" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F149" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G149" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H149" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I149" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D150" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E150" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F150" s="1">
         <v>0</v>
       </c>
       <c r="G150" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H150" s="3">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="I150" s="3">
         <v>5.9</v>
@@ -8482,28 +8485,55 @@
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D151" s="1">
+        <v>0</v>
+      </c>
+      <c r="E151" s="1">
+        <v>0</v>
+      </c>
+      <c r="F151" s="1">
+        <v>0</v>
+      </c>
+      <c r="G151" s="1">
+        <v>0</v>
+      </c>
+      <c r="H151" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I151" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="152" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B152" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C152" s="5">
+        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D152" s="1">
         <v>2</v>
       </c>
-      <c r="E151" s="1">
+      <c r="E152" s="1">
         <v>1</v>
       </c>
-      <c r="F151" s="1">
+      <c r="F152" s="1">
         <v>2</v>
       </c>
-      <c r="G151" s="1">
+      <c r="G152" s="1">
         <v>2</v>
       </c>
-      <c r="H151" s="3">
+      <c r="H152" s="3">
         <v>4.3</v>
       </c>
-      <c r="I151" s="3">
+      <c r="I152" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 131 "El fuego de la venganza"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558F1314-1B16-449D-A73C-CE804AA33B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D087A1A-F106-4260-A173-BE490E30CD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -78,6 +78,7 @@
     <author>tc={3E762906-7E78-4A82-82BD-91226BEEE65F}</author>
     <author>tc={A836A830-A167-47D8-ADFF-FC6A88D1B4AF}</author>
     <author>tc={153818FB-95E4-42BD-AB45-ADAC7CCB6F82}</author>
+    <author>tc={25130372-4D49-4F87-AE9D-9CE5F4E681C1}</author>
     <author>tc={83190950-04EC-4A0B-AFCD-A5040D1110EE}</author>
     <author>tc={05CBDE97-3245-4537-8EC3-A451CBCFADDC}</author>
     <author>tc={3D8C30B1-4F7A-4A97-801E-73E85EF747E6}</author>
@@ -407,7 +408,15 @@
     14 temporadas</t>
       </text>
     </comment>
-    <comment ref="B49" authorId="39" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+    <comment ref="B49" authorId="39" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    1 temporada</t>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -415,7 +424,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -423,7 +432,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -431,7 +440,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -439,7 +448,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B55" authorId="43" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+    <comment ref="B56" authorId="44" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -447,7 +456,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B56" authorId="44" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -455,7 +464,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -463,7 +472,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -471,7 +480,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -479,7 +488,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B65" authorId="48" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+    <comment ref="B66" authorId="49" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -487,7 +496,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B66" authorId="49" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -495,7 +504,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -503,7 +512,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -511,7 +520,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -519,7 +528,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -594,7 +603,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="235">
   <si>
     <t>Película</t>
   </si>
@@ -1296,6 +1305,9 @@
   </si>
   <si>
     <t>Las damas primero</t>
+  </si>
+  <si>
+    <t>El fuego de la venganza</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1317,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1341,6 +1353,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1384,7 +1402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1407,9 +1425,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1622,10 +1637,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M70" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M70" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M70">
-    <sortCondition descending="1" ref="C2:C70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M71" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M71" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M71">
+    <sortCondition descending="1" ref="C2:C71"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -2049,49 +2064,52 @@
   <threadedComment ref="B47" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
     <text>14 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B49" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+  <threadedComment ref="B49" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+    <text>1 temporada</text>
+  </threadedComment>
+  <threadedComment ref="B50" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B50" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+  <threadedComment ref="B51" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B51" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+  <threadedComment ref="B52" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B52" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+  <threadedComment ref="B53" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B55" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+  <threadedComment ref="B56" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B56" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+  <threadedComment ref="B57" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B57" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+  <threadedComment ref="B58" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B58" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+  <threadedComment ref="B59" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B59" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+  <threadedComment ref="B60" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B65" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+  <threadedComment ref="B66" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B66" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B67" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B67" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B68" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B68" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B69" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B69" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B70" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B70" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B71" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2103,7 +2121,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O70"/>
+  <dimension ref="B2:O71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -2165,7 +2183,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2199,7 +2217,7 @@
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2232,7 +2250,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2268,7 +2286,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2304,7 +2322,7 @@
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2338,7 +2356,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2371,7 +2389,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2404,7 +2422,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2437,7 +2455,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2470,7 +2488,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2505,7 +2523,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2540,7 +2558,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2573,7 +2591,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2606,7 +2624,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2641,7 +2659,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2674,7 +2692,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2707,7 +2725,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2740,7 +2758,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2771,7 +2789,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2804,7 +2822,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2837,7 +2855,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2870,7 +2888,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2903,7 +2921,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
         <v>7.8750000000000009</v>
       </c>
       <c r="D25" s="1">
@@ -2936,7 +2954,7 @@
         <v>43</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
         <v>7.8125000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -2969,7 +2987,7 @@
         <v>138</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
         <v>7.8125</v>
       </c>
       <c r="D27" s="1">
@@ -3002,7 +3020,7 @@
         <v>82</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
         <v>7.7874999999999996</v>
       </c>
       <c r="D28" s="1">
@@ -3035,7 +3053,7 @@
         <v>73</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
         <v>7.7250000000000005</v>
       </c>
       <c r="D29" s="1">
@@ -3070,7 +3088,7 @@
         <v>142</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D30" s="1">
@@ -3103,7 +3121,7 @@
         <v>192</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3136,7 +3154,7 @@
         <v>47</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
         <v>7.6000000000000005</v>
       </c>
       <c r="D32" s="1">
@@ -3169,7 +3187,7 @@
         <v>198</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
         <v>7.5625</v>
       </c>
       <c r="D33" s="1">
@@ -3202,7 +3220,7 @@
         <v>15</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D34" s="1">
@@ -3238,7 +3256,7 @@
         <v>210</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3271,7 +3289,7 @@
         <v>105</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D36" s="1">
@@ -3306,7 +3324,7 @@
         <v>141</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3339,7 +3357,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
         <v>7.4874999999999989</v>
       </c>
       <c r="D38" s="1">
@@ -3371,7 +3389,7 @@
         <v>50</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
         <v>7.35</v>
       </c>
       <c r="D39" s="1">
@@ -3403,7 +3421,7 @@
         <v>185</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
         <v>7.3</v>
       </c>
       <c r="D40" s="1">
@@ -3436,7 +3454,7 @@
         <v>80</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
         <v>7.2500000000000009</v>
       </c>
       <c r="D41" s="1">
@@ -3469,7 +3487,7 @@
         <v>115</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
         <v>7.25</v>
       </c>
       <c r="D42" s="1">
@@ -3502,7 +3520,7 @@
         <v>29</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
         <v>7.2</v>
       </c>
       <c r="D43" s="1">
@@ -3537,7 +3555,7 @@
         <v>22</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
         <v>7.2</v>
       </c>
       <c r="D44" s="1">
@@ -3569,7 +3587,7 @@
         <v>140</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
         <v>7.1875000000000009</v>
       </c>
       <c r="D45" s="1">
@@ -3602,7 +3620,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
         <v>7.1875</v>
       </c>
       <c r="D46" s="1">
@@ -3635,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -3669,7 +3687,7 @@
         <v>49</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D48" s="1">
@@ -3699,29 +3717,29 @@
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
-        <v>7.0875000000000004</v>
+        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
+        <v>7.1000000000000005</v>
       </c>
       <c r="D49" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E49" s="1">
         <v>8</v>
       </c>
       <c r="F49" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G49" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H49" s="3">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="I49" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="J49" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3732,14 +3750,14 @@
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D50" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1">
         <v>8</v>
@@ -3748,144 +3766,145 @@
         <v>7</v>
       </c>
       <c r="G50" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H50" s="3">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="I50" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="J50" s="1"/>
+        <v>6.3</v>
+      </c>
+      <c r="J50" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>71</v>
+        <v>231</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9750000000000005</v>
+        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D51" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E51" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F51" s="1">
         <v>7</v>
       </c>
       <c r="G51" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H51" s="3">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="I51" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J51" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K51" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+        <v>5.5</v>
+      </c>
+      <c r="J51" s="1"/>
+      <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9</v>
+        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <v>6.9750000000000005</v>
       </c>
       <c r="D52" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E52" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F52" s="1">
         <v>7</v>
       </c>
       <c r="G52" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H52" s="3">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="I52" s="3">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="J52" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K52" s="1"/>
+      <c r="K52" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8750000000000009</v>
+        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <v>6.9</v>
       </c>
       <c r="D53" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E53" s="1">
         <v>6</v>
       </c>
       <c r="F53" s="1">
+        <v>7</v>
+      </c>
+      <c r="G53" s="1">
         <v>5</v>
       </c>
-      <c r="G53" s="1">
-        <v>7</v>
-      </c>
       <c r="H53" s="3">
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
       <c r="I53" s="3">
-        <v>8.6</v>
-      </c>
-      <c r="J53" s="1"/>
+        <v>7.2</v>
+      </c>
+      <c r="J53" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K53" s="1"/>
-      <c r="L53" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8</v>
+        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <v>6.8750000000000009</v>
       </c>
       <c r="D54" s="1">
         <v>6</v>
       </c>
       <c r="E54" s="1">
+        <v>6</v>
+      </c>
+      <c r="F54" s="1">
         <v>5</v>
       </c>
-      <c r="F54" s="1">
-        <v>6</v>
-      </c>
       <c r="G54" s="1">
         <v>7</v>
       </c>
       <c r="H54" s="3">
-        <v>8.5</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="I54" s="3">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
@@ -3895,17 +3914,17 @@
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7750000000000004</v>
+        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <v>6.8</v>
       </c>
       <c r="D55" s="1">
         <v>6</v>
       </c>
       <c r="E55" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F55" s="1">
         <v>6</v>
@@ -3914,43 +3933,42 @@
         <v>7</v>
       </c>
       <c r="H55" s="3">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="I55" s="3">
-        <v>6.8</v>
-      </c>
-      <c r="J55" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K55" s="1"/>
-      <c r="L55" s="1"/>
-      <c r="M55" s="1"/>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
-        <v>6.75</v>
+        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <v>6.7750000000000004</v>
       </c>
       <c r="D56" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E56" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F56" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G56" s="1">
         <v>7</v>
       </c>
       <c r="H56" s="3">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I56" s="3">
-        <v>4.2</v>
+        <v>6.8</v>
       </c>
       <c r="J56" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3961,61 +3979,62 @@
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7250000000000005</v>
+        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <v>6.75</v>
       </c>
       <c r="D57" s="1">
         <v>8</v>
       </c>
       <c r="E57" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F57" s="1">
         <v>7</v>
       </c>
       <c r="G57" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H57" s="3">
-        <v>7.7</v>
+        <v>5.9</v>
       </c>
       <c r="I57" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J57" s="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="J57" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K57" s="1"/>
-      <c r="L57" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7</v>
+        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <v>6.7250000000000005</v>
       </c>
       <c r="D58" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E58" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F58" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G58" s="1">
         <v>6</v>
       </c>
       <c r="H58" s="3">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
       <c r="I58" s="3">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
@@ -4025,79 +4044,76 @@
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
-        <v>6.55</v>
+        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <v>6.7</v>
       </c>
       <c r="D59" s="1">
         <v>5</v>
       </c>
       <c r="E59" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F59" s="1">
         <v>6</v>
       </c>
       <c r="G59" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H59" s="3">
-        <v>7</v>
+        <v>8.6</v>
       </c>
       <c r="I59" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J59" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="L59" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K59" s="1"/>
-      <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4875000000000007</v>
+        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <v>6.55</v>
       </c>
       <c r="D60" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E60" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F60" s="1">
         <v>6</v>
       </c>
       <c r="G60" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H60" s="3">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="I60" s="3">
-        <v>7.7</v>
-      </c>
-      <c r="J60" s="1"/>
-      <c r="K60" t="e" vm="2">
+        <v>5.4</v>
+      </c>
+      <c r="J60" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K60" s="1"/>
       <c r="L60" s="1"/>
-      <c r="M60" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="M60" s="1"/>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4</v>
+        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <v>6.4875000000000007</v>
       </c>
       <c r="D61" s="1">
         <v>6</v>
@@ -4109,46 +4125,48 @@
         <v>6</v>
       </c>
       <c r="G61" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H61" s="3">
         <v>8.1</v>
       </c>
       <c r="I61" s="3">
-        <v>6</v>
-      </c>
-      <c r="J61" t="e" vm="1">
+        <v>7.7</v>
+      </c>
+      <c r="J61" s="1"/>
+      <c r="K61" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K61" s="1"/>
       <c r="L61" s="1"/>
-      <c r="M61" s="1"/>
+      <c r="M61" s="1" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <v>6.4</v>
       </c>
       <c r="D62" s="1">
         <v>6</v>
       </c>
       <c r="E62" s="1">
+        <v>6</v>
+      </c>
+      <c r="F62" s="1">
+        <v>6</v>
+      </c>
+      <c r="G62" s="1">
         <v>5</v>
       </c>
-      <c r="F62" s="1">
-        <v>6</v>
-      </c>
-      <c r="G62" s="1">
-        <v>6</v>
-      </c>
       <c r="H62" s="3">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="I62" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="J62" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4159,66 +4177,66 @@
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
-        <v>6.2250000000000005</v>
+        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D63" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E63" s="1">
         <v>5</v>
       </c>
       <c r="F63" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G63" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H63" s="3">
-        <v>8.1999999999999993</v>
+        <v>7.8</v>
       </c>
       <c r="I63" s="3">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="J63" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K63" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K63" s="1"/>
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1750000000000007</v>
+        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D64" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E64" s="1">
         <v>5</v>
       </c>
       <c r="F64" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G64" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H64" s="3">
-        <v>6.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I64" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="J64" s="1"/>
+        <v>6.4</v>
+      </c>
+      <c r="J64" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K64" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -4227,62 +4245,62 @@
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1624999999999996</v>
+        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <v>6.1750000000000007</v>
       </c>
       <c r="D65" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E65" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F65" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G65" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H65" s="3">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="I65" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="J65" t="e" vm="1">
+        <v>6.2</v>
+      </c>
+      <c r="J65" s="1"/>
+      <c r="K65" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K65" s="1"/>
       <c r="L65" s="1"/>
       <c r="M65" s="1"/>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
-        <v>5.9749999999999996</v>
+        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D66" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E66" s="1">
         <v>7</v>
       </c>
       <c r="F66" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G66" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H66" s="3">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I66" s="3">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J66" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4293,29 +4311,29 @@
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C70" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
-        <v>5.7750000000000004</v>
+        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D67" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E67" s="1">
         <v>7</v>
       </c>
       <c r="F67" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G67" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H67" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I67" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J67" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4326,29 +4344,29 @@
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C68" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7625000000000002</v>
+        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D68" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E68" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" s="1">
+        <v>7</v>
+      </c>
+      <c r="G68" s="1">
+        <v>3</v>
+      </c>
+      <c r="H68" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I68" s="3">
         <v>5</v>
-      </c>
-      <c r="G68" s="1">
-        <v>5</v>
-      </c>
-      <c r="H68" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I68" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J68" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4359,68 +4377,101 @@
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C69" s="5">
-        <f t="shared" si="2"/>
-        <v>5.4625000000000004</v>
+        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D69" s="1">
+        <v>8</v>
+      </c>
+      <c r="E69" s="1">
+        <v>8</v>
+      </c>
+      <c r="F69" s="1">
         <v>5</v>
       </c>
-      <c r="E69" s="1">
-        <v>7</v>
-      </c>
-      <c r="F69" s="1">
-        <v>6</v>
-      </c>
       <c r="G69" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H69" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I69" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I69" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J69" s="1"/>
+      <c r="J69" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K69" s="1"/>
-      <c r="L69" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L69" s="1"/>
+      <c r="M69" s="1"/>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C70" s="5">
+        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D70" s="1">
+        <v>5</v>
+      </c>
+      <c r="E70" s="1">
+        <v>7</v>
+      </c>
+      <c r="F70" s="1">
+        <v>6</v>
+      </c>
+      <c r="G70" s="1">
+        <v>7</v>
+      </c>
+      <c r="H70" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I70" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="L70" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B71" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C70" s="5">
-        <f t="shared" si="2"/>
+      <c r="C71" s="5">
+        <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D71" s="1">
         <v>2</v>
       </c>
-      <c r="E70" s="1">
+      <c r="E71" s="1">
         <v>4</v>
       </c>
-      <c r="F70" s="1">
+      <c r="F71" s="1">
         <v>2</v>
       </c>
-      <c r="G70" s="1">
+      <c r="G71" s="1">
         <v>5</v>
       </c>
-      <c r="H70" s="3">
+      <c r="H71" s="3">
         <v>7.7</v>
       </c>
-      <c r="I70" s="3">
+      <c r="I71" s="3">
         <v>6.3</v>
       </c>
-      <c r="J70" t="e" vm="1">
+      <c r="J71" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K70" s="1"/>
-      <c r="L70" s="1"/>
-      <c r="M70" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4490,7 +4541,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4518,7 +4569,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4546,7 +4597,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4573,7 +4624,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4600,7 +4651,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4627,7 +4678,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4654,7 +4705,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4681,7 +4732,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4708,7 +4759,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4735,7 +4786,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -4762,7 +4813,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -4789,7 +4840,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -4816,7 +4867,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -4843,7 +4894,7 @@
         <v>125</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.1750000000000007</v>
       </c>
       <c r="D16" s="1">
@@ -4870,7 +4921,7 @@
         <v>81</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.1624999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -4897,7 +4948,7 @@
         <v>77</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.15</v>
       </c>
       <c r="D18" s="1">
@@ -4924,7 +4975,7 @@
         <v>54</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D19" s="1">
@@ -4951,7 +5002,7 @@
         <v>126</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.0750000000000011</v>
       </c>
       <c r="D20" s="1">
@@ -4978,7 +5029,7 @@
         <v>58</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8.0625</v>
       </c>
       <c r="D21" s="1">
@@ -5005,7 +5056,7 @@
         <v>23</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>7.9249999999999998</v>
       </c>
       <c r="D22" s="1">
@@ -5032,7 +5083,7 @@
         <v>122</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>7.9124999999999996</v>
       </c>
       <c r="D23" s="1">
@@ -5059,7 +5110,7 @@
         <v>108</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>7.8999999999999995</v>
       </c>
       <c r="D24" s="1">
@@ -5086,7 +5137,7 @@
         <v>78</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.875</v>
       </c>
       <c r="D25" s="1">
@@ -5113,7 +5164,7 @@
         <v>109</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D26" s="1">
@@ -5140,7 +5191,7 @@
         <v>61</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5167,7 +5218,7 @@
         <v>193</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7750000000000004</v>
       </c>
       <c r="D28" s="1">
@@ -5194,7 +5245,7 @@
         <v>60</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7375000000000007</v>
       </c>
       <c r="D29" s="1">
@@ -5221,7 +5272,7 @@
         <v>38</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7000000000000011</v>
       </c>
       <c r="D30" s="1">
@@ -5248,7 +5299,7 @@
         <v>63</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999993</v>
       </c>
       <c r="D31" s="1">
@@ -5275,7 +5326,7 @@
         <v>123</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.5874999999999995</v>
       </c>
       <c r="D32" s="1">
@@ -5302,7 +5353,7 @@
         <v>37</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000011</v>
       </c>
       <c r="D33" s="1">
@@ -5329,7 +5380,7 @@
         <v>67</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000002</v>
       </c>
       <c r="D34" s="1">
@@ -5356,7 +5407,7 @@
         <v>62</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5625</v>
       </c>
       <c r="D35" s="1">
@@ -5383,7 +5434,7 @@
         <v>217</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5410,7 +5461,7 @@
         <v>55</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5624999999999991</v>
       </c>
       <c r="D37" s="1">
@@ -5437,7 +5488,7 @@
         <v>201</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.55</v>
       </c>
       <c r="D38" s="1">
@@ -5464,7 +5515,7 @@
         <v>69</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D39" s="1">
@@ -5491,7 +5542,7 @@
         <v>132</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.5125000000000002</v>
       </c>
       <c r="D40" s="1">
@@ -5518,7 +5569,7 @@
         <v>230</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.5124999999999993</v>
       </c>
       <c r="D41" s="1">
@@ -5545,7 +5596,7 @@
         <v>205</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.4875000000000007</v>
       </c>
       <c r="D42" s="1">
@@ -5572,7 +5623,7 @@
         <v>172</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.4749999999999996</v>
       </c>
       <c r="D43" s="1">
@@ -5599,7 +5650,7 @@
         <v>130</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D44" s="1">
@@ -5626,7 +5677,7 @@
         <v>97</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.4375</v>
       </c>
       <c r="D45" s="1">
@@ -5653,7 +5704,7 @@
         <v>100</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.4249999999999998</v>
       </c>
       <c r="D46" s="1">
@@ -5680,7 +5731,7 @@
         <v>131</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.4124999999999996</v>
       </c>
       <c r="D47" s="1">
@@ -5707,7 +5758,7 @@
         <v>220</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999998</v>
       </c>
       <c r="D48" s="1">
@@ -5734,7 +5785,7 @@
         <v>175</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999989</v>
       </c>
       <c r="D49" s="1">
@@ -5761,7 +5812,7 @@
         <v>52</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.3500000000000005</v>
       </c>
       <c r="D50" s="1">
@@ -5788,7 +5839,7 @@
         <v>165</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.3249999999999993</v>
       </c>
       <c r="D51" s="1">
@@ -5815,7 +5866,7 @@
         <v>224</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.3125</v>
       </c>
       <c r="D52" s="1">
@@ -5842,7 +5893,7 @@
         <v>111</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D53" s="1">
@@ -5869,7 +5920,7 @@
         <v>103</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D54" s="1">
@@ -5896,7 +5947,7 @@
         <v>181</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D55" s="1">
@@ -5923,7 +5974,7 @@
         <v>225</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>7.2624999999999993</v>
       </c>
       <c r="D56" s="1">
@@ -5950,7 +6001,7 @@
         <v>147</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>7.2374999999999998</v>
       </c>
       <c r="D57" s="1">
@@ -5977,7 +6028,7 @@
         <v>59</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>7.2250000000000005</v>
       </c>
       <c r="D58" s="1">
@@ -6004,7 +6055,7 @@
         <v>65</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>7.2125000000000004</v>
       </c>
       <c r="D59" s="1">
@@ -6031,7 +6082,7 @@
         <v>146</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>7.2124999999999995</v>
       </c>
       <c r="D60" s="1">
@@ -6058,7 +6109,7 @@
         <v>94</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
       <c r="D61" s="1">
@@ -6085,7 +6136,7 @@
         <v>53</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="D62" s="1">
@@ -6112,7 +6163,7 @@
         <v>104</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>7.1375000000000011</v>
       </c>
       <c r="D63" s="1">
@@ -6139,7 +6190,7 @@
         <v>40</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>7.1250000000000009</v>
       </c>
       <c r="D64" s="1">
@@ -6166,7 +6217,7 @@
         <v>39</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>7.125</v>
       </c>
       <c r="D65" s="1">
@@ -6193,7 +6244,7 @@
         <v>133</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D66" s="1">
@@ -6220,7 +6271,7 @@
         <v>98</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D67" s="1">
@@ -6247,7 +6298,7 @@
         <v>171</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D68" s="1">
@@ -6274,7 +6325,7 @@
         <v>110</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D69" s="1">
@@ -6301,7 +6352,7 @@
         <v>143</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D70" s="1">
@@ -6328,7 +6379,7 @@
         <v>177</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>7.0749999999999993</v>
       </c>
       <c r="D71" s="1">
@@ -6355,7 +6406,7 @@
         <v>176</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="D72" s="1">
@@ -6382,7 +6433,7 @@
         <v>221</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="D73" s="1">
@@ -6409,7 +6460,7 @@
         <v>95</v>
       </c>
       <c r="C74" s="5">
-        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
+        <f t="shared" si="2"/>
         <v>6.9375</v>
       </c>
       <c r="D74" s="1">
@@ -6436,7 +6487,7 @@
         <v>164</v>
       </c>
       <c r="C75" s="5">
-        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
+        <f t="shared" si="2"/>
         <v>6.9124999999999996</v>
       </c>
       <c r="D75" s="1">
@@ -6463,7 +6514,7 @@
         <v>157</v>
       </c>
       <c r="C76" s="5">
-        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
+        <f t="shared" si="2"/>
         <v>6.8999999999999995</v>
       </c>
       <c r="D76" s="1">
@@ -6490,7 +6541,7 @@
         <v>88</v>
       </c>
       <c r="C77" s="5">
-        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D77" s="1">
@@ -6517,7 +6568,7 @@
         <v>184</v>
       </c>
       <c r="C78" s="5">
-        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D78" s="1">
@@ -6544,7 +6595,7 @@
         <v>119</v>
       </c>
       <c r="C79" s="5">
-        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
+        <f t="shared" si="2"/>
         <v>6.85</v>
       </c>
       <c r="D79" s="1">
@@ -6571,7 +6622,7 @@
         <v>196</v>
       </c>
       <c r="C80" s="5">
-        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
+        <f t="shared" si="2"/>
         <v>6.7999999999999989</v>
       </c>
       <c r="D80" s="1">
@@ -6598,7 +6649,7 @@
         <v>57</v>
       </c>
       <c r="C81" s="5">
-        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
+        <f t="shared" si="2"/>
         <v>6.6999999999999993</v>
       </c>
       <c r="D81" s="1">
@@ -6625,7 +6676,7 @@
         <v>87</v>
       </c>
       <c r="C82" s="5">
-        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
+        <f t="shared" si="2"/>
         <v>6.6875</v>
       </c>
       <c r="D82" s="1">
@@ -6652,7 +6703,7 @@
         <v>211</v>
       </c>
       <c r="C83" s="5">
-        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
+        <f t="shared" si="2"/>
         <v>6.6375000000000002</v>
       </c>
       <c r="D83" s="1">
@@ -6679,7 +6730,7 @@
         <v>219</v>
       </c>
       <c r="C84" s="5">
-        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
+        <f t="shared" si="2"/>
         <v>6.6374999999999993</v>
       </c>
       <c r="D84" s="1">
@@ -6706,7 +6757,7 @@
         <v>41</v>
       </c>
       <c r="C85" s="5">
-        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999989</v>
       </c>
       <c r="D85" s="1">
@@ -6733,7 +6784,7 @@
         <v>117</v>
       </c>
       <c r="C86" s="5">
-        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D86" s="1">
@@ -6760,7 +6811,7 @@
         <v>179</v>
       </c>
       <c r="C87" s="5">
-        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D87" s="1">
@@ -6787,7 +6838,7 @@
         <v>215</v>
       </c>
       <c r="C88" s="5">
-        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
+        <f t="shared" si="2"/>
         <v>6.5750000000000002</v>
       </c>
       <c r="D88" s="1">
@@ -6814,7 +6865,7 @@
         <v>168</v>
       </c>
       <c r="C89" s="5">
-        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
+        <f t="shared" si="2"/>
         <v>6.5499999999999989</v>
       </c>
       <c r="D89" s="1">
@@ -6841,7 +6892,7 @@
         <v>197</v>
       </c>
       <c r="C90" s="5">
-        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
+        <f t="shared" si="2"/>
         <v>6.5375000000000005</v>
       </c>
       <c r="D90" s="1">
@@ -6868,7 +6919,7 @@
         <v>202</v>
       </c>
       <c r="C91" s="5">
-        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D91" s="1">
@@ -6895,7 +6946,7 @@
         <v>183</v>
       </c>
       <c r="C92" s="5">
-        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D92" s="1">
@@ -6922,7 +6973,7 @@
         <v>200</v>
       </c>
       <c r="C93" s="5">
-        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D93" s="1">
@@ -6949,7 +7000,7 @@
         <v>188</v>
       </c>
       <c r="C94" s="5">
-        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D94" s="1">
@@ -6976,7 +7027,7 @@
         <v>208</v>
       </c>
       <c r="C95" s="5">
-        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D95" s="1">
@@ -7003,7 +7054,7 @@
         <v>134</v>
       </c>
       <c r="C96" s="5">
-        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <f t="shared" si="2"/>
         <v>6.3125</v>
       </c>
       <c r="D96" s="1">
@@ -7030,7 +7081,7 @@
         <v>144</v>
       </c>
       <c r="C97" s="5">
-        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
+        <f t="shared" si="2"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D97" s="1">
@@ -7057,7 +7108,7 @@
         <v>64</v>
       </c>
       <c r="C98" s="5">
-        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <f t="shared" si="2"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D98" s="1">
@@ -7084,7 +7135,7 @@
         <v>75</v>
       </c>
       <c r="C99" s="5">
-        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.2125000000000004</v>
       </c>
       <c r="D99" s="1">
@@ -7111,7 +7162,7 @@
         <v>19</v>
       </c>
       <c r="C100" s="5">
-        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
+        <f t="shared" si="3"/>
         <v>6.2124999999999995</v>
       </c>
       <c r="D100" s="1">
@@ -7138,7 +7189,7 @@
         <v>101</v>
       </c>
       <c r="C101" s="5">
-        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <f t="shared" si="3"/>
         <v>6.15</v>
       </c>
       <c r="D101" s="1">
@@ -7165,7 +7216,7 @@
         <v>158</v>
       </c>
       <c r="C102" s="5">
-        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <f t="shared" si="3"/>
         <v>6.0874999999999995</v>
       </c>
       <c r="D102" s="1">
@@ -7192,7 +7243,7 @@
         <v>222</v>
       </c>
       <c r="C103" s="5">
-        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <f t="shared" si="3"/>
         <v>6.0625</v>
       </c>
       <c r="D103" s="1">
@@ -7219,7 +7270,7 @@
         <v>214</v>
       </c>
       <c r="C104" s="5">
-        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <f t="shared" si="3"/>
         <v>6.0500000000000007</v>
       </c>
       <c r="D104" s="1">
@@ -7246,7 +7297,7 @@
         <v>160</v>
       </c>
       <c r="C105" s="5">
-        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D105" s="1">
@@ -7273,7 +7324,7 @@
         <v>206</v>
       </c>
       <c r="C106" s="5">
-        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D106" s="1">
@@ -7300,7 +7351,7 @@
         <v>159</v>
       </c>
       <c r="C107" s="5">
-        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <f t="shared" si="3"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="D107" s="1">
@@ -7327,7 +7378,7 @@
         <v>195</v>
       </c>
       <c r="C108" s="5">
-        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <f t="shared" si="3"/>
         <v>5.8875000000000011</v>
       </c>
       <c r="D108" s="1">
@@ -7354,7 +7405,7 @@
         <v>186</v>
       </c>
       <c r="C109" s="5">
-        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
+        <f t="shared" si="3"/>
         <v>5.8125000000000009</v>
       </c>
       <c r="D109" s="1">
@@ -7381,7 +7432,7 @@
         <v>209</v>
       </c>
       <c r="C110" s="5">
-        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <f t="shared" si="3"/>
         <v>5.8000000000000007</v>
       </c>
       <c r="D110" s="1">
@@ -7408,7 +7459,7 @@
         <v>113</v>
       </c>
       <c r="C111" s="5">
-        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <f t="shared" si="3"/>
         <v>5.7374999999999989</v>
       </c>
       <c r="D111" s="1">
@@ -7435,7 +7486,7 @@
         <v>187</v>
       </c>
       <c r="C112" s="5">
-        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <f t="shared" si="3"/>
         <v>5.7250000000000005</v>
       </c>
       <c r="D112" s="1">
@@ -7462,7 +7513,7 @@
         <v>26</v>
       </c>
       <c r="C113" s="5">
-        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <f t="shared" si="3"/>
         <v>5.6749999999999998</v>
       </c>
       <c r="D113" s="1">
@@ -7489,7 +7540,7 @@
         <v>149</v>
       </c>
       <c r="C114" s="5">
-        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D114" s="1">
@@ -7516,7 +7567,7 @@
         <v>156</v>
       </c>
       <c r="C115" s="5">
-        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D115" s="1">
@@ -7543,7 +7594,7 @@
         <v>229</v>
       </c>
       <c r="C116" s="5">
-        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <f t="shared" si="3"/>
         <v>5.5375000000000005</v>
       </c>
       <c r="D116" s="1">
@@ -7570,7 +7621,7 @@
         <v>166</v>
       </c>
       <c r="C117" s="5">
-        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D117" s="1">
@@ -7597,7 +7648,7 @@
         <v>191</v>
       </c>
       <c r="C118" s="5">
-        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D118" s="1">
@@ -7624,7 +7675,7 @@
         <v>228</v>
       </c>
       <c r="C119" s="5">
-        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <f t="shared" si="3"/>
         <v>5.3875000000000011</v>
       </c>
       <c r="D119" s="1">
@@ -7651,7 +7702,7 @@
         <v>204</v>
       </c>
       <c r="C120" s="5">
-        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <f t="shared" si="3"/>
         <v>5.3750000000000009</v>
       </c>
       <c r="D120" s="1">
@@ -7678,7 +7729,7 @@
         <v>190</v>
       </c>
       <c r="C121" s="5">
-        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <f t="shared" si="3"/>
         <v>5.375</v>
       </c>
       <c r="D121" s="1">
@@ -7705,7 +7756,7 @@
         <v>182</v>
       </c>
       <c r="C122" s="5">
-        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
+        <f t="shared" si="3"/>
         <v>5.2875000000000005</v>
       </c>
       <c r="D122" s="1">
@@ -7732,7 +7783,7 @@
         <v>232</v>
       </c>
       <c r="C123" s="5">
-        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <f t="shared" si="3"/>
         <v>5.2</v>
       </c>
       <c r="D123" s="1">
@@ -7759,7 +7810,7 @@
         <v>74</v>
       </c>
       <c r="C124" s="5">
-        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <f t="shared" si="3"/>
         <v>5.1875</v>
       </c>
       <c r="D124" s="1">
@@ -7786,7 +7837,7 @@
         <v>145</v>
       </c>
       <c r="C125" s="5">
-        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <f t="shared" si="3"/>
         <v>5.1124999999999998</v>
       </c>
       <c r="D125" s="1">
@@ -7813,7 +7864,7 @@
         <v>223</v>
       </c>
       <c r="C126" s="5">
-        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <f t="shared" si="3"/>
         <v>5.0750000000000002</v>
       </c>
       <c r="D126" s="1">
@@ -7840,7 +7891,7 @@
         <v>21</v>
       </c>
       <c r="C127" s="5">
-        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <f t="shared" si="3"/>
         <v>5.05</v>
       </c>
       <c r="D127" s="1">
@@ -7867,7 +7918,7 @@
         <v>203</v>
       </c>
       <c r="C128" s="5">
-        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <f t="shared" si="3"/>
         <v>4.9875000000000007</v>
       </c>
       <c r="D128" s="1">
@@ -7894,7 +7945,7 @@
         <v>169</v>
       </c>
       <c r="C129" s="5">
-        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <f t="shared" si="3"/>
         <v>4.9874999999999998</v>
       </c>
       <c r="D129" s="1">
@@ -7921,7 +7972,7 @@
         <v>163</v>
       </c>
       <c r="C130" s="5">
-        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <f t="shared" si="3"/>
         <v>4.8499999999999996</v>
       </c>
       <c r="D130" s="1">
@@ -7948,7 +7999,7 @@
         <v>162</v>
       </c>
       <c r="C131" s="5">
-        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>4.7875000000000005</v>
       </c>
       <c r="D131" s="1">
@@ -7975,7 +8026,7 @@
         <v>213</v>
       </c>
       <c r="C132" s="5">
-        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <f t="shared" si="4"/>
         <v>4.6124999999999998</v>
       </c>
       <c r="D132" s="1">
@@ -8002,7 +8053,7 @@
         <v>154</v>
       </c>
       <c r="C133" s="5">
-        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <f t="shared" si="4"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="D133" s="1">
@@ -8029,7 +8080,7 @@
         <v>135</v>
       </c>
       <c r="C134" s="5">
-        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <f t="shared" si="4"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D134" s="1">
@@ -8056,7 +8107,7 @@
         <v>161</v>
       </c>
       <c r="C135" s="5">
-        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <f t="shared" si="4"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="D135" s="1">
@@ -8083,7 +8134,7 @@
         <v>114</v>
       </c>
       <c r="C136" s="5">
-        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <f t="shared" si="4"/>
         <v>4.4124999999999996</v>
       </c>
       <c r="D136" s="1">
@@ -8110,7 +8161,7 @@
         <v>207</v>
       </c>
       <c r="C137" s="5">
-        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <f t="shared" si="4"/>
         <v>4.3375000000000004</v>
       </c>
       <c r="D137" s="1">
@@ -8137,7 +8188,7 @@
         <v>150</v>
       </c>
       <c r="C138" s="5">
-        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <f t="shared" si="4"/>
         <v>4.3374999999999995</v>
       </c>
       <c r="D138" s="1">
@@ -8164,7 +8215,7 @@
         <v>173</v>
       </c>
       <c r="C139" s="5">
-        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <f t="shared" si="4"/>
         <v>4.3125</v>
       </c>
       <c r="D139" s="1">
@@ -8191,7 +8242,7 @@
         <v>212</v>
       </c>
       <c r="C140" s="5">
-        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <f t="shared" si="4"/>
         <v>4.3</v>
       </c>
       <c r="D140" s="1">
@@ -8218,7 +8269,7 @@
         <v>167</v>
       </c>
       <c r="C141" s="5">
-        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <f t="shared" si="4"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="D141" s="1">
@@ -8241,11 +8292,11 @@
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B142" s="9" t="s">
+      <c r="B142" s="2" t="s">
         <v>233</v>
       </c>
       <c r="C142" s="5">
-        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <f t="shared" si="4"/>
         <v>4.1625000000000005</v>
       </c>
       <c r="D142" s="1">
@@ -8272,7 +8323,7 @@
         <v>68</v>
       </c>
       <c r="C143" s="5">
-        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <f t="shared" si="4"/>
         <v>4.1124999999999998</v>
       </c>
       <c r="D143" s="1">
@@ -8299,7 +8350,7 @@
         <v>218</v>
       </c>
       <c r="C144" s="5">
-        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <f t="shared" si="4"/>
         <v>3.9499999999999997</v>
       </c>
       <c r="D144" s="1">
@@ -8326,7 +8377,7 @@
         <v>199</v>
       </c>
       <c r="C145" s="5">
-        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <f t="shared" si="4"/>
         <v>3.7375000000000003</v>
       </c>
       <c r="D145" s="1">
@@ -8353,7 +8404,7 @@
         <v>180</v>
       </c>
       <c r="C146" s="5">
-        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <f t="shared" si="4"/>
         <v>3.5625000000000004</v>
       </c>
       <c r="D146" s="1">
@@ -8380,7 +8431,7 @@
         <v>216</v>
       </c>
       <c r="C147" s="5">
-        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <f t="shared" si="4"/>
         <v>3.5375000000000005</v>
       </c>
       <c r="D147" s="1">
@@ -8407,7 +8458,7 @@
         <v>189</v>
       </c>
       <c r="C148" s="5">
-        <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
+        <f t="shared" si="4"/>
         <v>3.3250000000000002</v>
       </c>
       <c r="D148" s="1">
@@ -8434,7 +8485,7 @@
         <v>194</v>
       </c>
       <c r="C149" s="5">
-        <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
+        <f t="shared" si="4"/>
         <v>3.2749999999999995</v>
       </c>
       <c r="D149" s="1">
@@ -8461,7 +8512,7 @@
         <v>155</v>
       </c>
       <c r="C150" s="5">
-        <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <f t="shared" si="4"/>
         <v>2.9124999999999996</v>
       </c>
       <c r="D150" s="1">
@@ -8488,7 +8539,7 @@
         <v>174</v>
       </c>
       <c r="C151" s="5">
-        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <f t="shared" si="4"/>
         <v>2.6375000000000002</v>
       </c>
       <c r="D151" s="1">
@@ -8515,7 +8566,7 @@
         <v>226</v>
       </c>
       <c r="C152" s="5">
-        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
+        <f t="shared" si="4"/>
         <v>2.5125000000000002</v>
       </c>
       <c r="D152" s="1">

</xml_diff>

<commit_message>
V. 133 "Lo nunca visto"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89928A73-EDDE-4CC1-B83C-05D8F6209757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36806CC4-92ED-495C-999F-725F2012C591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -603,7 +603,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="237">
   <si>
     <t>Película</t>
   </si>
@@ -1311,6 +1311,9 @@
   </si>
   <si>
     <t>The Mandalorian and Grogu</t>
+  </si>
+  <si>
+    <t>Lo nunca visto</t>
   </si>
 </sst>
 </file>
@@ -1414,13 +1417,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1432,45 +1435,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1511,6 +1475,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1637,48 +1640,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M71" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M71" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M71" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M71">
     <sortCondition descending="1" ref="C2:C71"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I153" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I153" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I153">
-    <sortCondition descending="1" ref="C2:C153"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I154" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I154" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I154">
+    <sortCondition descending="1" ref="C2:C154"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2174,7 +2177,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2210,7 +2213,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2277,7 +2280,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2315,7 +2318,7 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -2349,7 +2352,7 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -4314,7 +4317,7 @@
         <v>89</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C71" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>5.9749999999999996</v>
       </c>
       <c r="D67" s="1">
@@ -4494,7 +4497,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K153"/>
+  <dimension ref="B2:K154"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4532,7 +4535,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4562,7 +4565,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4590,7 +4593,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -4890,7 +4893,7 @@
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="2" t="s">
         <v>235</v>
       </c>
       <c r="C16" s="5">
@@ -8319,93 +8322,93 @@
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B143" s="2" t="s">
-        <v>233</v>
+      <c r="B143" s="9" t="s">
+        <v>236</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D143" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E143" s="1">
         <v>3</v>
       </c>
       <c r="F143" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G143" s="1">
         <v>4</v>
       </c>
       <c r="H143" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I143" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D144" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E144" s="1">
+        <v>3</v>
+      </c>
+      <c r="F144" s="1">
+        <v>3</v>
+      </c>
+      <c r="G144" s="1">
         <v>4</v>
       </c>
-      <c r="F144" s="1">
-        <v>2</v>
-      </c>
-      <c r="G144" s="1">
-        <v>5</v>
-      </c>
       <c r="H144" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I144" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D145" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E145" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F145" s="1">
         <v>2</v>
       </c>
       <c r="G145" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H145" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I145" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D146" s="1">
         <v>3</v>
@@ -8414,25 +8417,25 @@
         <v>3</v>
       </c>
       <c r="F146" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G146" s="1">
         <v>4</v>
       </c>
       <c r="H146" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I146" s="3">
         <v>4.8</v>
       </c>
-      <c r="I146" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B147" s="2">
-        <v>180</v>
+      <c r="B147" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D147" s="1">
         <v>3</v>
@@ -8444,145 +8447,145 @@
         <v>3</v>
       </c>
       <c r="G147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H147" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I147" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B148" s="2" t="s">
-        <v>216</v>
+      <c r="B148" s="2">
+        <v>180</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D148" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E148" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F148" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G148" s="1">
         <v>3</v>
       </c>
       <c r="H148" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I148" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D149" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E149" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F149" s="1">
         <v>2</v>
       </c>
       <c r="G149" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H149" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I149" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D150" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E150" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="1">
         <v>2</v>
       </c>
       <c r="G150" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H150" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I150" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D151" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E151" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F151" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G151" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H151" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I151" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>2.6375000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D152" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F152" s="1">
         <v>0</v>
       </c>
       <c r="G152" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H152" s="3">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="I152" s="3">
         <v>5.9</v>
@@ -8590,28 +8593,55 @@
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D153" s="1">
+        <v>0</v>
+      </c>
+      <c r="E153" s="1">
+        <v>0</v>
+      </c>
+      <c r="F153" s="1">
+        <v>0</v>
+      </c>
+      <c r="G153" s="1">
+        <v>0</v>
+      </c>
+      <c r="H153" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I153" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="154" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B154" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C154" s="5">
+        <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D154" s="1">
         <v>2</v>
       </c>
-      <c r="E153" s="1">
+      <c r="E154" s="1">
         <v>1</v>
       </c>
-      <c r="F153" s="1">
+      <c r="F154" s="1">
         <v>2</v>
       </c>
-      <c r="G153" s="1">
+      <c r="G154" s="1">
         <v>2</v>
       </c>
-      <c r="H153" s="3">
+      <c r="H154" s="3">
         <v>4.3</v>
       </c>
-      <c r="I153" s="3">
+      <c r="I154" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 134 "La gente como vosotros"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36806CC4-92ED-495C-999F-725F2012C591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E1870B-836E-4E2F-865A-ED627919E178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -603,7 +603,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="238">
   <si>
     <t>Película</t>
   </si>
@@ -1314,6 +1314,9 @@
   </si>
   <si>
     <t>Lo nunca visto</t>
+  </si>
+  <si>
+    <t>La gente como vosotros</t>
   </si>
 </sst>
 </file>
@@ -1666,10 +1669,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I154" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I154" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I154">
-    <sortCondition descending="1" ref="C2:C154"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I155" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I155" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I155">
+    <sortCondition descending="1" ref="C2:C155"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4497,7 +4500,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K154"/>
+  <dimension ref="B2:K155"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -8322,7 +8325,7 @@
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B143" s="9" t="s">
+      <c r="B143" s="2" t="s">
         <v>236</v>
       </c>
       <c r="C143" s="5">
@@ -8592,56 +8595,83 @@
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B153" s="2" t="s">
-        <v>174</v>
+      <c r="B153" s="9" t="s">
+        <v>237</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>2.6375000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D153" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E153" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F153" s="1">
         <v>0</v>
       </c>
       <c r="G153" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H153" s="3">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
       <c r="I153" s="3">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D154" s="1">
+        <v>0</v>
+      </c>
+      <c r="E154" s="1">
+        <v>0</v>
+      </c>
+      <c r="F154" s="1">
+        <v>0</v>
+      </c>
+      <c r="G154" s="1">
+        <v>0</v>
+      </c>
+      <c r="H154" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I154" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="155" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B155" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C155" s="5">
+        <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D155" s="1">
         <v>2</v>
       </c>
-      <c r="E154" s="1">
+      <c r="E155" s="1">
         <v>1</v>
       </c>
-      <c r="F154" s="1">
+      <c r="F155" s="1">
         <v>2</v>
       </c>
-      <c r="G154" s="1">
+      <c r="G155" s="1">
         <v>2</v>
       </c>
-      <c r="H154" s="3">
+      <c r="H155" s="3">
         <v>4.3</v>
       </c>
-      <c r="I154" s="3">
+      <c r="I155" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 135 "El nuevo empleado"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E1870B-836E-4E2F-865A-ED627919E178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF6250D-9252-47FC-B089-EE9EA20C5DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -59,6 +59,7 @@
     <author>tc={905D74EB-1C41-4120-8733-E9C8C2FF351A}</author>
     <author>tc={B4E0A9EE-3277-494F-88A8-61F8EE265DDE}</author>
     <author>tc={97D38487-0228-4117-9D87-BCCFD4EC6983}</author>
+    <author>tc={39402C95-AD3B-446E-8FD4-EC7A8F7EBC34}</author>
     <author>tc={BE581C86-E71E-4F40-9F43-00EDE88FB108}</author>
     <author>tc={9C26C127-20FF-4258-B62D-B6B902EB0E98}</author>
     <author>tc={B1E35BAB-7C71-4B4F-9EE2-76495541B293}</author>
@@ -256,7 +257,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B25" authorId="20" shapeId="0" xr:uid="{BE581C86-E71E-4F40-9F43-00EDE88FB108}">
+    <comment ref="B25" authorId="20" shapeId="0" xr:uid="{39402C95-AD3B-446E-8FD4-EC7A8F7EBC34}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -264,7 +265,7 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B26" authorId="21" shapeId="0" xr:uid="{9C26C127-20FF-4258-B62D-B6B902EB0E98}">
+    <comment ref="B26" authorId="21" shapeId="0" xr:uid="{BE581C86-E71E-4F40-9F43-00EDE88FB108}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -272,7 +273,15 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B29" authorId="22" shapeId="0" xr:uid="{B1E35BAB-7C71-4B4F-9EE2-76495541B293}">
+    <comment ref="B27" authorId="22" shapeId="0" xr:uid="{9C26C127-20FF-4258-B62D-B6B902EB0E98}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    2 temporadas</t>
+      </text>
+    </comment>
+    <comment ref="B30" authorId="23" shapeId="0" xr:uid="{B1E35BAB-7C71-4B4F-9EE2-76495541B293}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -280,7 +289,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B30" authorId="23" shapeId="0" xr:uid="{C7D97E8C-DE70-4119-AC31-C6C9E2D35A59}">
+    <comment ref="B31" authorId="24" shapeId="0" xr:uid="{C7D97E8C-DE70-4119-AC31-C6C9E2D35A59}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -288,7 +297,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B31" authorId="24" shapeId="0" xr:uid="{B1A9CC41-51C1-4F65-B085-E2CB980F4BF9}">
+    <comment ref="B32" authorId="25" shapeId="0" xr:uid="{B1A9CC41-51C1-4F65-B085-E2CB980F4BF9}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -296,7 +305,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B32" authorId="25" shapeId="0" xr:uid="{E34E6F01-0047-4D5E-A9F0-76B7D80CE842}">
+    <comment ref="B33" authorId="26" shapeId="0" xr:uid="{E34E6F01-0047-4D5E-A9F0-76B7D80CE842}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -304,7 +313,7 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B33" authorId="26" shapeId="0" xr:uid="{66A44D43-B718-4B72-9103-F3288A2AC23B}">
+    <comment ref="B34" authorId="27" shapeId="0" xr:uid="{66A44D43-B718-4B72-9103-F3288A2AC23B}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -312,7 +321,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B34" authorId="27" shapeId="0" xr:uid="{162EA199-65BB-48FF-A9B1-580BDA0F2A25}">
+    <comment ref="B35" authorId="28" shapeId="0" xr:uid="{162EA199-65BB-48FF-A9B1-580BDA0F2A25}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -320,7 +329,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B35" authorId="28" shapeId="0" xr:uid="{A8DD2670-DAB9-48F0-9B69-06BCBECDF83A}">
+    <comment ref="B36" authorId="29" shapeId="0" xr:uid="{A8DD2670-DAB9-48F0-9B69-06BCBECDF83A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -328,7 +337,7 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B36" authorId="29" shapeId="0" xr:uid="{BC097833-5E05-4B57-A72A-B55B23EF385A}">
+    <comment ref="B37" authorId="30" shapeId="0" xr:uid="{BC097833-5E05-4B57-A72A-B55B23EF385A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -336,7 +345,7 @@
     10 temporadas</t>
       </text>
     </comment>
-    <comment ref="B37" authorId="30" shapeId="0" xr:uid="{D69ACFED-A245-418D-8836-7787A10A08B4}">
+    <comment ref="B38" authorId="31" shapeId="0" xr:uid="{D69ACFED-A245-418D-8836-7787A10A08B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -344,7 +353,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B38" authorId="31" shapeId="0" xr:uid="{FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}">
+    <comment ref="B39" authorId="32" shapeId="0" xr:uid="{FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -352,7 +361,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B40" authorId="32" shapeId="0" xr:uid="{0372C847-801C-4993-BA73-8301D595FCF1}">
+    <comment ref="B41" authorId="33" shapeId="0" xr:uid="{0372C847-801C-4993-BA73-8301D595FCF1}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -360,7 +369,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B41" authorId="33" shapeId="0" xr:uid="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
+    <comment ref="B42" authorId="34" shapeId="0" xr:uid="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -368,7 +377,7 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B42" authorId="34" shapeId="0" xr:uid="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
+    <comment ref="B43" authorId="35" shapeId="0" xr:uid="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -376,7 +385,7 @@
     6 temporadas</t>
       </text>
     </comment>
-    <comment ref="B44" authorId="35" shapeId="0" xr:uid="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
+    <comment ref="B45" authorId="36" shapeId="0" xr:uid="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -384,7 +393,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B45" authorId="36" shapeId="0" xr:uid="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
+    <comment ref="B46" authorId="37" shapeId="0" xr:uid="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -392,7 +401,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B46" authorId="37" shapeId="0" xr:uid="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
+    <comment ref="B47" authorId="38" shapeId="0" xr:uid="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -400,7 +409,7 @@
     6 temporadas</t>
       </text>
     </comment>
-    <comment ref="B47" authorId="38" shapeId="0" xr:uid="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
+    <comment ref="B48" authorId="39" shapeId="0" xr:uid="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -408,7 +417,7 @@
     14 temporadas</t>
       </text>
     </comment>
-    <comment ref="B49" authorId="39" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -416,7 +425,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -424,7 +433,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -432,7 +441,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -440,7 +449,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+    <comment ref="B54" authorId="44" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -448,7 +457,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B56" authorId="44" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -456,7 +465,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -464,7 +473,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -472,7 +481,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -480,7 +489,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+    <comment ref="B61" authorId="49" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -488,7 +497,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B66" authorId="49" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -496,7 +505,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -504,7 +513,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -512,7 +521,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -520,7 +529,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -528,7 +537,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -603,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="239">
   <si>
     <t>Película</t>
   </si>
@@ -1317,6 +1326,9 @@
   </si>
   <si>
     <t>La gente como vosotros</t>
+  </si>
+  <si>
+    <t>El nuevo empleado</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1338,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1362,6 +1374,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1405,7 +1423,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1428,9 +1446,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1643,10 +1658,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M71" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M71" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M71">
-    <sortCondition descending="1" ref="C2:C71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M72" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M72" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M72">
+    <sortCondition descending="1" ref="C2:C72"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -2013,109 +2028,112 @@
   <threadedComment ref="B24" dT="2024-07-08T19:03:23.53" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{97D38487-0228-4117-9D87-BCCFD4EC6983}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B25" dT="2024-07-08T19:02:11.85" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{BE581C86-E71E-4F40-9F43-00EDE88FB108}">
+  <threadedComment ref="B25" dT="2026-06-09T21:51:25.58" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{39402C95-AD3B-446E-8FD4-EC7A8F7EBC34}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B26" dT="2024-07-08T19:03:46.50" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{9C26C127-20FF-4258-B62D-B6B902EB0E98}">
+  <threadedComment ref="B26" dT="2024-07-08T19:02:11.85" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{BE581C86-E71E-4F40-9F43-00EDE88FB108}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B29" dT="2024-07-08T19:01:48.87" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1E35BAB-7C71-4B4F-9EE2-76495541B293}">
+  <threadedComment ref="B27" dT="2024-07-08T19:03:46.50" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{9C26C127-20FF-4258-B62D-B6B902EB0E98}">
+    <text>2 temporadas</text>
+  </threadedComment>
+  <threadedComment ref="B30" dT="2024-07-08T19:01:48.87" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1E35BAB-7C71-4B4F-9EE2-76495541B293}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B30" dT="2025-04-19T09:54:12.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C7D97E8C-DE70-4119-AC31-C6C9E2D35A59}">
+  <threadedComment ref="B31" dT="2025-04-19T09:54:12.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C7D97E8C-DE70-4119-AC31-C6C9E2D35A59}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B31" dT="2025-11-11T13:19:02.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1A9CC41-51C1-4F65-B085-E2CB980F4BF9}">
+  <threadedComment ref="B32" dT="2025-11-11T13:19:02.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1A9CC41-51C1-4F65-B085-E2CB980F4BF9}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B32" dT="2024-07-08T19:08:09.20" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{E34E6F01-0047-4D5E-A9F0-76B7D80CE842}">
+  <threadedComment ref="B33" dT="2024-07-08T19:08:09.20" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{E34E6F01-0047-4D5E-A9F0-76B7D80CE842}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B33" dT="2025-11-25T11:49:06.94" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{66A44D43-B718-4B72-9103-F3288A2AC23B}">
+  <threadedComment ref="B34" dT="2025-11-25T11:49:06.94" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{66A44D43-B718-4B72-9103-F3288A2AC23B}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B34" dT="2024-07-08T19:06:42.39" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{162EA199-65BB-48FF-A9B1-580BDA0F2A25}">
+  <threadedComment ref="B35" dT="2024-07-08T19:06:42.39" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{162EA199-65BB-48FF-A9B1-580BDA0F2A25}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B35" dT="2026-01-04T19:50:03.78" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A8DD2670-DAB9-48F0-9B69-06BCBECDF83A}">
+  <threadedComment ref="B36" dT="2026-01-04T19:50:03.78" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A8DD2670-DAB9-48F0-9B69-06BCBECDF83A}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B36" dT="2024-07-08T19:06:30.81" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{BC097833-5E05-4B57-A72A-B55B23EF385A}">
+  <threadedComment ref="B37" dT="2024-07-08T19:06:30.81" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{BC097833-5E05-4B57-A72A-B55B23EF385A}">
     <text>10 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B37" dT="2025-04-18T12:26:08.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{D69ACFED-A245-418D-8836-7787A10A08B4}">
+  <threadedComment ref="B38" dT="2025-04-18T12:26:08.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{D69ACFED-A245-418D-8836-7787A10A08B4}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B38" dT="2024-07-08T19:08:20.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}">
+  <threadedComment ref="B39" dT="2024-07-08T19:08:20.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B40" dT="2025-10-21T19:53:14.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{0372C847-801C-4993-BA73-8301D595FCF1}">
+  <threadedComment ref="B41" dT="2025-10-21T19:53:14.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{0372C847-801C-4993-BA73-8301D595FCF1}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B41" dT="2024-07-08T19:04:29.42" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
+  <threadedComment ref="B42" dT="2024-07-08T19:04:29.42" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B42" dT="2024-12-19T19:39:49.29" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
+  <threadedComment ref="B43" dT="2024-12-19T19:39:49.29" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
     <text>6 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B44" dT="2024-07-08T19:08:48.45" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
+  <threadedComment ref="B45" dT="2024-07-08T19:08:48.45" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B45" dT="2025-04-09T21:18:34.74" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
+  <threadedComment ref="B46" dT="2025-04-09T21:18:34.74" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B46" dT="2024-07-08T19:09:26.44" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
+  <threadedComment ref="B47" dT="2024-07-08T19:09:26.44" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
     <text>6 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B47" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
+  <threadedComment ref="B48" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
     <text>14 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B49" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+  <threadedComment ref="B50" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B50" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+  <threadedComment ref="B51" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B51" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+  <threadedComment ref="B52" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B52" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+  <threadedComment ref="B53" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B53" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+  <threadedComment ref="B54" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B56" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+  <threadedComment ref="B57" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B57" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+  <threadedComment ref="B58" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B58" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+  <threadedComment ref="B59" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B59" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+  <threadedComment ref="B60" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B60" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+  <threadedComment ref="B61" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B66" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+  <threadedComment ref="B67" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B67" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B68" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B68" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B69" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B69" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B70" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B70" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B71" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B71" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B72" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2127,7 +2145,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O71"/>
+  <dimension ref="B2:O72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -2189,7 +2207,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2223,7 +2241,7 @@
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2256,7 +2274,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2292,7 +2310,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2328,7 +2346,7 @@
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2362,7 +2380,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2395,7 +2413,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2428,7 +2446,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2461,7 +2479,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2494,7 +2512,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2529,7 +2547,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2564,7 +2582,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2597,7 +2615,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2630,7 +2648,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2665,7 +2683,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2698,7 +2716,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2731,7 +2749,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2764,7 +2782,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2795,7 +2813,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2828,7 +2846,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2861,7 +2879,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2894,7 +2912,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2924,14 +2942,14 @@
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
-        <v>5</v>
+        <v>238</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
-        <v>7.8750000000000009</v>
+        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
+        <v>7.8874999999999993</v>
       </c>
       <c r="D25" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E25" s="1">
         <v>8</v>
@@ -2940,13 +2958,13 @@
         <v>9</v>
       </c>
       <c r="G25" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H25" s="3">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="I25" s="3">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="J25" t="e" vm="1">
         <v>#VALUE!</v>
@@ -2957,14 +2975,14 @@
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
-        <v>7.8125000000000009</v>
+        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
+        <v>7.8750000000000009</v>
       </c>
       <c r="D26" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E26" s="1">
         <v>8</v>
@@ -2976,58 +2994,58 @@
         <v>8</v>
       </c>
       <c r="H26" s="3">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
       <c r="I26" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="J26" s="1"/>
-      <c r="K26" t="e" vm="2">
+        <v>6.6</v>
+      </c>
+      <c r="J26" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>138</v>
+        <v>43</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
-        <v>7.8125</v>
+        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
+        <v>7.8125000000000009</v>
       </c>
       <c r="D27" s="1">
         <v>8</v>
       </c>
       <c r="E27" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F27" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G27" s="1">
         <v>8</v>
       </c>
       <c r="H27" s="3">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="I27" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="J27" t="e" vm="1">
+        <v>6.1</v>
+      </c>
+      <c r="J27" s="1"/>
+      <c r="K27" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
-        <v>7.7874999999999996</v>
+        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
+        <v>7.8125</v>
       </c>
       <c r="D28" s="1">
         <v>8</v>
@@ -3039,13 +3057,13 @@
         <v>8</v>
       </c>
       <c r="G28" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H28" s="3">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="I28" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="J28" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3056,11 +3074,11 @@
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B29" s="2" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
-        <v>7.7250000000000005</v>
+        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
+        <v>7.7874999999999996</v>
       </c>
       <c r="D29" s="1">
         <v>8</v>
@@ -3072,36 +3090,34 @@
         <v>8</v>
       </c>
       <c r="G29" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H29" s="3">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="I29" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J29" s="1" t="e" vm="4">
+        <v>6.3</v>
+      </c>
+      <c r="J29" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K29" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
-        <v>142</v>
+        <v>73</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
-        <v>7.6624999999999996</v>
+        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
+        <v>7.7250000000000005</v>
       </c>
       <c r="D30" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F30" s="1">
         <v>8</v>
@@ -3110,24 +3126,26 @@
         <v>8</v>
       </c>
       <c r="H30" s="3">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="I30" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="J30" t="e" vm="1">
+        <v>6.4</v>
+      </c>
+      <c r="J30" s="1" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
-      <c r="K30" s="1"/>
+      <c r="K30" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B31" s="2" t="s">
-        <v>192</v>
+        <v>142</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3143,10 +3161,10 @@
         <v>8</v>
       </c>
       <c r="H31" s="3">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="I31" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="J31" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3157,44 +3175,44 @@
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32" s="2" t="s">
-        <v>47</v>
+        <v>192</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
-        <v>7.6000000000000005</v>
+        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
+        <v>7.6624999999999996</v>
       </c>
       <c r="D32" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F32" s="1">
         <v>8</v>
       </c>
       <c r="G32" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H32" s="3">
-        <v>8.6</v>
+        <v>7.5</v>
       </c>
       <c r="I32" s="3">
-        <v>7.6</v>
-      </c>
-      <c r="J32" s="1"/>
-      <c r="K32" t="e" vm="2">
+        <v>6.3</v>
+      </c>
+      <c r="J32" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
-        <v>198</v>
+        <v>47</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
-        <v>7.5625</v>
+        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
+        <v>7.6000000000000005</v>
       </c>
       <c r="D33" s="1">
         <v>8</v>
@@ -3203,218 +3221,219 @@
         <v>8</v>
       </c>
       <c r="F33" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G33" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H33" s="3">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="I33" s="3">
-        <v>6.7</v>
-      </c>
-      <c r="J33" t="e" vm="1">
+        <v>7.6</v>
+      </c>
+      <c r="J33" s="1"/>
+      <c r="K33" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="s">
-        <v>15</v>
+        <v>198</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
-        <v>7.5250000000000004</v>
+        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
+        <v>7.5625</v>
       </c>
       <c r="D34" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E34" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F34" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G34" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H34" s="3">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="I34" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="J34" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K34" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
-      <c r="L34" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="2" t="s">
-        <v>210</v>
+        <v>15</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E35" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" s="1">
         <v>8</v>
       </c>
       <c r="G35" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H35" s="3">
-        <v>7</v>
+        <v>8.1</v>
       </c>
       <c r="I35" s="3">
-        <v>5.2</v>
+        <v>7</v>
       </c>
       <c r="J35" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-      <c r="M35" s="1"/>
+      <c r="K35" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L35" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
-        <v>105</v>
+        <v>210</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
-        <v>7.5249999999999995</v>
+        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
+        <v>7.5250000000000004</v>
       </c>
       <c r="D36" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E36" s="1">
         <v>8</v>
       </c>
       <c r="F36" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G36" s="1">
         <v>8</v>
       </c>
       <c r="H36" s="3">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="I36" s="3">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
       <c r="J36" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K36" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
-        <v>141</v>
+        <v>105</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
         <v>8</v>
       </c>
       <c r="E37" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37" s="1">
         <v>7</v>
       </c>
       <c r="G37" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H37" s="3">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="I37" s="3">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="J37" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K37" s="1"/>
+      <c r="K37" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38" s="2" t="s">
-        <v>16</v>
+        <v>141</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
-        <v>7.4874999999999989</v>
+        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
+        <v>7.5249999999999995</v>
       </c>
       <c r="D38" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E38" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F38" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G38" s="1">
         <v>7</v>
       </c>
       <c r="H38" s="3">
-        <v>8.3000000000000007</v>
+        <v>7.8</v>
       </c>
       <c r="I38" s="3">
-        <v>7.3</v>
-      </c>
-      <c r="J38" s="1"/>
+        <v>6.6</v>
+      </c>
+      <c r="J38" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K38" s="1"/>
-      <c r="L38" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B39" s="2" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
-        <v>7.35</v>
+        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
+        <v>7.4874999999999989</v>
       </c>
       <c r="D39" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E39" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F39" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G39" s="1">
         <v>7</v>
       </c>
       <c r="H39" s="3">
-        <v>8.5</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="I39" s="3">
-        <v>7.8</v>
+        <v>7.3</v>
       </c>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
@@ -3424,62 +3443,61 @@
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40" s="2" t="s">
-        <v>185</v>
+        <v>50</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
-        <v>7.3</v>
+        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
+        <v>7.35</v>
       </c>
       <c r="D40" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E40" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F40" s="1">
         <v>7</v>
       </c>
       <c r="G40" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H40" s="3">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="I40" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J40" t="e" vm="1">
+        <v>7.8</v>
+      </c>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" s="2" t="s">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
-        <v>7.2500000000000009</v>
+        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
+        <v>7.3</v>
       </c>
       <c r="D41" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E41" s="1">
         <v>8</v>
       </c>
       <c r="F41" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G41" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H41" s="3">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="I41" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="J41" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3490,29 +3508,29 @@
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
-        <v>7.25</v>
+        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
+        <v>7.2500000000000009</v>
       </c>
       <c r="D42" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E42" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F42" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G42" s="1">
         <v>7</v>
       </c>
       <c r="H42" s="3">
-        <v>8.4</v>
+        <v>6.7</v>
       </c>
       <c r="I42" s="3">
-        <v>7.2</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="J42" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3523,129 +3541,129 @@
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
+        <v>7.25</v>
+      </c>
+      <c r="D43" s="1">
+        <v>8</v>
+      </c>
+      <c r="E43" s="1">
+        <v>5</v>
+      </c>
+      <c r="F43" s="1">
+        <v>7</v>
+      </c>
+      <c r="G43" s="1">
+        <v>7</v>
+      </c>
+      <c r="H43" s="3">
+        <v>8.4</v>
+      </c>
+      <c r="I43" s="3">
         <v>7.2</v>
-      </c>
-      <c r="D43" s="1">
-        <v>8</v>
-      </c>
-      <c r="E43" s="1">
-        <v>8</v>
-      </c>
-      <c r="F43" s="1">
-        <v>7</v>
-      </c>
-      <c r="G43" s="1">
-        <v>5</v>
-      </c>
-      <c r="H43" s="3">
-        <v>8</v>
-      </c>
-      <c r="I43" s="3">
-        <v>6.6</v>
       </c>
       <c r="J43" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K43" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
         <v>7.2</v>
       </c>
       <c r="D44" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E44" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F44" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G44" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H44" s="3">
-        <v>8.6</v>
+        <v>8</v>
       </c>
       <c r="I44" s="3">
-        <v>7.4</v>
-      </c>
-      <c r="J44" s="1"/>
-      <c r="K44" s="1"/>
-      <c r="L44" t="e" vm="5">
+        <v>6.6</v>
+      </c>
+      <c r="J44" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K44" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1875000000000009</v>
+        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
+        <v>7.2</v>
       </c>
       <c r="D45" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E45" s="1">
         <v>7</v>
       </c>
       <c r="F45" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G45" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H45" s="3">
-        <v>6.7</v>
+        <v>8.6</v>
       </c>
       <c r="I45" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="J45" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K45" s="1"/>
-      <c r="L45" s="1"/>
-      <c r="M45" s="1"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1875</v>
+        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
+        <v>7.1875000000000009</v>
       </c>
       <c r="D46" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E46" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F46" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G46" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H46" s="3">
-        <v>9.1</v>
+        <v>6.7</v>
       </c>
       <c r="I46" s="3">
-        <v>8.3000000000000007</v>
+        <v>6.1</v>
       </c>
       <c r="J46" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3656,129 +3674,129 @@
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1749999999999998</v>
+        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
+        <v>7.1875</v>
       </c>
       <c r="D47" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E47" s="1">
         <v>6</v>
       </c>
       <c r="F47" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G47" s="1">
         <v>7</v>
       </c>
       <c r="H47" s="3">
-        <v>7.5</v>
+        <v>9.1</v>
       </c>
       <c r="I47" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J47" s="1"/>
-      <c r="K47" t="e" vm="2">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J47" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="L47" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D48" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E48" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F48" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G48" s="1">
         <v>7</v>
       </c>
       <c r="H48" s="3">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="I48" s="3">
-        <v>7.4</v>
+        <v>5.4</v>
       </c>
       <c r="J48" s="1"/>
       <c r="K48" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="L48" s="1"/>
-      <c r="M48" s="1"/>
+      <c r="L48" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>234</v>
+        <v>49</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1000000000000005</v>
+        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
+        <v>7.1749999999999998</v>
       </c>
       <c r="D49" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E49" s="1">
         <v>8</v>
       </c>
       <c r="F49" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G49" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H49" s="3">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
       <c r="I49" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J49" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J49" s="1"/>
+      <c r="K49" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
-        <v>7.0875000000000004</v>
+        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
+        <v>7.1000000000000005</v>
       </c>
       <c r="D50" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E50" s="1">
         <v>8</v>
       </c>
       <c r="F50" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G50" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H50" s="3">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="I50" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="J50" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3789,14 +3807,14 @@
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D51" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E51" s="1">
         <v>8</v>
@@ -3805,144 +3823,145 @@
         <v>7</v>
       </c>
       <c r="G51" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H51" s="3">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="I51" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="J51" s="1"/>
+        <v>6.3</v>
+      </c>
+      <c r="J51" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>71</v>
+        <v>231</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9750000000000005</v>
+        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D52" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E52" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F52" s="1">
         <v>7</v>
       </c>
       <c r="G52" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H52" s="3">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="I52" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J52" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K52" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+        <v>5.5</v>
+      </c>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9</v>
+        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <v>6.9750000000000005</v>
       </c>
       <c r="D53" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E53" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F53" s="1">
         <v>7</v>
       </c>
       <c r="G53" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H53" s="3">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="I53" s="3">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="J53" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K53" s="1"/>
+      <c r="K53" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8750000000000009</v>
+        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <v>6.9</v>
       </c>
       <c r="D54" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E54" s="1">
         <v>6</v>
       </c>
       <c r="F54" s="1">
+        <v>7</v>
+      </c>
+      <c r="G54" s="1">
         <v>5</v>
       </c>
-      <c r="G54" s="1">
-        <v>7</v>
-      </c>
       <c r="H54" s="3">
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
       <c r="I54" s="3">
-        <v>8.6</v>
-      </c>
-      <c r="J54" s="1"/>
+        <v>7.2</v>
+      </c>
+      <c r="J54" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K54" s="1"/>
-      <c r="L54" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8</v>
+        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <v>6.8750000000000009</v>
       </c>
       <c r="D55" s="1">
         <v>6</v>
       </c>
       <c r="E55" s="1">
+        <v>6</v>
+      </c>
+      <c r="F55" s="1">
         <v>5</v>
       </c>
-      <c r="F55" s="1">
-        <v>6</v>
-      </c>
       <c r="G55" s="1">
         <v>7</v>
       </c>
       <c r="H55" s="3">
-        <v>8.5</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="I55" s="3">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
@@ -3952,17 +3971,17 @@
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7750000000000004</v>
+        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <v>6.8</v>
       </c>
       <c r="D56" s="1">
         <v>6</v>
       </c>
       <c r="E56" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F56" s="1">
         <v>6</v>
@@ -3971,43 +3990,42 @@
         <v>7</v>
       </c>
       <c r="H56" s="3">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="I56" s="3">
-        <v>6.8</v>
-      </c>
-      <c r="J56" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K56" s="1"/>
-      <c r="L56" s="1"/>
-      <c r="M56" s="1"/>
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
-        <v>6.75</v>
+        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <v>6.7750000000000004</v>
       </c>
       <c r="D57" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E57" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F57" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G57" s="1">
         <v>7</v>
       </c>
       <c r="H57" s="3">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I57" s="3">
-        <v>4.2</v>
+        <v>6.8</v>
       </c>
       <c r="J57" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4018,61 +4036,62 @@
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7250000000000005</v>
+        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <v>6.75</v>
       </c>
       <c r="D58" s="1">
         <v>8</v>
       </c>
       <c r="E58" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F58" s="1">
         <v>7</v>
       </c>
       <c r="G58" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H58" s="3">
-        <v>7.7</v>
+        <v>5.9</v>
       </c>
       <c r="I58" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J58" s="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="J58" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K58" s="1"/>
-      <c r="L58" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7</v>
+        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <v>6.7250000000000005</v>
       </c>
       <c r="D59" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E59" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F59" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G59" s="1">
         <v>6</v>
       </c>
       <c r="H59" s="3">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
       <c r="I59" s="3">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
@@ -4082,79 +4101,76 @@
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
-        <v>6.55</v>
+        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <v>6.7</v>
       </c>
       <c r="D60" s="1">
         <v>5</v>
       </c>
       <c r="E60" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F60" s="1">
         <v>6</v>
       </c>
       <c r="G60" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H60" s="3">
-        <v>7</v>
+        <v>8.6</v>
       </c>
       <c r="I60" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J60" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K60" s="1"/>
-      <c r="L60" s="1"/>
-      <c r="M60" s="1"/>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4875000000000007</v>
+        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <v>6.55</v>
       </c>
       <c r="D61" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E61" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F61" s="1">
         <v>6</v>
       </c>
       <c r="G61" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H61" s="3">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="I61" s="3">
-        <v>7.7</v>
-      </c>
-      <c r="J61" s="1"/>
-      <c r="K61" t="e" vm="2">
+        <v>5.4</v>
+      </c>
+      <c r="J61" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K61" s="1"/>
       <c r="L61" s="1"/>
-      <c r="M61" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="M61" s="1"/>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4</v>
+        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <v>6.4875000000000007</v>
       </c>
       <c r="D62" s="1">
         <v>6</v>
@@ -4166,46 +4182,48 @@
         <v>6</v>
       </c>
       <c r="G62" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H62" s="3">
         <v>8.1</v>
       </c>
       <c r="I62" s="3">
-        <v>6</v>
-      </c>
-      <c r="J62" t="e" vm="1">
+        <v>7.7</v>
+      </c>
+      <c r="J62" s="1"/>
+      <c r="K62" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K62" s="1"/>
       <c r="L62" s="1"/>
-      <c r="M62" s="1"/>
+      <c r="M62" s="1" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <v>6.4</v>
       </c>
       <c r="D63" s="1">
         <v>6</v>
       </c>
       <c r="E63" s="1">
+        <v>6</v>
+      </c>
+      <c r="F63" s="1">
+        <v>6</v>
+      </c>
+      <c r="G63" s="1">
         <v>5</v>
       </c>
-      <c r="F63" s="1">
-        <v>6</v>
-      </c>
-      <c r="G63" s="1">
-        <v>6</v>
-      </c>
       <c r="H63" s="3">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="I63" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="J63" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4216,66 +4234,66 @@
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
-        <v>6.2250000000000005</v>
+        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D64" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E64" s="1">
         <v>5</v>
       </c>
       <c r="F64" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G64" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H64" s="3">
-        <v>8.1999999999999993</v>
+        <v>7.8</v>
       </c>
       <c r="I64" s="3">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="J64" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K64" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K64" s="1"/>
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1750000000000007</v>
+        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D65" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E65" s="1">
         <v>5</v>
       </c>
       <c r="F65" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G65" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H65" s="3">
-        <v>6.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I65" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="J65" s="1"/>
+        <v>6.4</v>
+      </c>
+      <c r="J65" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K65" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -4284,62 +4302,62 @@
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1624999999999996</v>
+        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <v>6.1750000000000007</v>
       </c>
       <c r="D66" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F66" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G66" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H66" s="3">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="I66" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="J66" t="e" vm="1">
+        <v>6.2</v>
+      </c>
+      <c r="J66" s="1"/>
+      <c r="K66" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K66" s="1"/>
       <c r="L66" s="1"/>
       <c r="M66" s="1"/>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C71" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
-        <v>5.9749999999999996</v>
+        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D67" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E67" s="1">
         <v>7</v>
       </c>
       <c r="F67" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G67" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H67" s="3">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I67" s="3">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J67" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4350,29 +4368,29 @@
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C68" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7750000000000004</v>
+        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D68" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E68" s="1">
         <v>7</v>
       </c>
       <c r="F68" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G68" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H68" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I68" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J68" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4383,29 +4401,29 @@
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C69" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7625000000000002</v>
+        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D69" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E69" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" s="1">
+        <v>7</v>
+      </c>
+      <c r="G69" s="1">
+        <v>3</v>
+      </c>
+      <c r="H69" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I69" s="3">
         <v>5</v>
-      </c>
-      <c r="G69" s="1">
-        <v>5</v>
-      </c>
-      <c r="H69" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I69" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J69" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4416,68 +4434,101 @@
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C70" s="5">
-        <f t="shared" si="2"/>
-        <v>5.4625000000000004</v>
+        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D70" s="1">
+        <v>8</v>
+      </c>
+      <c r="E70" s="1">
+        <v>8</v>
+      </c>
+      <c r="F70" s="1">
         <v>5</v>
       </c>
-      <c r="E70" s="1">
-        <v>7</v>
-      </c>
-      <c r="F70" s="1">
-        <v>6</v>
-      </c>
       <c r="G70" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H70" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I70" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I70" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J70" s="1"/>
+      <c r="J70" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K70" s="1"/>
-      <c r="L70" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L70" s="1"/>
+      <c r="M70" s="1"/>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C71" s="5">
+        <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D71" s="1">
+        <v>5</v>
+      </c>
+      <c r="E71" s="1">
+        <v>7</v>
+      </c>
+      <c r="F71" s="1">
+        <v>6</v>
+      </c>
+      <c r="G71" s="1">
+        <v>7</v>
+      </c>
+      <c r="H71" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I71" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B72" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C71" s="5">
-        <f t="shared" si="2"/>
+      <c r="C72" s="5">
+        <f>AVERAGE(D72,E72,F72,F72,G72,H72,H72,I72)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D72" s="1">
         <v>2</v>
       </c>
-      <c r="E71" s="1">
+      <c r="E72" s="1">
         <v>4</v>
       </c>
-      <c r="F71" s="1">
+      <c r="F72" s="1">
         <v>2</v>
       </c>
-      <c r="G71" s="1">
+      <c r="G72" s="1">
         <v>5</v>
       </c>
-      <c r="H71" s="3">
+      <c r="H72" s="3">
         <v>7.7</v>
       </c>
-      <c r="I71" s="3">
+      <c r="I72" s="3">
         <v>6.3</v>
       </c>
-      <c r="J71" t="e" vm="1">
+      <c r="J72" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K71" s="1"/>
-      <c r="L71" s="1"/>
-      <c r="M71" s="1"/>
+      <c r="K72" s="1"/>
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4547,7 +4598,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4575,7 +4626,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4603,7 +4654,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4630,7 +4681,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4657,7 +4708,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4684,7 +4735,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4711,7 +4762,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4738,7 +4789,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4765,7 +4816,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4792,7 +4843,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -4819,7 +4870,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -4846,7 +4897,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -4873,7 +4924,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -4900,7 +4951,7 @@
         <v>235</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.1875</v>
       </c>
       <c r="D16" s="1">
@@ -4927,7 +4978,7 @@
         <v>125</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.1750000000000007</v>
       </c>
       <c r="D17" s="1">
@@ -4954,7 +5005,7 @@
         <v>81</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.1624999999999996</v>
       </c>
       <c r="D18" s="1">
@@ -4981,7 +5032,7 @@
         <v>77</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.15</v>
       </c>
       <c r="D19" s="1">
@@ -5008,7 +5059,7 @@
         <v>54</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -5035,7 +5086,7 @@
         <v>126</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8.0750000000000011</v>
       </c>
       <c r="D21" s="1">
@@ -5062,7 +5113,7 @@
         <v>58</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>8.0625</v>
       </c>
       <c r="D22" s="1">
@@ -5089,7 +5140,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>7.9249999999999998</v>
       </c>
       <c r="D23" s="1">
@@ -5116,7 +5167,7 @@
         <v>122</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>7.9124999999999996</v>
       </c>
       <c r="D24" s="1">
@@ -5143,7 +5194,7 @@
         <v>108</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.8999999999999995</v>
       </c>
       <c r="D25" s="1">
@@ -5170,7 +5221,7 @@
         <v>78</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.875</v>
       </c>
       <c r="D26" s="1">
@@ -5197,7 +5248,7 @@
         <v>109</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5224,7 +5275,7 @@
         <v>61</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D28" s="1">
@@ -5251,7 +5302,7 @@
         <v>193</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7750000000000004</v>
       </c>
       <c r="D29" s="1">
@@ -5278,7 +5329,7 @@
         <v>60</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7375000000000007</v>
       </c>
       <c r="D30" s="1">
@@ -5305,7 +5356,7 @@
         <v>38</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.7000000000000011</v>
       </c>
       <c r="D31" s="1">
@@ -5332,7 +5383,7 @@
         <v>63</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999993</v>
       </c>
       <c r="D32" s="1">
@@ -5359,7 +5410,7 @@
         <v>123</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5874999999999995</v>
       </c>
       <c r="D33" s="1">
@@ -5386,7 +5437,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000011</v>
       </c>
       <c r="D34" s="1">
@@ -5413,7 +5464,7 @@
         <v>67</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5750000000000002</v>
       </c>
       <c r="D35" s="1">
@@ -5440,7 +5491,7 @@
         <v>62</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5467,7 +5518,7 @@
         <v>217</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D37" s="1">
@@ -5494,7 +5545,7 @@
         <v>55</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.5624999999999991</v>
       </c>
       <c r="D38" s="1">
@@ -5521,7 +5572,7 @@
         <v>201</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.55</v>
       </c>
       <c r="D39" s="1">
@@ -5548,7 +5599,7 @@
         <v>69</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -5575,7 +5626,7 @@
         <v>132</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.5125000000000002</v>
       </c>
       <c r="D41" s="1">
@@ -5602,7 +5653,7 @@
         <v>230</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.5124999999999993</v>
       </c>
       <c r="D42" s="1">
@@ -5629,7 +5680,7 @@
         <v>205</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.4875000000000007</v>
       </c>
       <c r="D43" s="1">
@@ -5656,7 +5707,7 @@
         <v>172</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.4749999999999996</v>
       </c>
       <c r="D44" s="1">
@@ -5683,7 +5734,7 @@
         <v>130</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D45" s="1">
@@ -5710,7 +5761,7 @@
         <v>97</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.4375</v>
       </c>
       <c r="D46" s="1">
@@ -5737,7 +5788,7 @@
         <v>100</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.4249999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -5764,7 +5815,7 @@
         <v>131</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.4124999999999996</v>
       </c>
       <c r="D48" s="1">
@@ -5791,7 +5842,7 @@
         <v>220</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999998</v>
       </c>
       <c r="D49" s="1">
@@ -5818,7 +5869,7 @@
         <v>175</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999989</v>
       </c>
       <c r="D50" s="1">
@@ -5845,7 +5896,7 @@
         <v>52</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.3500000000000005</v>
       </c>
       <c r="D51" s="1">
@@ -5872,7 +5923,7 @@
         <v>165</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.3249999999999993</v>
       </c>
       <c r="D52" s="1">
@@ -5899,7 +5950,7 @@
         <v>224</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.3125</v>
       </c>
       <c r="D53" s="1">
@@ -5926,7 +5977,7 @@
         <v>111</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D54" s="1">
@@ -5953,7 +6004,7 @@
         <v>103</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D55" s="1">
@@ -5980,7 +6031,7 @@
         <v>181</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D56" s="1">
@@ -6007,7 +6058,7 @@
         <v>225</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>7.2624999999999993</v>
       </c>
       <c r="D57" s="1">
@@ -6034,7 +6085,7 @@
         <v>147</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>7.2374999999999998</v>
       </c>
       <c r="D58" s="1">
@@ -6061,7 +6112,7 @@
         <v>59</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>7.2250000000000005</v>
       </c>
       <c r="D59" s="1">
@@ -6088,7 +6139,7 @@
         <v>65</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>7.2125000000000004</v>
       </c>
       <c r="D60" s="1">
@@ -6115,7 +6166,7 @@
         <v>146</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>7.2124999999999995</v>
       </c>
       <c r="D61" s="1">
@@ -6142,7 +6193,7 @@
         <v>94</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
       <c r="D62" s="1">
@@ -6169,7 +6220,7 @@
         <v>53</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="D63" s="1">
@@ -6196,7 +6247,7 @@
         <v>104</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>7.1375000000000011</v>
       </c>
       <c r="D64" s="1">
@@ -6223,7 +6274,7 @@
         <v>40</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>7.1250000000000009</v>
       </c>
       <c r="D65" s="1">
@@ -6250,7 +6301,7 @@
         <v>39</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>7.125</v>
       </c>
       <c r="D66" s="1">
@@ -6277,7 +6328,7 @@
         <v>133</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D67" s="1">
@@ -6304,7 +6355,7 @@
         <v>98</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D68" s="1">
@@ -6331,7 +6382,7 @@
         <v>171</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D69" s="1">
@@ -6358,7 +6409,7 @@
         <v>110</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D70" s="1">
@@ -6385,7 +6436,7 @@
         <v>143</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D71" s="1">
@@ -6412,7 +6463,7 @@
         <v>177</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>7.0749999999999993</v>
       </c>
       <c r="D72" s="1">
@@ -6439,7 +6490,7 @@
         <v>176</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="D73" s="1">
@@ -6466,7 +6517,7 @@
         <v>221</v>
       </c>
       <c r="C74" s="5">
-        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
+        <f t="shared" si="2"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="D74" s="1">
@@ -6493,7 +6544,7 @@
         <v>95</v>
       </c>
       <c r="C75" s="5">
-        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
+        <f t="shared" si="2"/>
         <v>6.9375</v>
       </c>
       <c r="D75" s="1">
@@ -6520,7 +6571,7 @@
         <v>164</v>
       </c>
       <c r="C76" s="5">
-        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
+        <f t="shared" si="2"/>
         <v>6.9124999999999996</v>
       </c>
       <c r="D76" s="1">
@@ -6547,7 +6598,7 @@
         <v>157</v>
       </c>
       <c r="C77" s="5">
-        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
+        <f t="shared" si="2"/>
         <v>6.8999999999999995</v>
       </c>
       <c r="D77" s="1">
@@ -6574,7 +6625,7 @@
         <v>88</v>
       </c>
       <c r="C78" s="5">
-        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D78" s="1">
@@ -6601,7 +6652,7 @@
         <v>184</v>
       </c>
       <c r="C79" s="5">
-        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D79" s="1">
@@ -6628,7 +6679,7 @@
         <v>119</v>
       </c>
       <c r="C80" s="5">
-        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
+        <f t="shared" si="2"/>
         <v>6.85</v>
       </c>
       <c r="D80" s="1">
@@ -6655,7 +6706,7 @@
         <v>196</v>
       </c>
       <c r="C81" s="5">
-        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
+        <f t="shared" si="2"/>
         <v>6.7999999999999989</v>
       </c>
       <c r="D81" s="1">
@@ -6682,7 +6733,7 @@
         <v>57</v>
       </c>
       <c r="C82" s="5">
-        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
+        <f t="shared" si="2"/>
         <v>6.6999999999999993</v>
       </c>
       <c r="D82" s="1">
@@ -6709,7 +6760,7 @@
         <v>87</v>
       </c>
       <c r="C83" s="5">
-        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
+        <f t="shared" si="2"/>
         <v>6.6875</v>
       </c>
       <c r="D83" s="1">
@@ -6736,7 +6787,7 @@
         <v>211</v>
       </c>
       <c r="C84" s="5">
-        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
+        <f t="shared" si="2"/>
         <v>6.6375000000000002</v>
       </c>
       <c r="D84" s="1">
@@ -6763,7 +6814,7 @@
         <v>219</v>
       </c>
       <c r="C85" s="5">
-        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
+        <f t="shared" si="2"/>
         <v>6.6374999999999993</v>
       </c>
       <c r="D85" s="1">
@@ -6790,7 +6841,7 @@
         <v>41</v>
       </c>
       <c r="C86" s="5">
-        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999989</v>
       </c>
       <c r="D86" s="1">
@@ -6817,7 +6868,7 @@
         <v>117</v>
       </c>
       <c r="C87" s="5">
-        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D87" s="1">
@@ -6844,7 +6895,7 @@
         <v>179</v>
       </c>
       <c r="C88" s="5">
-        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D88" s="1">
@@ -6871,7 +6922,7 @@
         <v>215</v>
       </c>
       <c r="C89" s="5">
-        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
+        <f t="shared" si="2"/>
         <v>6.5750000000000002</v>
       </c>
       <c r="D89" s="1">
@@ -6898,7 +6949,7 @@
         <v>168</v>
       </c>
       <c r="C90" s="5">
-        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
+        <f t="shared" si="2"/>
         <v>6.5499999999999989</v>
       </c>
       <c r="D90" s="1">
@@ -6925,7 +6976,7 @@
         <v>197</v>
       </c>
       <c r="C91" s="5">
-        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <f t="shared" si="2"/>
         <v>6.5375000000000005</v>
       </c>
       <c r="D91" s="1">
@@ -6952,7 +7003,7 @@
         <v>202</v>
       </c>
       <c r="C92" s="5">
-        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D92" s="1">
@@ -6979,7 +7030,7 @@
         <v>183</v>
       </c>
       <c r="C93" s="5">
-        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D93" s="1">
@@ -7006,7 +7057,7 @@
         <v>200</v>
       </c>
       <c r="C94" s="5">
-        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D94" s="1">
@@ -7033,7 +7084,7 @@
         <v>188</v>
       </c>
       <c r="C95" s="5">
-        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D95" s="1">
@@ -7060,7 +7111,7 @@
         <v>208</v>
       </c>
       <c r="C96" s="5">
-        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D96" s="1">
@@ -7087,7 +7138,7 @@
         <v>134</v>
       </c>
       <c r="C97" s="5">
-        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
+        <f t="shared" si="2"/>
         <v>6.3125</v>
       </c>
       <c r="D97" s="1">
@@ -7114,7 +7165,7 @@
         <v>144</v>
       </c>
       <c r="C98" s="5">
-        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <f t="shared" si="2"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D98" s="1">
@@ -7141,7 +7192,7 @@
         <v>64</v>
       </c>
       <c r="C99" s="5">
-        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.2749999999999995</v>
       </c>
       <c r="D99" s="1">
@@ -7168,7 +7219,7 @@
         <v>75</v>
       </c>
       <c r="C100" s="5">
-        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
+        <f t="shared" si="3"/>
         <v>6.2125000000000004</v>
       </c>
       <c r="D100" s="1">
@@ -7195,7 +7246,7 @@
         <v>19</v>
       </c>
       <c r="C101" s="5">
-        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <f t="shared" si="3"/>
         <v>6.2124999999999995</v>
       </c>
       <c r="D101" s="1">
@@ -7222,7 +7273,7 @@
         <v>101</v>
       </c>
       <c r="C102" s="5">
-        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <f t="shared" si="3"/>
         <v>6.15</v>
       </c>
       <c r="D102" s="1">
@@ -7249,7 +7300,7 @@
         <v>158</v>
       </c>
       <c r="C103" s="5">
-        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <f t="shared" si="3"/>
         <v>6.0874999999999995</v>
       </c>
       <c r="D103" s="1">
@@ -7276,7 +7327,7 @@
         <v>222</v>
       </c>
       <c r="C104" s="5">
-        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <f t="shared" si="3"/>
         <v>6.0625</v>
       </c>
       <c r="D104" s="1">
@@ -7303,7 +7354,7 @@
         <v>214</v>
       </c>
       <c r="C105" s="5">
-        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <f t="shared" si="3"/>
         <v>6.0500000000000007</v>
       </c>
       <c r="D105" s="1">
@@ -7330,7 +7381,7 @@
         <v>160</v>
       </c>
       <c r="C106" s="5">
-        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D106" s="1">
@@ -7357,7 +7408,7 @@
         <v>206</v>
       </c>
       <c r="C107" s="5">
-        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D107" s="1">
@@ -7384,7 +7435,7 @@
         <v>159</v>
       </c>
       <c r="C108" s="5">
-        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <f t="shared" si="3"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="D108" s="1">
@@ -7411,7 +7462,7 @@
         <v>195</v>
       </c>
       <c r="C109" s="5">
-        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
+        <f t="shared" si="3"/>
         <v>5.8875000000000011</v>
       </c>
       <c r="D109" s="1">
@@ -7438,7 +7489,7 @@
         <v>186</v>
       </c>
       <c r="C110" s="5">
-        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <f t="shared" si="3"/>
         <v>5.8125000000000009</v>
       </c>
       <c r="D110" s="1">
@@ -7465,7 +7516,7 @@
         <v>209</v>
       </c>
       <c r="C111" s="5">
-        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <f t="shared" si="3"/>
         <v>5.8000000000000007</v>
       </c>
       <c r="D111" s="1">
@@ -7492,7 +7543,7 @@
         <v>113</v>
       </c>
       <c r="C112" s="5">
-        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <f t="shared" si="3"/>
         <v>5.7374999999999989</v>
       </c>
       <c r="D112" s="1">
@@ -7519,7 +7570,7 @@
         <v>187</v>
       </c>
       <c r="C113" s="5">
-        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <f t="shared" si="3"/>
         <v>5.7250000000000005</v>
       </c>
       <c r="D113" s="1">
@@ -7546,7 +7597,7 @@
         <v>26</v>
       </c>
       <c r="C114" s="5">
-        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <f t="shared" si="3"/>
         <v>5.6749999999999998</v>
       </c>
       <c r="D114" s="1">
@@ -7573,7 +7624,7 @@
         <v>149</v>
       </c>
       <c r="C115" s="5">
-        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D115" s="1">
@@ -7600,7 +7651,7 @@
         <v>156</v>
       </c>
       <c r="C116" s="5">
-        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D116" s="1">
@@ -7627,7 +7678,7 @@
         <v>229</v>
       </c>
       <c r="C117" s="5">
-        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <f t="shared" si="3"/>
         <v>5.5375000000000005</v>
       </c>
       <c r="D117" s="1">
@@ -7654,7 +7705,7 @@
         <v>166</v>
       </c>
       <c r="C118" s="5">
-        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D118" s="1">
@@ -7681,7 +7732,7 @@
         <v>191</v>
       </c>
       <c r="C119" s="5">
-        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D119" s="1">
@@ -7708,7 +7759,7 @@
         <v>228</v>
       </c>
       <c r="C120" s="5">
-        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <f t="shared" si="3"/>
         <v>5.3875000000000011</v>
       </c>
       <c r="D120" s="1">
@@ -7735,7 +7786,7 @@
         <v>204</v>
       </c>
       <c r="C121" s="5">
-        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <f t="shared" si="3"/>
         <v>5.3750000000000009</v>
       </c>
       <c r="D121" s="1">
@@ -7762,7 +7813,7 @@
         <v>190</v>
       </c>
       <c r="C122" s="5">
-        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
+        <f t="shared" si="3"/>
         <v>5.375</v>
       </c>
       <c r="D122" s="1">
@@ -7789,7 +7840,7 @@
         <v>182</v>
       </c>
       <c r="C123" s="5">
-        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <f t="shared" si="3"/>
         <v>5.2875000000000005</v>
       </c>
       <c r="D123" s="1">
@@ -7816,7 +7867,7 @@
         <v>232</v>
       </c>
       <c r="C124" s="5">
-        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <f t="shared" si="3"/>
         <v>5.2</v>
       </c>
       <c r="D124" s="1">
@@ -7843,7 +7894,7 @@
         <v>74</v>
       </c>
       <c r="C125" s="5">
-        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <f t="shared" si="3"/>
         <v>5.1875</v>
       </c>
       <c r="D125" s="1">
@@ -7870,7 +7921,7 @@
         <v>145</v>
       </c>
       <c r="C126" s="5">
-        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <f t="shared" si="3"/>
         <v>5.1124999999999998</v>
       </c>
       <c r="D126" s="1">
@@ -7897,7 +7948,7 @@
         <v>223</v>
       </c>
       <c r="C127" s="5">
-        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <f t="shared" si="3"/>
         <v>5.0750000000000002</v>
       </c>
       <c r="D127" s="1">
@@ -7924,7 +7975,7 @@
         <v>21</v>
       </c>
       <c r="C128" s="5">
-        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <f t="shared" si="3"/>
         <v>5.05</v>
       </c>
       <c r="D128" s="1">
@@ -7951,7 +8002,7 @@
         <v>203</v>
       </c>
       <c r="C129" s="5">
-        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <f t="shared" si="3"/>
         <v>4.9875000000000007</v>
       </c>
       <c r="D129" s="1">
@@ -7978,7 +8029,7 @@
         <v>169</v>
       </c>
       <c r="C130" s="5">
-        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <f t="shared" si="3"/>
         <v>4.9874999999999998</v>
       </c>
       <c r="D130" s="1">
@@ -8005,7 +8056,7 @@
         <v>163</v>
       </c>
       <c r="C131" s="5">
-        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>4.8499999999999996</v>
       </c>
       <c r="D131" s="1">
@@ -8032,7 +8083,7 @@
         <v>162</v>
       </c>
       <c r="C132" s="5">
-        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <f t="shared" si="4"/>
         <v>4.7875000000000005</v>
       </c>
       <c r="D132" s="1">
@@ -8059,7 +8110,7 @@
         <v>213</v>
       </c>
       <c r="C133" s="5">
-        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <f t="shared" si="4"/>
         <v>4.6124999999999998</v>
       </c>
       <c r="D133" s="1">
@@ -8086,7 +8137,7 @@
         <v>154</v>
       </c>
       <c r="C134" s="5">
-        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <f t="shared" si="4"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="D134" s="1">
@@ -8113,7 +8164,7 @@
         <v>135</v>
       </c>
       <c r="C135" s="5">
-        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <f t="shared" si="4"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D135" s="1">
@@ -8140,7 +8191,7 @@
         <v>161</v>
       </c>
       <c r="C136" s="5">
-        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <f t="shared" si="4"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="D136" s="1">
@@ -8167,7 +8218,7 @@
         <v>114</v>
       </c>
       <c r="C137" s="5">
-        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <f t="shared" si="4"/>
         <v>4.4124999999999996</v>
       </c>
       <c r="D137" s="1">
@@ -8194,7 +8245,7 @@
         <v>207</v>
       </c>
       <c r="C138" s="5">
-        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <f t="shared" si="4"/>
         <v>4.3375000000000004</v>
       </c>
       <c r="D138" s="1">
@@ -8221,7 +8272,7 @@
         <v>150</v>
       </c>
       <c r="C139" s="5">
-        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <f t="shared" si="4"/>
         <v>4.3374999999999995</v>
       </c>
       <c r="D139" s="1">
@@ -8248,7 +8299,7 @@
         <v>173</v>
       </c>
       <c r="C140" s="5">
-        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <f t="shared" si="4"/>
         <v>4.3125</v>
       </c>
       <c r="D140" s="1">
@@ -8275,7 +8326,7 @@
         <v>212</v>
       </c>
       <c r="C141" s="5">
-        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <f t="shared" si="4"/>
         <v>4.3</v>
       </c>
       <c r="D141" s="1">
@@ -8302,7 +8353,7 @@
         <v>167</v>
       </c>
       <c r="C142" s="5">
-        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <f t="shared" si="4"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="D142" s="1">
@@ -8329,7 +8380,7 @@
         <v>236</v>
       </c>
       <c r="C143" s="5">
-        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <f t="shared" si="4"/>
         <v>4.1749999999999998</v>
       </c>
       <c r="D143" s="1">
@@ -8356,7 +8407,7 @@
         <v>233</v>
       </c>
       <c r="C144" s="5">
-        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <f t="shared" si="4"/>
         <v>4.1625000000000005</v>
       </c>
       <c r="D144" s="1">
@@ -8383,7 +8434,7 @@
         <v>68</v>
       </c>
       <c r="C145" s="5">
-        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <f t="shared" si="4"/>
         <v>4.1124999999999998</v>
       </c>
       <c r="D145" s="1">
@@ -8410,7 +8461,7 @@
         <v>218</v>
       </c>
       <c r="C146" s="5">
-        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <f t="shared" si="4"/>
         <v>3.9499999999999997</v>
       </c>
       <c r="D146" s="1">
@@ -8437,7 +8488,7 @@
         <v>199</v>
       </c>
       <c r="C147" s="5">
-        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <f t="shared" si="4"/>
         <v>3.7375000000000003</v>
       </c>
       <c r="D147" s="1">
@@ -8464,7 +8515,7 @@
         <v>180</v>
       </c>
       <c r="C148" s="5">
-        <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
+        <f t="shared" si="4"/>
         <v>3.5625000000000004</v>
       </c>
       <c r="D148" s="1">
@@ -8491,7 +8542,7 @@
         <v>216</v>
       </c>
       <c r="C149" s="5">
-        <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
+        <f t="shared" si="4"/>
         <v>3.5375000000000005</v>
       </c>
       <c r="D149" s="1">
@@ -8518,7 +8569,7 @@
         <v>189</v>
       </c>
       <c r="C150" s="5">
-        <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <f t="shared" si="4"/>
         <v>3.3250000000000002</v>
       </c>
       <c r="D150" s="1">
@@ -8545,7 +8596,7 @@
         <v>194</v>
       </c>
       <c r="C151" s="5">
-        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <f t="shared" si="4"/>
         <v>3.2749999999999995</v>
       </c>
       <c r="D151" s="1">
@@ -8572,7 +8623,7 @@
         <v>155</v>
       </c>
       <c r="C152" s="5">
-        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
+        <f t="shared" si="4"/>
         <v>2.9124999999999996</v>
       </c>
       <c r="D152" s="1">
@@ -8595,11 +8646,11 @@
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B153" s="9" t="s">
+      <c r="B153" s="2" t="s">
         <v>237</v>
       </c>
       <c r="C153" s="5">
-        <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
+        <f t="shared" si="4"/>
         <v>2.8125</v>
       </c>
       <c r="D153" s="1">
@@ -8626,7 +8677,7 @@
         <v>174</v>
       </c>
       <c r="C154" s="5">
-        <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
+        <f t="shared" si="4"/>
         <v>2.6375000000000002</v>
       </c>
       <c r="D154" s="1">
@@ -8653,7 +8704,7 @@
         <v>226</v>
       </c>
       <c r="C155" s="5">
-        <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
+        <f t="shared" si="4"/>
         <v>2.5125000000000002</v>
       </c>
       <c r="D155" s="1">

</xml_diff>

<commit_message>
V. 137 "El país de los sueños"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5768374-CE86-4B0C-BF95-867E94318FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27437830-5826-439E-8225-4522AFA832CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="241">
   <si>
     <t>Película</t>
   </si>
@@ -1332,6 +1332,9 @@
   </si>
   <si>
     <t>Superintelligence</t>
+  </si>
+  <si>
+    <t>El país de los sueños</t>
   </si>
 </sst>
 </file>
@@ -1435,13 +1438,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1453,45 +1456,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1532,6 +1496,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1658,48 +1661,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M72" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M72" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M72" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M72">
     <sortCondition descending="1" ref="C2:C72"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I156" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I156" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I156">
-    <sortCondition descending="1" ref="C2:C156"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I157" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I157" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I157">
+    <sortCondition descending="1" ref="C2:C157"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2198,7 +2201,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2234,7 +2237,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2301,7 +2304,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2339,7 +2342,7 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -2373,7 +2376,7 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -4338,7 +4341,7 @@
         <v>11</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C72" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>6.1624999999999996</v>
       </c>
       <c r="D67" s="1">
@@ -4551,7 +4554,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K156"/>
+  <dimension ref="B2:K157"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4589,7 +4592,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4619,7 +4622,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4647,7 +4650,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -7296,15 +7299,15 @@
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B103" s="2" t="s">
-        <v>158</v>
+      <c r="B103" s="9" t="s">
+        <v>240</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>6.0874999999999995</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D103" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E103" s="1">
         <v>7</v>
@@ -7316,46 +7319,46 @@
         <v>7</v>
       </c>
       <c r="H103" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I103" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D104" s="1">
         <v>7</v>
       </c>
       <c r="E104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H104" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I104" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D105" s="1">
         <v>7</v>
@@ -7364,25 +7367,25 @@
         <v>6</v>
       </c>
       <c r="F105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G105" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I105" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
@@ -7394,49 +7397,49 @@
         <v>7</v>
       </c>
       <c r="G106" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H106" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I106" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
         <v>6.05</v>
       </c>
       <c r="D107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E107" s="1">
         <v>6</v>
       </c>
       <c r="F107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H107" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I107" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D108" s="1">
         <v>6</v>
@@ -7445,133 +7448,133 @@
         <v>6</v>
       </c>
       <c r="F108" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G108" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H108" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I108" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D109" s="1">
         <v>6</v>
       </c>
       <c r="E109" s="1">
+        <v>6</v>
+      </c>
+      <c r="F109" s="1">
+        <v>8</v>
+      </c>
+      <c r="G109" s="1">
         <v>5</v>
       </c>
-      <c r="F109" s="1">
-        <v>6</v>
-      </c>
-      <c r="G109" s="1">
-        <v>6</v>
-      </c>
       <c r="H109" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I109" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D110" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E110" s="1">
         <v>5</v>
       </c>
       <c r="F110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G110" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I110" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D111" s="1">
         <v>7</v>
       </c>
       <c r="E111" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F111" s="1">
         <v>5</v>
       </c>
       <c r="G111" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H111" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I111" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D112" s="1">
         <v>7</v>
       </c>
       <c r="E112" s="1">
+        <v>6</v>
+      </c>
+      <c r="F112" s="1">
         <v>5</v>
       </c>
-      <c r="F112" s="1">
-        <v>4</v>
-      </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H112" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I112" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
@@ -7583,37 +7586,37 @@
         <v>4</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I113" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D114" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E114" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F114" s="1">
+        <v>4</v>
+      </c>
+      <c r="G114" s="1">
         <v>5</v>
       </c>
-      <c r="G114" s="1">
-        <v>6</v>
-      </c>
       <c r="H114" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I114" s="3">
         <v>6.4</v>
@@ -7621,50 +7624,50 @@
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D115" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E115" s="1">
+        <v>3</v>
+      </c>
+      <c r="F115" s="1">
         <v>5</v>
       </c>
-      <c r="F115" s="1">
-        <v>6</v>
-      </c>
       <c r="G115" s="1">
         <v>6</v>
       </c>
       <c r="H115" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I115" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D116" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E116" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F116" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3">
         <v>5.8</v>
@@ -7675,26 +7678,26 @@
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.5375000000000005</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D117" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E117" s="1">
+        <v>6</v>
+      </c>
+      <c r="F117" s="1">
+        <v>8</v>
+      </c>
+      <c r="G117" s="1">
         <v>5</v>
       </c>
-      <c r="F117" s="1">
-        <v>6</v>
-      </c>
-      <c r="G117" s="1">
-        <v>6</v>
-      </c>
       <c r="H117" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I117" s="3">
         <v>4.9000000000000004</v>
@@ -7702,17 +7705,17 @@
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>166</v>
+        <v>229</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D118" s="1">
         <v>6</v>
       </c>
       <c r="E118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F118" s="1">
         <v>6</v>
@@ -7721,322 +7724,322 @@
         <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I118" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E119" s="1">
         <v>6</v>
       </c>
       <c r="F119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I119" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.3875000000000011</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D120" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E120" s="1">
         <v>6</v>
       </c>
       <c r="F120" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G120" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H120" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I120" s="3">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.3750000000000009</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D121" s="1">
         <v>6</v>
       </c>
       <c r="E121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F121" s="1">
         <v>6</v>
       </c>
       <c r="G121" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H121" s="3">
         <v>4.7</v>
       </c>
       <c r="I121" s="3">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D122" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F122" s="1">
         <v>6</v>
       </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H122" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I122" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D123" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I123" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.2</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D124" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E124" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G124" s="1">
         <v>5</v>
       </c>
       <c r="H124" s="3">
-        <v>7.1</v>
+        <v>6.1</v>
       </c>
       <c r="I124" s="3">
-        <v>6.4</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>74</v>
+        <v>232</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.1875</v>
+        <v>5.2</v>
       </c>
       <c r="D125" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E125" s="1">
+        <v>4</v>
+      </c>
+      <c r="F125" s="1">
+        <v>2</v>
+      </c>
+      <c r="G125" s="1">
         <v>5</v>
       </c>
-      <c r="F125" s="1">
-        <v>6</v>
-      </c>
-      <c r="G125" s="1">
-        <v>6</v>
-      </c>
       <c r="H125" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I125" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D126" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E126" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G126" s="1">
         <v>6</v>
       </c>
       <c r="H126" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I126" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E127" s="1">
         <v>4</v>
       </c>
       <c r="F127" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H127" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I127" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D128" s="1">
         <v>5</v>
       </c>
       <c r="E128" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F128" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G128" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I128" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D129" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E129" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F129" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G129" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H129" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I129" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D130" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E130" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F130" s="1">
         <v>5</v>
@@ -8045,451 +8048,451 @@
         <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I130" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D131" s="1">
+        <v>6</v>
+      </c>
+      <c r="E131" s="1">
+        <v>3</v>
+      </c>
+      <c r="F131" s="1">
         <v>5</v>
       </c>
-      <c r="E131" s="1">
-        <v>5</v>
-      </c>
-      <c r="F131" s="1">
-        <v>3</v>
-      </c>
       <c r="G131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I131" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D132" s="1">
         <v>5</v>
       </c>
       <c r="E132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F132" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G132" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H132" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I132" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I132" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D133" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F133" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G133" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H133" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I133" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D134" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E134" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F134" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G134" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H134" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I134" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D135" s="1">
         <v>5</v>
       </c>
       <c r="E135" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F135" s="1">
         <v>5</v>
       </c>
       <c r="G135" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H135" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I135" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D136" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
         <v>4</v>
       </c>
       <c r="F136" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G136" s="1">
         <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I136" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D137" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E137" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F137" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G137" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H137" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I137" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D138" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E138" s="1">
+        <v>0</v>
+      </c>
+      <c r="F138" s="1">
         <v>2</v>
       </c>
-      <c r="F138" s="1">
-        <v>4</v>
-      </c>
       <c r="G138" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H138" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I138" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D139" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E139" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F139" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G139" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H139" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I139" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D140" s="1">
+        <v>5</v>
+      </c>
+      <c r="E140" s="1">
         <v>3</v>
       </c>
-      <c r="E140" s="1">
-        <v>4</v>
-      </c>
       <c r="F140" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G140" s="1">
         <v>4</v>
       </c>
       <c r="H140" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I140" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D141" s="1">
+        <v>3</v>
+      </c>
+      <c r="E141" s="1">
         <v>4</v>
       </c>
-      <c r="E141" s="1">
-        <v>3</v>
-      </c>
       <c r="F141" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G141" s="1">
         <v>4</v>
       </c>
       <c r="H141" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I141" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D142" s="1">
         <v>4</v>
       </c>
       <c r="E142" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F142" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G142" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H142" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I142" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.1749999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D143" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E143" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F143" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G143" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H143" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I143" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D144" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E144" s="1">
         <v>3</v>
       </c>
       <c r="F144" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G144" s="1">
         <v>4</v>
       </c>
       <c r="H144" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I144" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D145" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E145" s="1">
+        <v>3</v>
+      </c>
+      <c r="F145" s="1">
+        <v>3</v>
+      </c>
+      <c r="G145" s="1">
         <v>4</v>
       </c>
-      <c r="F145" s="1">
-        <v>2</v>
-      </c>
-      <c r="G145" s="1">
-        <v>5</v>
-      </c>
       <c r="H145" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I145" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D146" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E146" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F146" s="1">
         <v>2</v>
       </c>
       <c r="G146" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H146" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I146" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D147" s="1">
         <v>3</v>
@@ -8498,25 +8501,25 @@
         <v>3</v>
       </c>
       <c r="F147" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G147" s="1">
         <v>4</v>
       </c>
       <c r="H147" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I147" s="3">
         <v>4.8</v>
       </c>
-      <c r="I147" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B148" s="2">
-        <v>180</v>
+      <c r="B148" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D148" s="1">
         <v>3</v>
@@ -8528,228 +8531,255 @@
         <v>3</v>
       </c>
       <c r="G148" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H148" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I148" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B149" s="2" t="s">
-        <v>216</v>
+      <c r="B149" s="2">
+        <v>180</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D149" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E149" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F149" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G149" s="1">
         <v>3</v>
       </c>
       <c r="H149" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I149" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D150" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E150" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F150" s="1">
         <v>2</v>
       </c>
       <c r="G150" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H150" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I150" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D151" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E151" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F151" s="1">
         <v>2</v>
       </c>
       <c r="G151" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H151" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I151" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D152" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E152" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F152" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G152" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H152" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I152" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D153" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E153" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F153" s="1">
         <v>0</v>
       </c>
       <c r="G153" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H153" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I153" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="9" t="s">
-        <v>239</v>
+      <c r="B154" s="2" t="s">
+        <v>237</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D154" s="1">
         <v>2</v>
       </c>
       <c r="E154" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G154" s="1">
         <v>2</v>
       </c>
       <c r="H154" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I154" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I154" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>2.6375000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D155" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E155" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F155" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G155" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H155" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I155" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D156" s="1">
+        <v>0</v>
+      </c>
+      <c r="E156" s="1">
+        <v>0</v>
+      </c>
+      <c r="F156" s="1">
+        <v>0</v>
+      </c>
+      <c r="G156" s="1">
+        <v>0</v>
+      </c>
+      <c r="H156" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I156" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="157" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B157" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C157" s="5">
+        <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D157" s="1">
         <v>2</v>
       </c>
-      <c r="E156" s="1">
+      <c r="E157" s="1">
         <v>1</v>
       </c>
-      <c r="F156" s="1">
+      <c r="F157" s="1">
         <v>2</v>
       </c>
-      <c r="G156" s="1">
+      <c r="G157" s="1">
         <v>2</v>
       </c>
-      <c r="H156" s="3">
+      <c r="H157" s="3">
         <v>4.3</v>
       </c>
-      <c r="I156" s="3">
+      <c r="I157" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 138 "El campeón"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27437830-5826-439E-8225-4522AFA832CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1C1483-1959-4FB8-88D5-E831DD28B76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="242">
   <si>
     <t>Película</t>
   </si>
@@ -1335,6 +1335,9 @@
   </si>
   <si>
     <t>El país de los sueños</t>
+  </si>
+  <si>
+    <t>El campeón</t>
   </si>
 </sst>
 </file>
@@ -1687,10 +1690,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I157" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I157" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I157">
-    <sortCondition descending="1" ref="C2:C157"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I158" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I158" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I158">
+    <sortCondition descending="1" ref="C2:C158"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4554,7 +4557,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K157"/>
+  <dimension ref="B2:K158"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -7299,7 +7302,7 @@
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B103" s="9" t="s">
+      <c r="B103" s="2" t="s">
         <v>240</v>
       </c>
       <c r="C103" s="5">
@@ -8082,444 +8085,444 @@
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B132" s="2" t="s">
-        <v>163</v>
+      <c r="B132" s="9" t="s">
+        <v>241</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D132" s="1">
         <v>5</v>
       </c>
       <c r="E132" s="1">
+        <v>4</v>
+      </c>
+      <c r="F132" s="1">
         <v>5</v>
       </c>
-      <c r="F132" s="1">
-        <v>3</v>
-      </c>
       <c r="G132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H132" s="3">
         <v>5.5</v>
       </c>
       <c r="I132" s="3">
-        <v>4.8</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D133" s="1">
         <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F133" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G133" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H133" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I133" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I133" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D134" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E134" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F134" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G134" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H134" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I134" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D135" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E135" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F135" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G135" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H135" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I135" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D136" s="1">
         <v>5</v>
       </c>
       <c r="E136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F136" s="1">
         <v>5</v>
       </c>
       <c r="G136" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H136" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I136" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D137" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E137" s="1">
         <v>4</v>
       </c>
       <c r="F137" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G137" s="1">
         <v>5</v>
       </c>
       <c r="H137" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I137" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D138" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E138" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F138" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G138" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H138" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I138" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D139" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E139" s="1">
+        <v>0</v>
+      </c>
+      <c r="F139" s="1">
         <v>2</v>
       </c>
-      <c r="F139" s="1">
-        <v>4</v>
-      </c>
       <c r="G139" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H139" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I139" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D140" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E140" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F140" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G140" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H140" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I140" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D141" s="1">
+        <v>5</v>
+      </c>
+      <c r="E141" s="1">
         <v>3</v>
       </c>
-      <c r="E141" s="1">
-        <v>4</v>
-      </c>
       <c r="F141" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G141" s="1">
         <v>4</v>
       </c>
       <c r="H141" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I141" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D142" s="1">
+        <v>3</v>
+      </c>
+      <c r="E142" s="1">
         <v>4</v>
       </c>
-      <c r="E142" s="1">
-        <v>3</v>
-      </c>
       <c r="F142" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G142" s="1">
         <v>4</v>
       </c>
       <c r="H142" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I142" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D143" s="1">
         <v>4</v>
       </c>
       <c r="E143" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F143" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G143" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H143" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I143" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.1749999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D144" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E144" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F144" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G144" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H144" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I144" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D145" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E145" s="1">
         <v>3</v>
       </c>
       <c r="F145" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G145" s="1">
         <v>4</v>
       </c>
       <c r="H145" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I145" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D146" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E146" s="1">
+        <v>3</v>
+      </c>
+      <c r="F146" s="1">
+        <v>3</v>
+      </c>
+      <c r="G146" s="1">
         <v>4</v>
       </c>
-      <c r="F146" s="1">
-        <v>2</v>
-      </c>
-      <c r="G146" s="1">
-        <v>5</v>
-      </c>
       <c r="H146" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I146" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D147" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F147" s="1">
         <v>2</v>
       </c>
       <c r="G147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H147" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I147" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D148" s="1">
         <v>3</v>
@@ -8528,25 +8531,25 @@
         <v>3</v>
       </c>
       <c r="F148" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G148" s="1">
         <v>4</v>
       </c>
       <c r="H148" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I148" s="3">
         <v>4.8</v>
       </c>
-      <c r="I148" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B149" s="2">
-        <v>180</v>
+      <c r="B149" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D149" s="1">
         <v>3</v>
@@ -8558,228 +8561,255 @@
         <v>3</v>
       </c>
       <c r="G149" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H149" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I149" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B150" s="2" t="s">
-        <v>216</v>
+      <c r="B150" s="2">
+        <v>180</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D150" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E150" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F150" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G150" s="1">
         <v>3</v>
       </c>
       <c r="H150" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I150" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D151" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E151" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F151" s="1">
         <v>2</v>
       </c>
       <c r="G151" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H151" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I151" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D152" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E152" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="1">
         <v>2</v>
       </c>
       <c r="G152" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H152" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I152" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D153" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E153" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F153" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G153" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H153" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I153" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D154" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E154" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F154" s="1">
         <v>0</v>
       </c>
       <c r="G154" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H154" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I154" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D155" s="1">
         <v>2</v>
       </c>
       <c r="E155" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F155" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G155" s="1">
         <v>2</v>
       </c>
       <c r="H155" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I155" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I155" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>2.6375000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D156" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E156" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F156" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G156" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H156" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I156" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D157" s="1">
+        <v>0</v>
+      </c>
+      <c r="E157" s="1">
+        <v>0</v>
+      </c>
+      <c r="F157" s="1">
+        <v>0</v>
+      </c>
+      <c r="G157" s="1">
+        <v>0</v>
+      </c>
+      <c r="H157" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I157" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="158" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B158" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C158" s="5">
+        <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D157" s="1">
+      <c r="D158" s="1">
         <v>2</v>
       </c>
-      <c r="E157" s="1">
+      <c r="E158" s="1">
         <v>1</v>
       </c>
-      <c r="F157" s="1">
+      <c r="F158" s="1">
         <v>2</v>
       </c>
-      <c r="G157" s="1">
+      <c r="G158" s="1">
         <v>2</v>
       </c>
-      <c r="H157" s="3">
+      <c r="H158" s="3">
         <v>4.3</v>
       </c>
-      <c r="I157" s="3">
+      <c r="I158" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 140 "La desconocida"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7DD024-F9CC-4F13-A7B4-58BEF4905EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D3EF4F-04DE-48AA-87F7-711D9899EE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="244">
   <si>
     <t>Película</t>
   </si>
@@ -1341,6 +1341,9 @@
   </si>
   <si>
     <t>Escape</t>
+  </si>
+  <si>
+    <t>La desconocida</t>
   </si>
 </sst>
 </file>
@@ -1693,10 +1696,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I159" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I159" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I159">
-    <sortCondition descending="1" ref="C2:C159"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I160" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I160" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I160">
+    <sortCondition descending="1" ref="C2:C160"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4560,7 +4563,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K159"/>
+  <dimension ref="B2:K160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -7899,7 +7902,7 @@
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B125" s="9" t="s">
+      <c r="B125" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C125" s="5">
@@ -8277,309 +8280,309 @@
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B139" s="2" t="s">
-        <v>161</v>
+      <c r="B139" s="9" t="s">
+        <v>243</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5</v>
       </c>
       <c r="D139" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E139" s="1">
         <v>4</v>
       </c>
       <c r="F139" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G139" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H139" s="3">
         <v>5.5</v>
       </c>
       <c r="I139" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D140" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E140" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F140" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G140" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H140" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I140" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D141" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E141" s="1">
+        <v>0</v>
+      </c>
+      <c r="F141" s="1">
         <v>2</v>
       </c>
-      <c r="F141" s="1">
-        <v>4</v>
-      </c>
       <c r="G141" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H141" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I141" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D142" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E142" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F142" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G142" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H142" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I142" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D143" s="1">
+        <v>5</v>
+      </c>
+      <c r="E143" s="1">
         <v>3</v>
       </c>
-      <c r="E143" s="1">
-        <v>4</v>
-      </c>
       <c r="F143" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G143" s="1">
         <v>4</v>
       </c>
       <c r="H143" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I143" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.3</v>
+        <v>4.3125</v>
       </c>
       <c r="D144" s="1">
+        <v>3</v>
+      </c>
+      <c r="E144" s="1">
         <v>4</v>
       </c>
-      <c r="E144" s="1">
-        <v>3</v>
-      </c>
       <c r="F144" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G144" s="1">
         <v>4</v>
       </c>
       <c r="H144" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I144" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D145" s="1">
         <v>4</v>
       </c>
       <c r="E145" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F145" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G145" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H145" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I145" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.1749999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D146" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E146" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F146" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G146" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H146" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I146" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E147" s="1">
         <v>3</v>
       </c>
       <c r="F147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G147" s="1">
         <v>4</v>
       </c>
       <c r="H147" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I147" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D148" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E148" s="1">
+        <v>3</v>
+      </c>
+      <c r="F148" s="1">
+        <v>3</v>
+      </c>
+      <c r="G148" s="1">
         <v>4</v>
       </c>
-      <c r="F148" s="1">
-        <v>2</v>
-      </c>
-      <c r="G148" s="1">
-        <v>5</v>
-      </c>
       <c r="H148" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I148" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D149" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E149" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F149" s="1">
         <v>2</v>
       </c>
       <c r="G149" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H149" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I149" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D150" s="1">
         <v>3</v>
@@ -8588,25 +8591,25 @@
         <v>3</v>
       </c>
       <c r="F150" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G150" s="1">
         <v>4</v>
       </c>
       <c r="H150" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I150" s="3">
         <v>4.8</v>
       </c>
-      <c r="I150" s="3">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B151" s="2">
-        <v>180</v>
+      <c r="B151" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D151" s="1">
         <v>3</v>
@@ -8618,228 +8621,255 @@
         <v>3</v>
       </c>
       <c r="G151" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H151" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I151" s="3">
         <v>4.3</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B152" s="2" t="s">
-        <v>216</v>
+      <c r="B152" s="2">
+        <v>180</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D152" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E152" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F152" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G152" s="1">
         <v>3</v>
       </c>
       <c r="H152" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I152" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D153" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E153" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F153" s="1">
         <v>2</v>
       </c>
       <c r="G153" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H153" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I153" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D154" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E154" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F154" s="1">
         <v>2</v>
       </c>
       <c r="G154" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H154" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I154" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D155" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E155" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F155" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G155" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H155" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I155" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D156" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E156" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F156" s="1">
         <v>0</v>
       </c>
       <c r="G156" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H156" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I156" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D157" s="1">
         <v>2</v>
       </c>
       <c r="E157" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F157" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G157" s="1">
         <v>2</v>
       </c>
       <c r="H157" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I157" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I157" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>2.6375000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D158" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E158" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F158" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G158" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H158" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I158" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D159" s="1">
+        <v>0</v>
+      </c>
+      <c r="E159" s="1">
+        <v>0</v>
+      </c>
+      <c r="F159" s="1">
+        <v>0</v>
+      </c>
+      <c r="G159" s="1">
+        <v>0</v>
+      </c>
+      <c r="H159" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I159" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="160" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B160" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C160" s="5">
+        <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D160" s="1">
         <v>2</v>
       </c>
-      <c r="E159" s="1">
+      <c r="E160" s="1">
         <v>1</v>
       </c>
-      <c r="F159" s="1">
+      <c r="F160" s="1">
         <v>2</v>
       </c>
-      <c r="G159" s="1">
+      <c r="G160" s="1">
         <v>2</v>
       </c>
-      <c r="H159" s="3">
+      <c r="H160" s="3">
         <v>4.3</v>
       </c>
-      <c r="I159" s="3">
+      <c r="I160" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 141 "Campeones" & "Encurtido en el tiempo"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D3EF4F-04DE-48AA-87F7-711D9899EE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0B6D85-9E73-4C90-8E7D-E6366855CCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="246">
   <si>
     <t>Película</t>
   </si>
@@ -1344,6 +1344,12 @@
   </si>
   <si>
     <t>La desconocida</t>
+  </si>
+  <si>
+    <t>Campeones</t>
+  </si>
+  <si>
+    <t>Encurtido en el tiempo</t>
   </si>
 </sst>
 </file>
@@ -1696,10 +1702,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I160" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I160" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I160">
-    <sortCondition descending="1" ref="C2:C160"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I162" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I162" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I162">
+    <sortCondition descending="1" ref="C2:C162"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4563,7 +4569,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K160"/>
+  <dimension ref="B2:K162"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5823,18 +5829,18 @@
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="2" t="s">
-        <v>131</v>
+      <c r="B48" s="9" t="s">
+        <v>244</v>
       </c>
       <c r="C48" s="5">
         <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
-        <v>7.4124999999999996</v>
+        <v>7.4125000000000005</v>
       </c>
       <c r="D48" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E48" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F48" s="1">
         <v>8</v>
@@ -5843,25 +5849,25 @@
         <v>8</v>
       </c>
       <c r="H48" s="3">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="I48" s="3">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>220</v>
+        <v>131</v>
       </c>
       <c r="C49" s="5">
         <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
-        <v>7.3624999999999998</v>
+        <v>7.4124999999999996</v>
       </c>
       <c r="D49" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E49" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F49" s="1">
         <v>8</v>
@@ -5870,46 +5876,46 @@
         <v>8</v>
       </c>
       <c r="H49" s="3">
+        <v>7.4</v>
+      </c>
+      <c r="I49" s="3">
         <v>6.5</v>
-      </c>
-      <c r="I49" s="3">
-        <v>5.9</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>175</v>
+        <v>220</v>
       </c>
       <c r="C50" s="5">
         <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
-        <v>7.3624999999999989</v>
+        <v>7.3624999999999998</v>
       </c>
       <c r="D50" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F50" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G50" s="1">
         <v>8</v>
       </c>
       <c r="H50" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I50" s="3">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>52</v>
+        <v>175</v>
       </c>
       <c r="C51" s="5">
         <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
-        <v>7.3500000000000005</v>
+        <v>7.3624999999999989</v>
       </c>
       <c r="D51" s="1">
         <v>8</v>
@@ -5918,25 +5924,25 @@
         <v>8</v>
       </c>
       <c r="F51" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G51" s="1">
         <v>8</v>
       </c>
       <c r="H51" s="3">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="I51" s="3">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>165</v>
+        <v>52</v>
       </c>
       <c r="C52" s="5">
         <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
-        <v>7.3249999999999993</v>
+        <v>7.3500000000000005</v>
       </c>
       <c r="D52" s="1">
         <v>8</v>
@@ -5948,109 +5954,109 @@
         <v>8</v>
       </c>
       <c r="G52" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H52" s="3">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="I52" s="3">
-        <v>6</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>224</v>
+        <v>165</v>
       </c>
       <c r="C53" s="5">
         <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
-        <v>7.3125</v>
+        <v>7.3249999999999993</v>
       </c>
       <c r="D53" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E53" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F53" s="1">
         <v>8</v>
       </c>
       <c r="G53" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H53" s="3">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="I53" s="3">
-        <v>6.7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>111</v>
+        <v>224</v>
       </c>
       <c r="C54" s="5">
         <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
-        <v>7.3</v>
+        <v>7.3125</v>
       </c>
       <c r="D54" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E54" s="1">
         <v>7</v>
       </c>
       <c r="F54" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G54" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H54" s="3">
-        <v>6.5</v>
+        <v>7.4</v>
       </c>
       <c r="I54" s="3">
-        <v>5.4</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C55" s="5">
         <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
-        <v>7.2750000000000004</v>
+        <v>7.3</v>
       </c>
       <c r="D55" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E55" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F55" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G55" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H55" s="3">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="I55" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="C56" s="5">
         <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D56" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E56" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F56" s="1">
         <v>8</v>
@@ -6059,22 +6065,22 @@
         <v>8</v>
       </c>
       <c r="H56" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="I56" s="3">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>225</v>
+        <v>181</v>
       </c>
       <c r="C57" s="5">
         <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
-        <v>7.2624999999999993</v>
+        <v>7.2750000000000004</v>
       </c>
       <c r="D57" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E57" s="1">
         <v>7</v>
@@ -6086,25 +6092,25 @@
         <v>8</v>
       </c>
       <c r="H57" s="3">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="I57" s="3">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>147</v>
+        <v>225</v>
       </c>
       <c r="C58" s="5">
         <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
-        <v>7.2374999999999998</v>
+        <v>7.2624999999999993</v>
       </c>
       <c r="D58" s="1">
         <v>7</v>
       </c>
       <c r="E58" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F58" s="1">
         <v>8</v>
@@ -6113,127 +6119,127 @@
         <v>8</v>
       </c>
       <c r="H58" s="3">
-        <v>6</v>
+        <v>7.3</v>
       </c>
       <c r="I58" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="C59" s="5">
         <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
-        <v>7.2250000000000005</v>
+        <v>7.2374999999999998</v>
       </c>
       <c r="D59" s="1">
         <v>7</v>
       </c>
       <c r="E59" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F59" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G59" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H59" s="3">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="I59" s="3">
-        <v>7.6</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C60" s="5">
         <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
-        <v>7.2125000000000004</v>
+        <v>7.2250000000000005</v>
       </c>
       <c r="D60" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E60" s="1">
         <v>7</v>
       </c>
       <c r="F60" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G60" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H60" s="3">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="I60" s="3">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>146</v>
+        <v>65</v>
       </c>
       <c r="C61" s="5">
         <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
-        <v>7.2124999999999995</v>
+        <v>7.2125000000000004</v>
       </c>
       <c r="D61" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E61" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F61" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G61" s="1">
         <v>8</v>
       </c>
       <c r="H61" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I61" s="3">
         <v>6.3</v>
-      </c>
-      <c r="I61" s="3">
-        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="C62" s="5">
         <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
-        <v>7.1999999999999993</v>
+        <v>7.2124999999999995</v>
       </c>
       <c r="D62" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E62" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F62" s="1">
         <v>9</v>
       </c>
       <c r="G62" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H62" s="3">
         <v>6.3</v>
       </c>
       <c r="I62" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="C63" s="5">
         <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
-        <v>7.1499999999999995</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D63" s="1">
         <v>8</v>
@@ -6242,217 +6248,217 @@
         <v>7</v>
       </c>
       <c r="F63" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G63" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H63" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I63" s="3">
-        <v>6.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="C64" s="5">
         <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
-        <v>7.1375000000000011</v>
+        <v>7.1499999999999995</v>
       </c>
       <c r="D64" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G64" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H64" s="3">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="I64" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="C65" s="5">
         <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
-        <v>7.1250000000000009</v>
+        <v>7.1375000000000011</v>
       </c>
       <c r="D65" s="1">
         <v>7</v>
       </c>
       <c r="E65" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F65" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G65" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H65" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I65" s="3">
         <v>6.7</v>
-      </c>
-      <c r="I65" s="3">
-        <v>6.6</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C66" s="5">
         <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
-        <v>7.125</v>
+        <v>7.1250000000000009</v>
       </c>
       <c r="D66" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G66" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H66" s="3">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="I66" s="3">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>133</v>
+        <v>39</v>
       </c>
       <c r="C67" s="5">
         <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
-        <v>7.0875000000000004</v>
+        <v>7.125</v>
       </c>
       <c r="D67" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E67" s="1">
         <v>8</v>
       </c>
       <c r="F67" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G67" s="1">
         <v>7</v>
       </c>
       <c r="H67" s="3">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="I67" s="3">
-        <v>6.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="C68" s="5">
         <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
-        <v>7.0750000000000011</v>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D68" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E68" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F68" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G68" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H68" s="3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="I68" s="3">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C69" s="5">
         <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D69" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E69" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" s="1">
         <v>8</v>
       </c>
       <c r="G69" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H69" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I69" s="3">
         <v>6.2</v>
-      </c>
-      <c r="I69" s="3">
-        <v>5.2</v>
       </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
-        <v>7.0750000000000002</v>
+        <v>7.0750000000000011</v>
       </c>
       <c r="D70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F70" s="1">
         <v>8</v>
       </c>
       <c r="G70" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H70" s="3">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="I70" s="3">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D71" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E71" s="1">
         <v>7</v>
@@ -6461,55 +6467,55 @@
         <v>8</v>
       </c>
       <c r="G71" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H71" s="3">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="I71" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
-        <v>7.0749999999999993</v>
+        <v>7.0750000000000002</v>
       </c>
       <c r="D72" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E72" s="1">
         <v>7</v>
       </c>
       <c r="F72" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G72" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H72" s="3">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="I72" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
-        <v>7.05</v>
+        <v>7.0749999999999993</v>
       </c>
       <c r="D73" s="1">
         <v>8</v>
       </c>
       <c r="E73" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F73" s="1">
         <v>7</v>
@@ -6518,46 +6524,46 @@
         <v>8</v>
       </c>
       <c r="H73" s="3">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="I73" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>221</v>
+        <v>176</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
-        <v>7.0250000000000004</v>
+        <v>7.05</v>
       </c>
       <c r="D74" s="1">
         <v>8</v>
       </c>
       <c r="E74" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F74" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G74" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H74" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="I74" s="3">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
-        <v>95</v>
+        <v>221</v>
       </c>
       <c r="C75" s="5">
         <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
-        <v>6.9375</v>
+        <v>7.0250000000000004</v>
       </c>
       <c r="D75" s="1">
         <v>8</v>
@@ -6569,22 +6575,22 @@
         <v>8</v>
       </c>
       <c r="G75" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H75" s="3">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="I75" s="3">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="2" t="s">
-        <v>164</v>
+        <v>95</v>
       </c>
       <c r="C76" s="5">
         <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
-        <v>6.9124999999999996</v>
+        <v>6.9375</v>
       </c>
       <c r="D76" s="1">
         <v>8</v>
@@ -6596,72 +6602,72 @@
         <v>8</v>
       </c>
       <c r="G76" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H76" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="I76" s="3">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C77" s="5">
         <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
-        <v>6.8999999999999995</v>
+        <v>6.9124999999999996</v>
       </c>
       <c r="D77" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E77" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F77" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G77" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H77" s="3">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="I77" s="3">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
-        <v>88</v>
+        <v>157</v>
       </c>
       <c r="C78" s="5">
         <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
-        <v>6.8624999999999989</v>
+        <v>6.8999999999999995</v>
       </c>
       <c r="D78" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E78" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G78" s="1">
         <v>8</v>
       </c>
       <c r="H78" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I78" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" s="2" t="s">
-        <v>184</v>
+        <v>88</v>
       </c>
       <c r="C79" s="5">
         <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
@@ -6688,179 +6694,179 @@
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="C80" s="5">
         <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
-        <v>6.85</v>
+        <v>6.8624999999999989</v>
       </c>
       <c r="D80" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E80" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F80" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G80" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H80" s="3">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="I80" s="3">
-        <v>6.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="2" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="C81" s="5">
         <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
-        <v>6.7999999999999989</v>
+        <v>6.85</v>
       </c>
       <c r="D81" s="1">
         <v>8</v>
       </c>
       <c r="E81" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G81" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H81" s="3">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="I81" s="3">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="2" t="s">
-        <v>57</v>
+        <v>196</v>
       </c>
       <c r="C82" s="5">
         <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
-        <v>6.6999999999999993</v>
+        <v>6.7999999999999989</v>
       </c>
       <c r="D82" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E82" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F82" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G82" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H82" s="3">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="I82" s="3">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="2" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="C83" s="5">
         <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
-        <v>6.6875</v>
+        <v>6.6999999999999993</v>
       </c>
       <c r="D83" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E83" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G83" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H83" s="3">
-        <v>5.5</v>
+        <v>7.9</v>
       </c>
       <c r="I83" s="3">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
       <c r="C84" s="5">
         <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
-        <v>6.6375000000000002</v>
+        <v>6.6875</v>
       </c>
       <c r="D84" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1">
         <v>7</v>
       </c>
       <c r="F84" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G84" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H84" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I84" s="3">
-        <v>6.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C85" s="5">
         <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
-        <v>6.6374999999999993</v>
+        <v>6.6375000000000002</v>
       </c>
       <c r="D85" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E85" s="1">
         <v>7</v>
       </c>
       <c r="F85" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G85" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H85" s="3">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="I85" s="3">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="2" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="C86" s="5">
         <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6374999999999993</v>
       </c>
       <c r="D86" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E86" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F86" s="1">
         <v>8</v>
@@ -6869,106 +6875,106 @@
         <v>7</v>
       </c>
       <c r="H86" s="3">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I86" s="3">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D87" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E87" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G87" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H87" s="3">
         <v>6.3</v>
       </c>
       <c r="I87" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D88" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E88" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F88" s="1">
         <v>7</v>
       </c>
       <c r="G88" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H88" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I88" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D89" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E89" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" s="1">
         <v>7</v>
       </c>
       <c r="G89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H89" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I89" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D90" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F90" s="1">
         <v>7</v>
@@ -6977,76 +6983,76 @@
         <v>6</v>
       </c>
       <c r="H90" s="3">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="I90" s="3">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D91" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" s="1">
         <v>7</v>
       </c>
       <c r="G91" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H91" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I91" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D92" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F92" s="1">
         <v>7</v>
       </c>
       <c r="G92" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H92" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I92" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D93" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E93" s="1">
         <v>6</v>
@@ -7058,25 +7064,25 @@
         <v>7</v>
       </c>
       <c r="H93" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I93" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D94" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" s="1">
         <v>7</v>
@@ -7085,79 +7091,79 @@
         <v>7</v>
       </c>
       <c r="H94" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I94" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D95" s="1">
         <v>7</v>
       </c>
       <c r="E95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F95" s="1">
         <v>7</v>
       </c>
       <c r="G95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I95" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
         <v>6.35</v>
       </c>
       <c r="D96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G96" s="1">
         <v>6</v>
       </c>
       <c r="H96" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I96" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F97" s="1">
         <v>6</v>
@@ -7166,42 +7172,42 @@
         <v>6</v>
       </c>
       <c r="H97" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I97" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E98" s="1">
         <v>6</v>
       </c>
       <c r="F98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H98" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I98" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
@@ -7211,139 +7217,139 @@
         <v>6</v>
       </c>
       <c r="E99" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I99" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D100" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F100" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G100" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H100" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I100" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D101" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E101" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F101" s="1">
         <v>8</v>
       </c>
       <c r="G101" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H101" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I101" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D102" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E102" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F102" s="1">
         <v>8</v>
       </c>
       <c r="G102" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H102" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I102" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>6.1250000000000009</v>
+        <v>6.15</v>
       </c>
       <c r="D103" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E103" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F103" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G103" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H103" s="3">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="I103" s="3">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>158</v>
+        <v>240</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>6.0874999999999995</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D104" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E104" s="1">
         <v>7</v>
@@ -7355,46 +7361,46 @@
         <v>7</v>
       </c>
       <c r="H104" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I104" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D105" s="1">
         <v>7</v>
       </c>
       <c r="E105" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F105" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G105" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H105" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I105" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
@@ -7403,25 +7409,25 @@
         <v>6</v>
       </c>
       <c r="F106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G106" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H106" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I106" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D107" s="1">
         <v>7</v>
@@ -7433,49 +7439,49 @@
         <v>7</v>
       </c>
       <c r="G107" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H107" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I107" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
         <v>6.05</v>
       </c>
       <c r="D108" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E108" s="1">
         <v>6</v>
       </c>
       <c r="F108" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G108" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H108" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I108" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D109" s="1">
         <v>6</v>
@@ -7484,133 +7490,133 @@
         <v>6</v>
       </c>
       <c r="F109" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G109" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H109" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I109" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D110" s="1">
         <v>6</v>
       </c>
       <c r="E110" s="1">
+        <v>6</v>
+      </c>
+      <c r="F110" s="1">
+        <v>8</v>
+      </c>
+      <c r="G110" s="1">
         <v>5</v>
       </c>
-      <c r="F110" s="1">
-        <v>6</v>
-      </c>
-      <c r="G110" s="1">
-        <v>6</v>
-      </c>
       <c r="H110" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I110" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D111" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E111" s="1">
         <v>5</v>
       </c>
       <c r="F111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G111" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H111" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I111" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D112" s="1">
         <v>7</v>
       </c>
       <c r="E112" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F112" s="1">
         <v>5</v>
       </c>
       <c r="G112" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H112" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I112" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
       </c>
       <c r="E113" s="1">
+        <v>6</v>
+      </c>
+      <c r="F113" s="1">
         <v>5</v>
       </c>
-      <c r="F113" s="1">
-        <v>4</v>
-      </c>
       <c r="G113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H113" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I113" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D114" s="1">
         <v>7</v>
@@ -7622,37 +7628,37 @@
         <v>4</v>
       </c>
       <c r="G114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I114" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D115" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E115" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F115" s="1">
+        <v>4</v>
+      </c>
+      <c r="G115" s="1">
         <v>5</v>
       </c>
-      <c r="G115" s="1">
-        <v>6</v>
-      </c>
       <c r="H115" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I115" s="3">
         <v>6.4</v>
@@ -7660,50 +7666,50 @@
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D116" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E116" s="1">
+        <v>3</v>
+      </c>
+      <c r="F116" s="1">
         <v>5</v>
       </c>
-      <c r="F116" s="1">
-        <v>6</v>
-      </c>
       <c r="G116" s="1">
         <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I116" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D117" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E117" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F117" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H117" s="3">
         <v>5.8</v>
@@ -7714,26 +7720,26 @@
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.5375000000000005</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D118" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E118" s="1">
+        <v>6</v>
+      </c>
+      <c r="F118" s="1">
+        <v>8</v>
+      </c>
+      <c r="G118" s="1">
         <v>5</v>
       </c>
-      <c r="F118" s="1">
-        <v>6</v>
-      </c>
-      <c r="G118" s="1">
-        <v>6</v>
-      </c>
       <c r="H118" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I118" s="3">
         <v>4.9000000000000004</v>
@@ -7741,17 +7747,17 @@
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>166</v>
+        <v>229</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D119" s="1">
         <v>6</v>
       </c>
       <c r="E119" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F119" s="1">
         <v>6</v>
@@ -7760,46 +7766,46 @@
         <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I119" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B120" s="2" t="s">
-        <v>191</v>
+      <c r="B120" s="9" t="s">
+        <v>245</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D120" s="1">
+        <v>6</v>
+      </c>
+      <c r="E120" s="1">
         <v>5</v>
       </c>
-      <c r="E120" s="1">
-        <v>6</v>
-      </c>
       <c r="F120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="I120" s="3">
-        <v>5.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>228</v>
+        <v>166</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.3875000000000011</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D121" s="1">
         <v>6</v>
@@ -7814,49 +7820,49 @@
         <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="I121" s="3">
-        <v>3.7</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E122" s="1">
+        <v>6</v>
+      </c>
+      <c r="F122" s="1">
         <v>5</v>
       </c>
-      <c r="F122" s="1">
-        <v>6</v>
-      </c>
       <c r="G122" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H122" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I122" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>190</v>
+        <v>228</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.375</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D123" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E123" s="1">
         <v>6</v>
@@ -7868,127 +7874,127 @@
         <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I123" s="3">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.2875000000000005</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E124" s="1">
         <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G124" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H124" s="3">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="I124" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>242</v>
+        <v>190</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.25</v>
+        <v>5.375</v>
       </c>
       <c r="D125" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F125" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H125" s="3">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="I125" s="3">
-        <v>5.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.2</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D126" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E126" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G126" s="1">
         <v>5</v>
       </c>
       <c r="H126" s="3">
-        <v>7.1</v>
+        <v>6.1</v>
       </c>
       <c r="I126" s="3">
-        <v>6.4</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>74</v>
+        <v>242</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.1875</v>
+        <v>5.25</v>
       </c>
       <c r="D127" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E127" s="1">
         <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H127" s="3">
-        <v>4.5</v>
+        <v>5.7</v>
       </c>
       <c r="I127" s="3">
-        <v>3.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.1124999999999998</v>
+        <v>5.2</v>
       </c>
       <c r="D128" s="1">
         <v>6</v>
@@ -7997,139 +8003,139 @@
         <v>4</v>
       </c>
       <c r="F128" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G128" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>5.9</v>
+        <v>7.1</v>
       </c>
       <c r="I128" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>223</v>
+        <v>74</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1875</v>
       </c>
       <c r="D129" s="1">
+        <v>7</v>
+      </c>
+      <c r="E129" s="1">
         <v>5</v>
       </c>
-      <c r="E129" s="1">
-        <v>4</v>
-      </c>
       <c r="F129" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G129" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H129" s="3">
-        <v>6.3</v>
+        <v>4.5</v>
       </c>
       <c r="I129" s="3">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>5.05</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D130" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E130" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F130" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G130" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I130" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>4.9875000000000007</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D131" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E131" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F131" s="1">
         <v>5</v>
       </c>
       <c r="G131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H131" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.3</v>
       </c>
       <c r="I131" s="3">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>169</v>
+        <v>21</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>4.9874999999999998</v>
+        <v>5.05</v>
       </c>
       <c r="D132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E132" s="1">
         <v>3</v>
       </c>
       <c r="F132" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G132" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H132" s="3">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="I132" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>241</v>
+        <v>203</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>4.9249999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D133" s="1">
+        <v>7</v>
+      </c>
+      <c r="E133" s="1">
         <v>5</v>
-      </c>
-      <c r="E133" s="1">
-        <v>4</v>
       </c>
       <c r="F133" s="1">
         <v>5</v>
@@ -8138,304 +8144,304 @@
         <v>6</v>
       </c>
       <c r="H133" s="3">
-        <v>5.5</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I133" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D134" s="1">
+        <v>6</v>
+      </c>
+      <c r="E134" s="1">
+        <v>3</v>
+      </c>
+      <c r="F134" s="1">
         <v>5</v>
       </c>
-      <c r="E134" s="1">
-        <v>5</v>
-      </c>
-      <c r="F134" s="1">
-        <v>3</v>
-      </c>
       <c r="G134" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H134" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I134" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>162</v>
+        <v>241</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.7875000000000005</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D135" s="1">
         <v>5</v>
       </c>
       <c r="E135" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F135" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G135" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="I135" s="3">
-        <v>3.7</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>213</v>
+        <v>163</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.6124999999999998</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
+        <v>5</v>
+      </c>
+      <c r="F136" s="1">
         <v>3</v>
       </c>
-      <c r="F136" s="1">
-        <v>4</v>
-      </c>
       <c r="G136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>6.7</v>
+        <v>5.5</v>
       </c>
       <c r="I136" s="3">
-        <v>5.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.5999999999999996</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D137" s="1">
         <v>5</v>
       </c>
       <c r="E137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G137" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H137" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.8</v>
       </c>
       <c r="I137" s="3">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>135</v>
+        <v>213</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>4.5874999999999995</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D138" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E138" s="1">
+        <v>3</v>
+      </c>
+      <c r="F138" s="1">
         <v>4</v>
       </c>
-      <c r="F138" s="1">
-        <v>5</v>
-      </c>
       <c r="G138" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H138" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I138" s="3">
-        <v>3.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B139" s="9" t="s">
-        <v>243</v>
+      <c r="B139" s="2" t="s">
+        <v>154</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D139" s="1">
         <v>5</v>
       </c>
       <c r="E139" s="1">
+        <v>5</v>
+      </c>
+      <c r="F139" s="1">
+        <v>5</v>
+      </c>
+      <c r="G139" s="1">
+        <v>3</v>
+      </c>
+      <c r="H139" s="3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I139" s="3">
         <v>4</v>
-      </c>
-      <c r="F139" s="1">
-        <v>3</v>
-      </c>
-      <c r="G139" s="1">
-        <v>4</v>
-      </c>
-      <c r="H139" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I139" s="3">
-        <v>5</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D140" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E140" s="1">
         <v>4</v>
       </c>
       <c r="F140" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G140" s="1">
         <v>5</v>
       </c>
       <c r="H140" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I140" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>114</v>
+        <v>243</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.4124999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="D141" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E141" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F141" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G141" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H141" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I141" s="3">
-        <v>7.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>207</v>
+        <v>161</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D142" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E142" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F142" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G142" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H142" s="3">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="I142" s="3">
-        <v>4.7</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.3374999999999995</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D143" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E143" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F143" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H143" s="3">
-        <v>5.9</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I143" s="3">
-        <v>4.9000000000000004</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>173</v>
+        <v>207</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.3125</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D144" s="1">
         <v>3</v>
       </c>
       <c r="E144" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F144" s="1">
         <v>4</v>
       </c>
       <c r="G144" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H144" s="3">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="I144" s="3">
         <v>4.7</v>
@@ -8443,14 +8449,14 @@
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>212</v>
+        <v>150</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.3</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D145" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E145" s="1">
         <v>3</v>
@@ -8462,181 +8468,181 @@
         <v>4</v>
       </c>
       <c r="H145" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I145" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3125</v>
       </c>
       <c r="D146" s="1">
+        <v>3</v>
+      </c>
+      <c r="E146" s="1">
         <v>4</v>
       </c>
-      <c r="E146" s="1">
-        <v>2</v>
-      </c>
       <c r="F146" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G146" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H146" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.4</v>
       </c>
       <c r="I146" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>236</v>
+        <v>212</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.1749999999999998</v>
+        <v>4.3</v>
       </c>
       <c r="D147" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E147" s="1">
         <v>3</v>
       </c>
       <c r="F147" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G147" s="1">
         <v>4</v>
       </c>
       <c r="H147" s="3">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="I147" s="3">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>233</v>
+        <v>167</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.1625000000000005</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D148" s="1">
         <v>4</v>
       </c>
       <c r="E148" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F148" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G148" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H148" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I148" s="3">
-        <v>4.7</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>68</v>
+        <v>236</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D149" s="1">
         <v>5</v>
       </c>
       <c r="E149" s="1">
+        <v>3</v>
+      </c>
+      <c r="F149" s="1">
         <v>4</v>
       </c>
-      <c r="F149" s="1">
-        <v>2</v>
-      </c>
       <c r="G149" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H149" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="I149" s="3">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D150" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E150" s="1">
         <v>3</v>
       </c>
       <c r="F150" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G150" s="1">
         <v>4</v>
       </c>
       <c r="H150" s="3">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="I150" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>199</v>
+        <v>68</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>3.7375000000000003</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D151" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E151" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F151" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G151" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H151" s="3">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="I151" s="3">
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B152" s="2">
-        <v>180</v>
+      <c r="B152" s="2" t="s">
+        <v>218</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>3.5625000000000004</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D152" s="1">
         <v>3</v>
@@ -8645,82 +8651,82 @@
         <v>3</v>
       </c>
       <c r="F152" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G152" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H152" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I152" s="3">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>3.5375000000000005</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D153" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E153" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F153" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G153" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H153" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I153" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="2" t="s">
-        <v>189</v>
+      <c r="B154" s="2">
+        <v>180</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D154" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E154" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F154" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G154" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H154" s="3">
-        <v>5.8</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I154" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>3.2749999999999995</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D155" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E155" s="1">
         <v>2</v>
@@ -8732,46 +8738,46 @@
         <v>3</v>
       </c>
       <c r="H155" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I155" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>2.9124999999999996</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D156" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E156" s="1">
         <v>1</v>
       </c>
       <c r="F156" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G156" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H156" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I156" s="3">
-        <v>5.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>237</v>
+        <v>194</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>2.8125</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D157" s="1">
         <v>2</v>
@@ -8780,79 +8786,79 @@
         <v>2</v>
       </c>
       <c r="F157" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G157" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H157" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="I157" s="3">
-        <v>5.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>239</v>
+        <v>155</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>2.7625000000000002</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D158" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="1">
         <v>1</v>
       </c>
       <c r="F158" s="1">
+        <v>0</v>
+      </c>
+      <c r="G158" s="1">
         <v>1</v>
       </c>
-      <c r="G158" s="1">
-        <v>2</v>
-      </c>
       <c r="H158" s="3">
-        <v>5.5</v>
+        <v>6.7</v>
       </c>
       <c r="I158" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>174</v>
+        <v>237</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>2.6375000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D159" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E159" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F159" s="1">
         <v>0</v>
       </c>
       <c r="G159" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H159" s="3">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
       <c r="I159" s="3">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>2.5125000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D160" s="1">
         <v>2</v>
@@ -8861,15 +8867,69 @@
         <v>1</v>
       </c>
       <c r="F160" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G160" s="1">
         <v>2</v>
       </c>
       <c r="H160" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I160" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="161" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B161" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C161" s="5">
+        <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D161" s="1">
+        <v>0</v>
+      </c>
+      <c r="E161" s="1">
+        <v>0</v>
+      </c>
+      <c r="F161" s="1">
+        <v>0</v>
+      </c>
+      <c r="G161" s="1">
+        <v>0</v>
+      </c>
+      <c r="H161" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I161" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="162" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B162" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C162" s="5">
+        <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
+        <v>2.5125000000000002</v>
+      </c>
+      <c r="D162" s="1">
+        <v>2</v>
+      </c>
+      <c r="E162" s="1">
+        <v>1</v>
+      </c>
+      <c r="F162" s="1">
+        <v>2</v>
+      </c>
+      <c r="G162" s="1">
+        <v>2</v>
+      </c>
+      <c r="H162" s="3">
         <v>4.3</v>
       </c>
-      <c r="I160" s="3">
+      <c r="I162" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 142 "La leyenda de Tarzán"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0B6D85-9E73-4C90-8E7D-E6366855CCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7995AC5-21DE-454D-BBD5-887D265ED830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="247">
   <si>
     <t>Película</t>
   </si>
@@ -1350,6 +1350,9 @@
   </si>
   <si>
     <t>Encurtido en el tiempo</t>
+  </si>
+  <si>
+    <t>La leyenda de Tarzán</t>
   </si>
 </sst>
 </file>
@@ -1702,10 +1705,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I162" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I162" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I162">
-    <sortCondition descending="1" ref="C2:C162"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I163" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I163" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I163">
+    <sortCondition descending="1" ref="C2:C163"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4569,7 +4572,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K162"/>
+  <dimension ref="B2:K163"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -5829,7 +5832,7 @@
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="9" t="s">
+      <c r="B48" s="2" t="s">
         <v>244</v>
       </c>
       <c r="C48" s="5">
@@ -7773,7 +7776,7 @@
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B120" s="9" t="s">
+      <c r="B120" s="2" t="s">
         <v>245</v>
       </c>
       <c r="C120" s="5">
@@ -8691,245 +8694,272 @@
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="2">
-        <v>180</v>
+      <c r="B154" s="9" t="s">
+        <v>246</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>3.5625000000000004</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D154" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E154" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F154" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G154" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H154" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I154" s="3">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B155" s="2" t="s">
-        <v>216</v>
+      <c r="B155" s="2">
+        <v>180</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D155" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E155" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F155" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G155" s="1">
         <v>3</v>
       </c>
       <c r="H155" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I155" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D156" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E156" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F156" s="1">
         <v>2</v>
       </c>
       <c r="G156" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H156" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I156" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D157" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E157" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F157" s="1">
         <v>2</v>
       </c>
       <c r="G157" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H157" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I157" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D158" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E158" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F158" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G158" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H158" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I158" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D159" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E159" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F159" s="1">
         <v>0</v>
       </c>
       <c r="G159" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H159" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I159" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D160" s="1">
         <v>2</v>
       </c>
       <c r="E160" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F160" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G160" s="1">
         <v>2</v>
       </c>
       <c r="H160" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I160" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I160" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>2.6375000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D161" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E161" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F161" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G161" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H161" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I161" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D162" s="1">
+        <v>0</v>
+      </c>
+      <c r="E162" s="1">
+        <v>0</v>
+      </c>
+      <c r="F162" s="1">
+        <v>0</v>
+      </c>
+      <c r="G162" s="1">
+        <v>0</v>
+      </c>
+      <c r="H162" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I162" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="163" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B163" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C163" s="5">
+        <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D163" s="1">
         <v>2</v>
       </c>
-      <c r="E162" s="1">
+      <c r="E163" s="1">
         <v>1</v>
       </c>
-      <c r="F162" s="1">
+      <c r="F163" s="1">
         <v>2</v>
       </c>
-      <c r="G162" s="1">
+      <c r="G163" s="1">
         <v>2</v>
       </c>
-      <c r="H162" s="3">
+      <c r="H163" s="3">
         <v>4.3</v>
       </c>
-      <c r="I162" s="3">
+      <c r="I163" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>